<commit_message>
Add interface data viewer and champion tooling
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -7,9 +7,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'FIX_LABELS'!$A$1:$I$2</definedName>
-  </definedNames>
+  <definedNames/>
 </workbook>
 </file>
 
@@ -366,11 +364,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L488"/>
+  <dimension ref="A1:L503"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="26"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" style="3" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
@@ -24834,7 +24832,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>PlayerData_UIColourOffset</t>
+          <t>PlayerData_DialogueColourOffset</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -24849,12 +24847,12 @@
       </c>
       <c r="K478" t="inlineStr">
         <is>
-          <t>Active PlayerX_Data stores the current hardware/UI accent colour word at offset $4C.</t>
+          <t>Active PlayerX_Data stores the current hardware dialogue-text colour 15 word at offset $4C.</t>
         </is>
       </c>
       <c r="L478" t="inlineStr">
         <is>
-          <t>EQU-only definition; distinct from CharacterColours and ClassColours.</t>
+          <t>EQU-only definition; the Copper-scheduled interrupt writes this value for the active raster region.</t>
         </is>
       </c>
     </row>
@@ -24866,7 +24864,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>PlayerData_UIColourStateOffset</t>
+          <t>PlayerData_DialogueColourStateOffset</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -24881,7 +24879,7 @@
       </c>
       <c r="K479" t="inlineStr">
         <is>
-          <t>Active PlayerX_Data stores UI-colour animation/state flags at offset $52.</t>
+          <t>Active PlayerX_Data stores dialogue-colour fade and alternate-speaker flags at offset $52.</t>
         </is>
       </c>
       <c r="L479" t="inlineStr">
@@ -24913,7 +24911,7 @@
       </c>
       <c r="K480" t="inlineStr">
         <is>
-          <t>Bit 0 of the active player record selects the second player's colour-ramp family when set.</t>
+          <t>Bit 0 of the active player record selects Player 2's orange dialogue-ramp family when set.</t>
         </is>
       </c>
       <c r="L480" t="inlineStr">
@@ -24930,7 +24928,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>PlayerData_UIColourFadeBit</t>
+          <t>PlayerData_DialogueAlternateRampBit</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -24945,7 +24943,7 @@
       </c>
       <c r="K481" t="inlineStr">
         <is>
-          <t>Bit 6 of the player UI-colour state byte selects the alternate animated/fade ramp.</t>
+          <t>Bit 6 of the dialogue-colour state byte selects the shared red monster/alternate-speaker ramp.</t>
         </is>
       </c>
       <c r="L481" t="inlineStr">
@@ -24962,7 +24960,7 @@
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>PlayerColourRamp_EntriesPerState</t>
+          <t>DialogueColourRamp_EntriesPerState</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
@@ -24977,7 +24975,7 @@
       </c>
       <c r="K482" t="inlineStr">
         <is>
-          <t>Each player-colour state ramp contains six hardware-colour words.</t>
+          <t>Each dialogue-colour fade ramp contains six hardware-colour words ending at black.</t>
         </is>
       </c>
       <c r="L482" t="inlineStr">
@@ -24994,7 +24992,7 @@
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>PlayerColourRamp_Player2Offset</t>
+          <t>DialogueColourRamp_Player2Offset</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
@@ -25009,7 +25007,7 @@
       </c>
       <c r="K483" t="inlineStr">
         <is>
-          <t>Player 2 adds $0C to the colour entry index; after the code doubles d0 this selects a 24-byte displacement from the PC-relative base.</t>
+          <t>Player 2 adds $0C to the entry index to select its orange speech and red alternate ramps.</t>
         </is>
       </c>
       <c r="L483" t="inlineStr">
@@ -25175,6 +25173,598 @@
       <c r="L488" t="inlineStr">
         <is>
           <t>EQU-only definition; offset is within GFX_Pockets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>DialogueText_PaletteIndex</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>$0F</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>InitialiseText draws ordinary dialogue with foreground ink index 15.</t>
+        </is>
+      </c>
+      <c r="L489" t="inlineStr">
+        <is>
+          <t>EQU-only definition; colour register 15 is changed at raster interrupts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Copper_Player2RasterY</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>$98</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>CopperList_01 requests the Player 2 raster service after waiting for vertical position $98.</t>
+        </is>
+      </c>
+      <c r="L490" t="inlineStr">
+        <is>
+          <t>EQU-only definition; encoded by Copper wait word $9801.</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Copper_Player1FrameWrapRasterY</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>$FF</t>
+        </is>
+      </c>
+      <c r="J491" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K491" t="inlineStr">
+        <is>
+          <t>CopperList_01 requests the Player 1/frame service at the $FF raster wrap boundary.</t>
+        </is>
+      </c>
+      <c r="L491" t="inlineStr">
+        <is>
+          <t>EQU-only definition; encoded by Copper wait word $FF01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>CopperInterrupt_RequestWord</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>$8010</t>
+        </is>
+      </c>
+      <c r="J492" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K492" t="inlineStr">
+        <is>
+          <t>CopperList_01 writes $8010 to INTREQ at both raster waits to request the shared level-3 interrupt.</t>
+        </is>
+      </c>
+      <c r="L492" t="inlineStr">
+        <is>
+          <t>EQU-only definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>PlayerData_UIPrimaryColourOffset</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>$10</t>
+        </is>
+      </c>
+      <c r="J493" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t>PlayerX_Data stores the primary interface background and selection colour index at offset $10.</t>
+        </is>
+      </c>
+      <c r="L493" t="inlineStr">
+        <is>
+          <t>EQU-only definition; Player 1 uses $07 and Player 2 uses $09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>PlayerData_UISecondaryColourOffset</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>$12</t>
+        </is>
+      </c>
+      <c r="J494" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t>PlayerX_Data stores the colour index used to replace template ink $F in player-coloured interface graphics at offset $12.</t>
+        </is>
+      </c>
+      <c r="L494" t="inlineStr">
+        <is>
+          <t>EQU-only definition; Player 1 uses $08 and Player 2 uses $0C.</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>CompactStatsBar_LastIndex</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>$02</t>
+        </is>
+      </c>
+      <c r="J495" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K495" t="inlineStr">
+        <is>
+          <t>The compact player panel draws bar indices zero through two, giving exactly three statistics bars.</t>
+        </is>
+      </c>
+      <c r="L495" t="inlineStr">
+        <is>
+          <t>EQU-only definition for the DBRA loop terminal value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Player1_CompactStatsColourIndex</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>$07</t>
+        </is>
+      </c>
+      <c r="J496" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K496" t="inlineStr">
+        <is>
+          <t>The compact Player 1 statistics bars use hard-coded palette index $07.</t>
+        </is>
+      </c>
+      <c r="L496" t="inlineStr">
+        <is>
+          <t>Independent of both PlayerX_Data UI colour fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Player2_CompactStatsColourIndex</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>$0C</t>
+        </is>
+      </c>
+      <c r="J497" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K497" t="inlineStr">
+        <is>
+          <t>The compact Player 2 statistics bars use hard-coded palette index $0C.</t>
+        </is>
+      </c>
+      <c r="L497" t="inlineStr">
+        <is>
+          <t>Independent of both PlayerX_Data UI colour fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>PlayerData_InterfaceScreenBufferOffset</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>$0A</t>
+        </is>
+      </c>
+      <c r="J498" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K498" t="inlineStr">
+        <is>
+          <t>PlayerX_Data stores the framebuffer destination offset added to interface drawing addresses at offset $0A.</t>
+        </is>
+      </c>
+      <c r="L498" t="inlineStr">
+        <is>
+          <t>EQU-only definition; adrW_00EE86 is the Player 1 instance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>DeadPartyShieldClassColourMask</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>$00020103</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Draw_ShieldAvatar</t>
+        </is>
+      </c>
+      <c r="E499" t="inlineStr">
+        <is>
+          <t>adrCd00CDBC</t>
+        </is>
+      </c>
+      <c r="F499" t="inlineStr">
+        <is>
+          <t>move.l #$00020103,d0</t>
+        </is>
+      </c>
+      <c r="G499" t="inlineStr">
+        <is>
+          <t>203C00020103</t>
+        </is>
+      </c>
+      <c r="H499" t="inlineStr">
+        <is>
+          <t>move.l #DeadPartyShieldClassColourMask,d0</t>
+        </is>
+      </c>
+      <c r="I499" t="n">
+        <v>1</v>
+      </c>
+      <c r="J499" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K499" t="inlineStr">
+        <is>
+          <t>Fixed four-colour professional-symbol mask used when D3 is zero for a dead party member.</t>
+        </is>
+      </c>
+      <c r="L499" t="inlineStr">
+        <is>
+          <t>Draw_ShieldAvatar applies this mask only to GFX_Shield_Classes; D3 separately replaces source ink $F in every shield component.</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>GFX_Pockets_SelectedPartyShieldFrameOffset</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>$5070</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>adrCd007F86</t>
+        </is>
+      </c>
+      <c r="E500" t="inlineStr">
+        <is>
+          <t>adrCd007FB2</t>
+        </is>
+      </c>
+      <c r="F500" t="inlineStr">
+        <is>
+          <t>lea GFX_Pockets+$5070.l,a1</t>
+        </is>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>43F900051772</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>lea GFX_Pockets+GFX_Pockets_SelectedPartyShieldFrameOffset.l,a1</t>
+        </is>
+      </c>
+      <c r="I500" t="n">
+        <v>1</v>
+      </c>
+      <c r="J500" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K500" t="inlineStr">
+        <is>
+          <t>Offset of the 32x41 selected living-party shield surround in Pockets.gfx.</t>
+        </is>
+      </c>
+      <c r="L500" t="inlineStr">
+        <is>
+          <t>The active-living slot draws this surround before rendering the character inside it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>PartyShieldFrameSourceRowSkip</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>$0090</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>adrCd007F86</t>
+        </is>
+      </c>
+      <c r="E501" t="inlineStr">
+        <is>
+          <t>adrCd007FB2</t>
+        </is>
+      </c>
+      <c r="F501" t="inlineStr">
+        <is>
+          <t>move.l #$00000090,a3</t>
+        </is>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>267C00000090</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
+        <is>
+          <t>move.l #PartyShieldFrameSourceRowSkip,a3</t>
+        </is>
+      </c>
+      <c r="I501" t="n">
+        <v>1</v>
+      </c>
+      <c r="J501" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K501" t="inlineStr">
+        <is>
+          <t>Source-row skip after reading a two-word-wide crop from the 320-pixel Pockets sheet.</t>
+        </is>
+      </c>
+      <c r="L501" t="inlineStr">
+        <is>
+          <t>$90 skips the remaining eighteen planar words after each 32-pixel row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>ChampionStat_WornSpell</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>$11</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>adrCd00CCFE</t>
+        </is>
+      </c>
+      <c r="E502" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="F502" t="inlineStr">
+        <is>
+          <t>move.b $0011(a4),d0</t>
+        </is>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>102C0011</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>move.b ChampionStat_WornSpell(a4),d0</t>
+        </is>
+      </c>
+      <c r="I502" t="n">
+        <v>1</v>
+      </c>
+      <c r="J502" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K502" t="inlineStr">
+        <is>
+          <t>Reads the worn-spell field used to select the living shield-surround ink.</t>
+        </is>
+      </c>
+      <c r="L502" t="inlineStr">
+        <is>
+          <t>Zero retains default ink $04; nonzero values index the eight-byte lookup at $CD14.</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>PlayerData_PartyCommandStateOffset</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>$42</t>
+        </is>
+      </c>
+      <c r="J503" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t>Offset of the signed party-command/interface state word in each PlayerData record; $FFFF means inactive and states $0000-$0008 select dispatcher states.</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t>Player 1 live watch confirmed $EEBE-$EEBF changes from inactive $FFFF to transient $0001 when Communication is opened, then quickly to persistent $0008; Sleep restores $FFFF. The source dispatcher independently confirms states $0000-$0008 and Communication=$0008.</t>
         </is>
       </c>
     </row>
@@ -25248,7 +25838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F516"/>
+  <dimension ref="A1:F541"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -26873,7 +27463,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -26905,7 +27495,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -27065,7 +27655,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -27097,7 +27687,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -28697,7 +29287,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -30164,12 +30754,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>adrCd004EBE</t>
+          <t>CastSpell_ApplyVitalityCost</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>adrCd004EC8</t>
+          <t>CastSpell_ApplySpellPointCost</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -30329,7 +30919,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -30361,7 +30951,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>adrCd0050BC</t>
+          <t>Return_Beguile</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -32626,12 +33216,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>adrCd004EA0</t>
+          <t>CastSpell_ValidateSelection</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>adrCd004EBE</t>
+          <t>CastSpell_ApplyVitalityCost</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -32732,7 +33322,7 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>move.b #$0F,$001B(a4)</t>
+          <t>move.b #SpellCasting_ActionCooldown,$001B(a4)</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
@@ -32850,12 +33440,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>adrCd004EC8</t>
+          <t>CastSpell_ApplySpellPointCost</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>adrCd004EFA</t>
+          <t>CastSpell_CalculateQualityAndCooldown</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -32956,7 +33546,7 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>cmpi.b #$64,d1</t>
+          <t>cmpi.b #SpellCasting_CooldownMaximum,d1</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
@@ -33138,12 +33728,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>adrCd004F8E</t>
+          <t>CastSpell_RecordPractice</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>adrCd004FA8</t>
+          <t>CastSpell_Complete</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -33212,7 +33802,7 @@
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>and.w #$00F8,d7</t>
+          <t>and.w #~WornSpell_TypeMask&amp;$FF,d7</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
@@ -33308,7 +33898,7 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>bchg #$04,$01(a6,d0.w)</t>
+          <t>bchg #MapCell_MagelockedBit,$01(a6,d0.w)</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
@@ -33340,7 +33930,7 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>cmpi.b #$1B,d1</t>
+          <t>cmpi.b #Object_Armour_First,d1</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
@@ -33372,7 +33962,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>cmpi.b #$3F,d1</t>
+          <t>cmpi.b #Object_PowerStaff,d1</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -33404,7 +33994,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>addq.w #$05,d7</t>
+          <t>addq.w #Alchemy_BaseCoinageGain,d7</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -33436,7 +34026,7 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>move.b #$01,$00(a0,d0.w)</t>
+          <t>move.b #Object_Coinage,$00(a0,d0.w)</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
@@ -33468,7 +34058,7 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>sub.w #$0069,d0</t>
+          <t>sub.w #Object_MagicRings_First,d0</t>
         </is>
       </c>
       <c r="E257" t="inlineStr">
@@ -33500,7 +34090,7 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>lsr.w #$03,d7</t>
+          <t>lsr.w #Recharge_PowerShift,d7</t>
         </is>
       </c>
       <c r="E258" t="inlineStr">
@@ -33628,7 +34218,7 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>bclr #$03,$01(a6,d0.w)</t>
+          <t>bclr #MapCell_ConcealedBit,$01(a6,d0.w)</t>
         </is>
       </c>
       <c r="E262" t="inlineStr">
@@ -33660,7 +34250,7 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>bset #$07,$01(a6,d2.w)</t>
+          <t>bset #MapCell_SpellEntityBit,$01(a6,d2.w)</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
@@ -33756,7 +34346,7 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>moveq #$07,d5</t>
+          <t>moveq #Wychwind_ProjectileCount-1,d5</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
@@ -33788,7 +34378,7 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>add.b .wychwind_data(pc,d5.w),d6</t>
+          <t>add.b .Wychwind_DirectionAdjustments(pc,d5.w),d6</t>
         </is>
       </c>
       <c r="E267" t="inlineStr">
@@ -33820,7 +34410,7 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>or.b #$07,$01(a6,d0.w)</t>
+          <t>or.b #MapCell_MagicFeatureType,$01(a6,d0.w)</t>
         </is>
       </c>
       <c r="E268" t="inlineStr">
@@ -39009,7 +39599,7 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>Sets the selected interface page/action word to $FFFF, meaning no selection is active.</t>
+          <t>Initialises the party-command/interface state word to $FFFF, meaning no numbered command state is active.</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
@@ -41308,7 +41898,7 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>bra		adrCd00533C</t>
+          <t>bra SpellEntity_CheckPlacement</t>
         </is>
       </c>
       <c r="E502" t="inlineStr">
@@ -41631,7 +42221,7 @@
       </c>
       <c r="E512" t="inlineStr">
         <is>
-          <t>Selects Player 2's six-entry UI-colour ramp by adding $0C to the table entry index; the subsequent doubling makes the effective displacement 24 bytes.</t>
+          <t>Selects Player 2's orange dialogue-ramp family by adding $0C to the table index; doubling then produces a 24-byte displacement.</t>
         </is>
       </c>
       <c r="F512" t="inlineStr">
@@ -41663,7 +42253,7 @@
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Tests the UI-colour state bit that selects the alternate animated/fade ramp.</t>
+          <t>Tests the dialogue state bit that selects the shared red monster/alternate-speaker ramp.</t>
         </is>
       </c>
       <c r="F513" t="inlineStr">
@@ -41695,7 +42285,7 @@
       </c>
       <c r="E514" t="inlineStr">
         <is>
-          <t>Stores the selected hardware/UI accent colour word in the active PlayerX_Data record.</t>
+          <t>Stores the selected hardware dialogue-text colour 15 word in the active PlayerX_Data record.</t>
         </is>
       </c>
       <c r="F514" t="inlineStr">
@@ -41727,7 +42317,7 @@
       </c>
       <c r="E515" t="inlineStr">
         <is>
-          <t>Writes the selected PlayerX_Data accent colour to the custom-chip colour register used by the UI/VBlank path.</t>
+          <t>Writes the active player's dialogue ink to hardware colour register 15 for the current Copper-scheduled raster region.</t>
         </is>
       </c>
       <c r="F515" t="inlineStr">
@@ -41759,13 +42349,793 @@
       </c>
       <c r="E516" t="inlineStr">
         <is>
-          <t>Uses PlayerColourRampTable-2 as the original $8BE8 PC-relative base; after d0 is doubled, valid indices 1-24 address the 24-word UI-colour ramp beginning at $8BEA.</t>
+          <t>Uses PlayerColourRampTable-2 as the preserved $8BE8 PC-relative base; indices 1-24 address the green, red, orange, and red dialogue fades at $8BEA.</t>
         </is>
       </c>
       <c r="F516" t="inlineStr">
         <is>
           <t>1</t>
         </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>InitialiseText</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Print_fflim_text</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>move.l #$000F0000,adrW_00D92A.l</t>
+        </is>
+      </c>
+      <c r="E517" t="inlineStr">
+        <is>
+          <t>Sets ordinary dialogue foreground ink to palette index 15; raster interrupts supply its player/monster RGB value.</t>
+        </is>
+      </c>
+      <c r="F517" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>adrCd008B72</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>PlayerColourRampLookupBase_Exit</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>move.w $004C(a5),_custom+color+$0000001E.l</t>
+        </is>
+      </c>
+      <c r="E518" t="inlineStr">
+        <is>
+          <t>Restores the active player's current dialogue colour 15 at this Copper-scheduled raster region when no fade step advances.</t>
+        </is>
+      </c>
+      <c r="F518" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>VerticalBlankInterupt</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>adrCd008C62</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>lea Player2_Data.l,a5</t>
+        </is>
+      </c>
+      <c r="E519" t="inlineStr">
+        <is>
+          <t>Selects Player 2 for the first Copper-scheduled dialogue-colour raster service.</t>
+        </is>
+      </c>
+      <c r="F519" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>VerticalBlankInterupt</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>adrCd008C62</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>bsr adrCd008B72</t>
+        </is>
+      </c>
+      <c r="E520" t="inlineStr">
+        <is>
+          <t>Updates hardware colour 15 from Player 2's dialogue fade state for the lower player region.</t>
+        </is>
+      </c>
+      <c r="F520" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>adrCd008C62</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>adrL_008CC8</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>lea Player1_Data.l,a5</t>
+        </is>
+      </c>
+      <c r="E521" t="inlineStr">
+        <is>
+          <t>Selects Player 1 for the second Copper-scheduled dialogue-colour service and frame update.</t>
+        </is>
+      </c>
+      <c r="F521" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>adrCd008C62</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>adrL_008CC8</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>bsr adrCd008B72</t>
+        </is>
+      </c>
+      <c r="E522" t="inlineStr">
+        <is>
+          <t>Updates hardware colour 15 from Player 1's dialogue fade state after the raster/frame wrap.</t>
+        </is>
+      </c>
+      <c r="F522" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>adrCd008278</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>adrCd008396</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>move.w $0010(a5),d3</t>
+        </is>
+      </c>
+      <c r="E523" t="inlineStr">
+        <is>
+          <t>Loads the active player's primary UI colour for the champion-name background block.</t>
+        </is>
+      </c>
+      <c r="F523" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>adrCd008396</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>adrB_008412</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>move.w $0010(a5),d3</t>
+        </is>
+      </c>
+      <c r="E524" t="inlineStr">
+        <is>
+          <t>Loads the active player's primary UI colour for the selected team-member frame.</t>
+        </is>
+      </c>
+      <c r="F524" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>adrCd007B50</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>adrCd007BE8</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>move.w $0012(a5),d3</t>
+        </is>
+      </c>
+      <c r="E525" t="inlineStr">
+        <is>
+          <t>Loads the active player's secondary UI colour before drawing the six command/toggle pocket graphics.</t>
+        </is>
+      </c>
+      <c r="F525" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>adrCd007D6C</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>adrCd007EC0</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>move.w $0010(a5),d3</t>
+        </is>
+      </c>
+      <c r="E526" t="inlineStr">
+        <is>
+          <t>Uses the active player's primary UI colour for either selected party-command row state.</t>
+        </is>
+      </c>
+      <c r="F526" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>adrCd00C9BC</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>ObjectGraphic</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>move.w $0012(a5),d3</t>
+        </is>
+      </c>
+      <c r="E527" t="inlineStr">
+        <is>
+          <t>Loads the secondary UI colour used to recolour empty hand, armour, shield, and pocket template graphics.</t>
+        </is>
+      </c>
+      <c r="F527" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>adrCd0080CA</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>adrCd00813C</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>moveq #$02,d6</t>
+        </is>
+      </c>
+      <c r="E528" t="inlineStr">
+        <is>
+          <t>Sets a DBRA terminal index of two, so the compact player panel draws exactly three statistics bars.</t>
+        </is>
+      </c>
+      <c r="F528" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>adrCd0080CA</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>adrCd00813C</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>moveq #$07,d3</t>
+        </is>
+      </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>Selects hard-coded palette index $07 for Player 1's three compact statistics bars.</t>
+        </is>
+      </c>
+      <c r="F529" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>adrCd0080CA</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>adrCd00813C</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>moveq #$0C,d3</t>
+        </is>
+      </c>
+      <c r="E530" t="inlineStr">
+        <is>
+          <t>Selects hard-coded palette index $0C for Player 2's three compact statistics bars.</t>
+        </is>
+      </c>
+      <c r="F530" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>adrCd00CE86</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>ConvertByteToDecimal_HighNibbleAdjustments</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>move.w d3,d6</t>
+        </is>
+      </c>
+      <c r="E531" t="inlineStr">
+        <is>
+          <t>Begins converting the supplied colour index into bitplane masks that replace source ink $F pixels.</t>
+        </is>
+      </c>
+      <c r="F531" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>adrCd007F54</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>adrCd007FD4</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>move.b $18(a5,d0.w),d7</t>
+        </is>
+      </c>
+      <c r="E532" t="inlineStr">
+        <is>
+          <t>Loads the selected party-slot state byte; a negative value denotes a vacant slot and the low nibble identifies an occupied champion.</t>
+        </is>
+      </c>
+      <c r="F532" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>adrCd007F54</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>adrCd007FB2</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>btst d0,$003E(a5)</t>
+        </is>
+      </c>
+      <c r="E533" t="inlineStr">
+        <is>
+          <t>Tests whether this party slot is the active selected member before choosing its shield-rendering path.</t>
+        </is>
+      </c>
+      <c r="F533" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>adrCd007F86</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>adrCd007FB2</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>lea GFX_Pockets+GFX_Pockets_SelectedPartyShieldFrameOffset.l,a1</t>
+        </is>
+      </c>
+      <c r="E534" t="inlineStr">
+        <is>
+          <t>Selects the 32x41 light-grey shield surround used for the active living party member.</t>
+        </is>
+      </c>
+      <c r="F534" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>adrCd007F86</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>adrCd007FB2</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>move.l #PartyShieldFrameSourceRowSkip,a3</t>
+        </is>
+      </c>
+      <c r="E535" t="inlineStr">
+        <is>
+          <t>Skips the unused remainder of each Pockets.gfx source row after drawing the two-word-wide shield surround.</t>
+        </is>
+      </c>
+      <c r="F535" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>adrCd007FD6</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>adrCd007FF4</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>moveq #$00,d3</t>
+        </is>
+      </c>
+      <c r="E536" t="inlineStr">
+        <is>
+          <t>Selects black for shield ink $F and retains the fixed dead-state professional-symbol colour mask.</t>
+        </is>
+      </c>
+      <c r="F536" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>adrCd00CCFE</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>move.b ChampionStat_WornSpell(a4),d0</t>
+        </is>
+      </c>
+      <c r="E537" t="inlineStr">
+        <is>
+          <t>Reads the currently worn spell; zero leaves the normal light-grey shield-surround ink unchanged.</t>
+        </is>
+      </c>
+      <c r="F537" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>adrCd00CCFE</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>and.w #$0007,d0</t>
+        </is>
+      </c>
+      <c r="E538" t="inlineStr">
+        <is>
+          <t>Uses the worn spell's low three bits to select one of eight shield-surround ink colours.</t>
+        </is>
+      </c>
+      <c r="F538" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Draw_ShieldAvatar</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>adrCd00CDBC</t>
+        </is>
+      </c>
+      <c r="D539" t="inlineStr">
+        <is>
+          <t>tst.w d3</t>
+        </is>
+      </c>
+      <c r="E539" t="inlineStr">
+        <is>
+          <t>Keeps the fixed dead mask when D3 is zero; living shields replace it with a ClassColours record.</t>
+        </is>
+      </c>
+      <c r="F539" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Draw_ShieldAvatar</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>adrCd00CE26</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>move.w #$FFFF,Buffer_Colour_Mask_Toggle.l</t>
+        </is>
+      </c>
+      <c r="E540" t="inlineStr">
+        <is>
+          <t>Enables four-colour remapping only for the professional symbol; the face avatar is never passed through this mask.</t>
+        </is>
+      </c>
+      <c r="F540" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Draw_ShieldAvatar</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>adrCd00CE26</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>clr.w Buffer_Colour_Mask_Toggle.l</t>
+        </is>
+      </c>
+      <c r="E541" t="inlineStr">
+        <is>
+          <t>Disables four-colour remapping immediately after the professional symbol has been drawn.</t>
+        </is>
+      </c>
+      <c r="F541" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -41777,7 +43147,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -41886,7 +43256,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Various UI viewer fixes
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Rd1dd67d9f2a5480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rb6164ac7fcfe4d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R8853d8c4c1fe40d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Ra8614e96e4ff4df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R890b596655bc4d1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="Rc8e035c891334312"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9013,12 +9013,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Stats background packs X=$35 with horizontal terminal count $26, drawing $27 pixels wide.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">moveq #$02,d3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Stats background uses palette index $02, the light-grey panel fill.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">lea GFX_Pockets+$7580.l,a1</x:t>
@@ -9191,7 +9185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -9209,6 +9203,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -36392,23 +36389,23 @@
       </x:c>
     </x:row>
     <x:row r="554">
-      <x:c r="A554" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B554" t="s">
-        <x:v>2976</x:v>
-      </x:c>
-      <x:c r="C554" t="s">
-        <x:v>2173</x:v>
-      </x:c>
-      <x:c r="D554" t="s">
-        <x:v>3001</x:v>
-      </x:c>
-      <x:c r="E554" t="s">
-        <x:v>3002</x:v>
-      </x:c>
-      <x:c r="F554" t="s">
-        <x:v>20</x:v>
+      <x:c r="A554" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B554" t="str">
+        <x:v>adrCd007FF8</x:v>
+      </x:c>
+      <x:c r="C554" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="D554" t="str">
+        <x:v>moveq #$02,d3</x:v>
+      </x:c>
+      <x:c r="E554" t="str">
+        <x:v>Stats background uses palette index $02, the light-grey panel fill.</x:v>
+      </x:c>
+      <x:c r="F554" t="str">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="555">
@@ -36422,10 +36419,10 @@
         <x:v>2173</x:v>
       </x:c>
       <x:c r="D555" t="s">
-        <x:v>3003</x:v>
+        <x:v>3001</x:v>
       </x:c>
       <x:c r="E555" t="s">
-        <x:v>3004</x:v>
+        <x:v>3002</x:v>
       </x:c>
       <x:c r="F555" t="s">
         <x:v>20</x:v>
@@ -36442,10 +36439,10 @@
         <x:v>2173</x:v>
       </x:c>
       <x:c r="D556" t="s">
-        <x:v>3005</x:v>
+        <x:v>3003</x:v>
       </x:c>
       <x:c r="E556" t="s">
-        <x:v>3006</x:v>
+        <x:v>3004</x:v>
       </x:c>
       <x:c r="F556" t="s">
         <x:v>20</x:v>
@@ -36465,7 +36462,7 @@
         <x:v>2177</x:v>
       </x:c>
       <x:c r="E557" t="s">
-        <x:v>3007</x:v>
+        <x:v>3005</x:v>
       </x:c>
       <x:c r="F557" t="s">
         <x:v>20</x:v>
@@ -36485,7 +36482,7 @@
         <x:v>2182</x:v>
       </x:c>
       <x:c r="E558" t="s">
-        <x:v>3008</x:v>
+        <x:v>3006</x:v>
       </x:c>
       <x:c r="F558" t="s">
         <x:v>20</x:v>
@@ -36505,7 +36502,7 @@
         <x:v>2186</x:v>
       </x:c>
       <x:c r="E559" t="s">
-        <x:v>3009</x:v>
+        <x:v>3007</x:v>
       </x:c>
       <x:c r="F559" t="s">
         <x:v>20</x:v>
@@ -36516,16 +36513,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B560" s="8" t="s">
+        <x:v>3008</x:v>
+      </x:c>
+      <x:c r="C560" s="8" t="s">
+        <x:v>3009</x:v>
+      </x:c>
+      <x:c r="D560" s="8" t="s">
         <x:v>3010</x:v>
       </x:c>
-      <x:c r="C560" s="8" t="s">
+      <x:c r="E560" s="8" t="s">
         <x:v>3011</x:v>
-      </x:c>
-      <x:c r="D560" s="8" t="s">
-        <x:v>3012</x:v>
-      </x:c>
-      <x:c r="E560" s="8" t="s">
-        <x:v>3013</x:v>
       </x:c>
       <x:c r="F560" s="8">
         <x:v>1</x:v>
@@ -36536,16 +36533,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B561" s="8" t="s">
-        <x:v>3010</x:v>
+        <x:v>3008</x:v>
       </x:c>
       <x:c r="C561" s="8" t="s">
-        <x:v>3011</x:v>
+        <x:v>3009</x:v>
       </x:c>
       <x:c r="D561" s="8" t="s">
-        <x:v>3014</x:v>
+        <x:v>3012</x:v>
       </x:c>
       <x:c r="E561" s="8" t="s">
-        <x:v>3015</x:v>
+        <x:v>3013</x:v>
       </x:c>
       <x:c r="F561" s="8">
         <x:v>1</x:v>
@@ -36556,16 +36553,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B562" s="8" t="s">
-        <x:v>3016</x:v>
+        <x:v>3014</x:v>
       </x:c>
       <x:c r="C562" s="8" t="s">
-        <x:v>3011</x:v>
+        <x:v>3009</x:v>
       </x:c>
       <x:c r="D562" s="8" t="s">
         <x:v>2983</x:v>
       </x:c>
       <x:c r="E562" s="8" t="s">
-        <x:v>3017</x:v>
+        <x:v>3015</x:v>
       </x:c>
       <x:c r="F562" s="8">
         <x:v>1</x:v>
@@ -36582,10 +36579,10 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D563" s="8" t="s">
-        <x:v>3018</x:v>
+        <x:v>3016</x:v>
       </x:c>
       <x:c r="E563" s="8" t="s">
-        <x:v>3019</x:v>
+        <x:v>3017</x:v>
       </x:c>
       <x:c r="F563" s="8">
         <x:v>1</x:v>
@@ -36602,10 +36599,10 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D564" s="8" t="s">
-        <x:v>3020</x:v>
+        <x:v>3018</x:v>
       </x:c>
       <x:c r="E564" s="8" t="s">
-        <x:v>3021</x:v>
+        <x:v>3019</x:v>
       </x:c>
       <x:c r="F564" s="8">
         <x:v>1</x:v>
@@ -36625,7 +36622,7 @@
         <x:v>2195</x:v>
       </x:c>
       <x:c r="E565" s="8" t="s">
-        <x:v>3022</x:v>
+        <x:v>3020</x:v>
       </x:c>
       <x:c r="F565" s="8">
         <x:v>1</x:v>
@@ -36642,10 +36639,10 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D566" s="8" t="s">
-        <x:v>3023</x:v>
+        <x:v>3021</x:v>
       </x:c>
       <x:c r="E566" s="8" t="s">
-        <x:v>3024</x:v>
+        <x:v>3022</x:v>
       </x:c>
       <x:c r="F566" s="8">
         <x:v>1</x:v>
@@ -36662,10 +36659,10 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D567" s="8" t="s">
-        <x:v>3025</x:v>
+        <x:v>3023</x:v>
       </x:c>
       <x:c r="E567" s="8" t="s">
-        <x:v>3026</x:v>
+        <x:v>3024</x:v>
       </x:c>
       <x:c r="F567" s="8">
         <x:v>1</x:v>
@@ -36682,10 +36679,10 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D568" s="8" t="s">
-        <x:v>3027</x:v>
+        <x:v>3025</x:v>
       </x:c>
       <x:c r="E568" s="8" t="s">
-        <x:v>3028</x:v>
+        <x:v>3026</x:v>
       </x:c>
       <x:c r="F568" s="8">
         <x:v>1</x:v>
@@ -36702,12 +36699,232 @@
         <x:v>2192</x:v>
       </x:c>
       <x:c r="D569" s="8" t="s">
-        <x:v>3029</x:v>
+        <x:v>3027</x:v>
       </x:c>
       <x:c r="E569" s="8" t="s">
-        <x:v>3030</x:v>
+        <x:v>3028</x:v>
       </x:c>
       <x:c r="F569" s="8">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="570">
+      <x:c r="A570" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B570" t="str">
+        <x:v>adrCd007FF8</x:v>
+      </x:c>
+      <x:c r="C570" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="D570" t="str">
+        <x:v>bsr BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E570" t="str">
+        <x:v>Draws the stats background rectangle using the dimensions in D4 and the current palette index in D3.</x:v>
+      </x:c>
+      <x:c r="F570" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="571">
+      <x:c r="A571" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B571" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="C571" t="str">
+        <x:v>Draw_CompactStatsBarsLoop</x:v>
+      </x:c>
+      <x:c r="D571" t="str">
+        <x:v>moveq #$03,d3</x:v>
+      </x:c>
+      <x:c r="E571" t="str">
+        <x:v>The $80E8 stats-bar background call uses palette index $03, the lighter panel fill.</x:v>
+      </x:c>
+      <x:c r="F571" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="572">
+      <x:c r="A572" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B572" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="C572" t="str">
+        <x:v>Draw_CompactStatsBarsLoop</x:v>
+      </x:c>
+      <x:c r="D572" t="str">
+        <x:v>bsr BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E572" t="str">
+        <x:v>Draws the stats-bar background rectangle using D4 dimensions and D3.</x:v>
+      </x:c>
+      <x:c r="F572" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="573" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A573" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B573" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C573" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D573" t="str">
+        <x:v>move.l #$005F0000,d4</x:v>
+      </x:c>
+      <x:c r="E573" s="9" t="str">
+        <x:v>Clears the 96 by 89 player-local party-command panel before drawing the avatar, command pockets, menu rows, and chain strip.</x:v>
+      </x:c>
+      <x:c r="F573" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="574" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A574" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B574" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C574" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D574" t="str">
+        <x:v>moveq #$71,d7</x:v>
+      </x:c>
+      <x:c r="E574" s="9" t="str">
+        <x:v>Starts the command-pocket graphic sequence at Pockets icon $71; six consecutive icons form the visible command/toggle control bank, with the last two drawn only in Communication state.</x:v>
+      </x:c>
+      <x:c r="F574" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="575" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A575" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B575" t="str">
+        <x:v>Draw_PartyCommandMenu</x:v>
+      </x:c>
+      <x:c r="C575" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D575" t="str">
+        <x:v>move.w $0044(a5),d0</x:v>
+      </x:c>
+      <x:c r="E575" s="9" t="str">
+        <x:v>Loads the active party-command menu descriptor-stream index before selecting its stream through the ten-entry jump table.</x:v>
+      </x:c>
+      <x:c r="F575" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="576" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A576" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B576" t="str">
+        <x:v>Draw_PartyCommandMenu</x:v>
+      </x:c>
+      <x:c r="C576" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D576" t="str">
+        <x:v>move.l #$00060039,d5</x:v>
+      </x:c>
+      <x:c r="E576" s="9" t="str">
+        <x:v>Initialises a seven-pixel-tall menu bar at player-local Y=$39; each of the four rows advances by eight pixels, leaving a one-pixel black separator.</x:v>
+      </x:c>
+      <x:c r="F576" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="577" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A577" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B577" t="str">
+        <x:v>Draw_PartyCommandMenu</x:v>
+      </x:c>
+      <x:c r="C577" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D577" t="str">
+        <x:v>move.b $00(a6,d7.w),d4</x:v>
+      </x:c>
+      <x:c r="E577" s="9" t="str">
+        <x:v>Loads the descriptor byte that sets the current row's left bar extent; the remaining width is drawn as the right bar with the separating vertical line retained.</x:v>
+      </x:c>
+      <x:c r="F577" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="578" ht="16" hidden="0" customHeight="1">
+      <x:c r="A578" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B578" t="str">
+        <x:v>Draw_PartyCommandMenu</x:v>
+      </x:c>
+      <x:c r="C578" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D578" t="str">
+        <x:v>addq.w #$08,d5</x:v>
+      </x:c>
+      <x:c r="E578" s="9" t="str">
+        <x:v>Moves to the next of four menu rows: seven bar pixels plus one black separator pixel.</x:v>
+      </x:c>
+      <x:c r="F578" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="579" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A579" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B579" t="str">
+        <x:v>Draw_PartyCommandMenu</x:v>
+      </x:c>
+      <x:c r="C579" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D579" t="str">
+        <x:v>addq.w #$04,a6</x:v>
+      </x:c>
+      <x:c r="E579" s="9" t="str">
+        <x:v>Skips the four row-layout descriptor bytes before consuming the packed text entries for the same four visible rows.</x:v>
+      </x:c>
+      <x:c r="F579" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="580" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A580" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B580" t="str">
+        <x:v>adrCd007E12</x:v>
+      </x:c>
+      <x:c r="C580" t="str">
+        <x:v>adrCd007E4A</x:v>
+      </x:c>
+      <x:c r="D580" t="str">
+        <x:v>bsr Print_com_menu_entry</x:v>
+      </x:c>
+      <x:c r="E580" s="9" t="str">
+        <x:v>Prints one packed party-command text row; four passes consume the descriptor stream entries in display order.</x:v>
+      </x:c>
+      <x:c r="F580" t="str">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -36736,10 +36953,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="7" t="s">
-        <x:v>3031</x:v>
+        <x:v>3029</x:v>
       </x:c>
       <x:c r="C1" s="7" t="s">
-        <x:v>3032</x:v>
+        <x:v>3030</x:v>
       </x:c>
       <x:c r="D1" s="7" t="s">
         <x:v>5</x:v>
@@ -36765,19 +36982,19 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B2" s="7" t="s">
+        <x:v>3031</x:v>
+      </x:c>
+      <x:c r="C2" s="7" t="s">
+        <x:v>3032</x:v>
+      </x:c>
+      <x:c r="D2" s="7" t="s">
         <x:v>3033</x:v>
-      </x:c>
-      <x:c r="C2" s="7" t="s">
-        <x:v>3034</x:v>
-      </x:c>
-      <x:c r="D2" s="7" t="s">
-        <x:v>3035</x:v>
       </x:c>
       <x:c r="E2" s="7" t="s">
         <x:v>2912</x:v>
       </x:c>
       <x:c r="F2" s="7" t="s">
-        <x:v>3036</x:v>
+        <x:v>3034</x:v>
       </x:c>
       <x:c r="G2" s="7">
         <x:v>1</x:v>
@@ -36786,7 +37003,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="I2" s="7" t="s">
-        <x:v>3037</x:v>
+        <x:v>3035</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Various updates to the UI viewer
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Ra8614e96e4ff4df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R890b596655bc4d1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="Rc8e035c891334312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R20eae8ea89e64ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R03c75358b4e74ff6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R55b7d0b25079465f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -36802,7 +36802,7 @@
         <x:v>moveq #$71,d7</x:v>
       </x:c>
       <x:c r="E574" s="9" t="str">
-        <x:v>Starts the command-pocket graphic sequence at Pockets icon $71; six consecutive icons form the visible command/toggle control bank, with the last two drawn only in Communication state.</x:v>
+        <x:v>Seeds D7 with Pockets icon $71. The loop draws icon IDs $71-$74 in two-icon rows, and only draws $75-$76 when the interface is in active Communication state $08.</x:v>
       </x:c>
       <x:c r="F574" t="str">
         <x:v>1</x:v>
@@ -36925,6 +36925,2366 @@
         <x:v>Prints one packed party-command text row; four passes consume the descriptor stream entries in display order.</x:v>
       </x:c>
       <x:c r="F580" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="581" ht="16" hidden="0" customHeight="1">
+      <x:c r="A581" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B581" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C581" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D581" t="str">
+        <x:v>moveq #$0A,d5</x:v>
+      </x:c>
+      <x:c r="E581" s="9" t="str">
+        <x:v>Sets player-local Y=$0A for the outer pair of command-pocket decoration lines.</x:v>
+      </x:c>
+      <x:c r="F581" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="582" ht="16" hidden="0" customHeight="1">
+      <x:c r="A582" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B582" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C582" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D582" t="str">
+        <x:v>add.w $0008(a5),d5</x:v>
+      </x:c>
+      <x:c r="E582" s="9" t="str">
+        <x:v>Applies the active player's screen-buffer Y offset to this player-local drawing coordinate.</x:v>
+      </x:c>
+      <x:c r="F582" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="583" ht="16" hidden="0" customHeight="1">
+      <x:c r="A583" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B583" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C583" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D583" t="str">
+        <x:v>moveq #$32,d4</x:v>
+      </x:c>
+      <x:c r="E583" s="9" t="str">
+        <x:v>Sets the outer-left command-pocket decoration line at player-local X=$32.</x:v>
+      </x:c>
+      <x:c r="F583" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="584" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A584" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B584" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C584" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D584" t="str">
+        <x:v>move.l #$002B0002,d3</x:v>
+      </x:c>
+      <x:c r="E584" s="9" t="str">
+        <x:v>Sets the outer-line DBRA count to $2B (44 rendered pixels) and the shared grey palette index to $02.</x:v>
+      </x:c>
+      <x:c r="F584" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="585" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A585" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B585" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C585" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D585" t="str">
+        <x:v>bsr BW_blit_vertical_line</x:v>
+      </x:c>
+      <x:c r="E585" s="9" t="str">
+        <x:v>Draws one of the four command-pocket decoration lines using D4 X, D5 Y, the high-word DBRA count in D3, and the low-word palette index in D3.</x:v>
+      </x:c>
+      <x:c r="F585" t="str">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="586" ht="16" hidden="0" customHeight="1">
+      <x:c r="A586" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B586" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C586" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D586" t="str">
+        <x:v>moveq #$5D,d4</x:v>
+      </x:c>
+      <x:c r="E586" s="9" t="str">
+        <x:v>Sets the outer-right command-pocket decoration line at player-local X=$5D.</x:v>
+      </x:c>
+      <x:c r="F586" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="587" ht="16" hidden="0" customHeight="1">
+      <x:c r="A587" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B587" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C587" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D587" t="str">
+        <x:v>addq.w #$02,d5</x:v>
+      </x:c>
+      <x:c r="E587" s="9" t="str">
+        <x:v>Moves the inner decoration pair two pixels down to player-local Y=$0C.</x:v>
+      </x:c>
+      <x:c r="F587" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="588" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A588" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B588" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C588" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D588" t="str">
+        <x:v>sub.l #$00040000,d3</x:v>
+      </x:c>
+      <x:c r="E588" s="9" t="str">
+        <x:v>Reduces the high-word DBRA count from $2B to $27, making each inner line 40 pixels—four pixels shorter than the outer pair.</x:v>
+      </x:c>
+      <x:c r="F588" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="589" ht="16" hidden="0" customHeight="1">
+      <x:c r="A589" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B589" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C589" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D589" t="str">
+        <x:v>moveq #$5B,d4</x:v>
+      </x:c>
+      <x:c r="E589" s="9" t="str">
+        <x:v>Sets the inner-right command-pocket decoration line at player-local X=$5B.</x:v>
+      </x:c>
+      <x:c r="F589" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="590" ht="16" hidden="0" customHeight="1">
+      <x:c r="A590" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B590" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C590" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D590" t="str">
+        <x:v>moveq #$34,d4</x:v>
+      </x:c>
+      <x:c r="E590" s="9" t="str">
+        <x:v>Sets the inner-left command-pocket decoration line at player-local X=$34.</x:v>
+      </x:c>
+      <x:c r="F590" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="591" ht="16" hidden="0" customHeight="1">
+      <x:c r="A591" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B591" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C591" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D591" t="str">
+        <x:v>move.l screen_ptr.l,a0</x:v>
+      </x:c>
+      <x:c r="E591" s="9" t="str">
+        <x:v>Loads the screen base before positioning the first pair of Pockets command icons.</x:v>
+      </x:c>
+      <x:c r="F591" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="592" ht="16" hidden="0" customHeight="1">
+      <x:c r="A592" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B592" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C592" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D592" t="str">
+        <x:v>add.w #$0147,a0</x:v>
+      </x:c>
+      <x:c r="E592" s="9" t="str">
+        <x:v>Positions A0 at the player-local destination for the first two command-pocket icons.</x:v>
+      </x:c>
+      <x:c r="F592" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="593" ht="16" hidden="0" customHeight="1">
+      <x:c r="A593" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B593" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C593" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D593" t="str">
+        <x:v>add.w $000A(a5),a0</x:v>
+      </x:c>
+      <x:c r="E593" s="9" t="str">
+        <x:v>Applies the active player's screen-buffer byte offset to the command-pocket icon destination.</x:v>
+      </x:c>
+      <x:c r="F593" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="594" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A594" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B594" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C594" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D594" t="str">
+        <x:v>move.w $0012(a5),d3</x:v>
+      </x:c>
+      <x:c r="E594" s="9" t="str">
+        <x:v>Loads PlayerData_UISecondaryColourOffset: the replacement ink palette index for the player-coloured Pockets command and toggle icons.</x:v>
+      </x:c>
+      <x:c r="F594" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="595" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A595" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B595" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C595" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D595" t="str">
+        <x:v>move.w d7,d0</x:v>
+      </x:c>
+      <x:c r="E595" s="9" t="str">
+        <x:v>Passes the current Pockets icon ID from D7 to Draw_PocketGraphic; each loop pass draws two consecutive IDs.</x:v>
+      </x:c>
+      <x:c r="F595" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="596" ht="16" hidden="0" customHeight="1">
+      <x:c r="A596" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B596" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C596" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D596" t="str">
+        <x:v>bsr Draw_PocketGraphic</x:v>
+      </x:c>
+      <x:c r="E596" s="9" t="str">
+        <x:v>Draws the current player-coloured Pockets icon selected by D7/D0 at the destination in A0.</x:v>
+      </x:c>
+      <x:c r="F596" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="597" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A597" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B597" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C597" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D597" t="str">
+        <x:v>addq.w #$01,d7</x:v>
+      </x:c>
+      <x:c r="E597" s="9" t="str">
+        <x:v>Advances D7 to the next Pockets icon ID; the loop covers $71 through $74 unconditionally, then $75 and $76 only in communication state.</x:v>
+      </x:c>
+      <x:c r="F597" t="str">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="598" ht="16" hidden="0" customHeight="1">
+      <x:c r="A598" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B598" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C598" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D598" t="str">
+        <x:v>add.w #$027C,a0</x:v>
+      </x:c>
+      <x:c r="E598" s="9" t="str">
+        <x:v>Advances the drawing destination from one two-icon row to the next command-pocket row.</x:v>
+      </x:c>
+      <x:c r="F598" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="599" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A599" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B599" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C599" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D599" t="str">
+        <x:v>cmpi.w #$0075,d7</x:v>
+      </x:c>
+      <x:c r="E599" s="9" t="str">
+        <x:v>Repeats the two-icon drawing loop until the always-visible Pockets icons $71 through $74 have been drawn.</x:v>
+      </x:c>
+      <x:c r="F599" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="600" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A600" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B600" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C600" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D600" t="str">
+        <x:v>cmp.w #$0008,$0042(a5)</x:v>
+      </x:c>
+      <x:c r="E600" s="9" t="str">
+        <x:v>Tests for active communication state $08; other party-command states skip the final wide-toggle icon pair.</x:v>
+      </x:c>
+      <x:c r="F600" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="601" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A601" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B601" t="str">
+        <x:v>adrCd007BC0</x:v>
+      </x:c>
+      <x:c r="C601" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D601" t="str">
+        <x:v>cmpi.w #$0077,d7</x:v>
+      </x:c>
+      <x:c r="E601" s="9" t="str">
+        <x:v>Continues the loop only until the active-communication-only Pockets icons $75 and $76 have also been drawn.</x:v>
+      </x:c>
+      <x:c r="F601" t="str">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="602">
+      <x:c r="A602" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B602" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C602" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D602" t="str">
+        <x:v>lsr.w #$02,d0</x:v>
+      </x:c>
+      <x:c r="E602" t="str">
+        <x:v>Converts the dispatch-table byte offset into action number $06-$09 before calculating the party-slot index.</x:v>
+      </x:c>
+      <x:c r="F602" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="603">
+      <x:c r="A603" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B603" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C603" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D603" t="str">
+        <x:v>subq.w #$06,d0</x:v>
+      </x:c>
+      <x:c r="E603" t="str">
+        <x:v>Converts party-member action $06-$09 to PlayerX_Data party slot $00-$03.</x:v>
+      </x:c>
+      <x:c r="F603" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="604">
+      <x:c r="A604" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B604" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C604" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D604" t="str">
+        <x:v>tst.w $0016(a5)</x:v>
+      </x:c>
+      <x:c r="E604" t="str">
+        <x:v>Tests the pending party-slot selection. A negative value means this is the first click.</x:v>
+      </x:c>
+      <x:c r="F604" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="605">
+      <x:c r="A605" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B605" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C605" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D605" t="str">
+        <x:v>move.w d0,$0016(a5)</x:v>
+      </x:c>
+      <x:c r="E605" t="str">
+        <x:v>Stores the first-click party-slot index as the pending selection, then redraws the party command interface.</x:v>
+      </x:c>
+      <x:c r="F605" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="606">
+      <x:c r="A606" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B606" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C606" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D606" t="str">
+        <x:v>cmp.w $0016(a5),d0</x:v>
+      </x:c>
+      <x:c r="E606" t="str">
+        <x:v>A second click on the same pending slot commits that champion as current; a different slot instead enters the reorder path.</x:v>
+      </x:c>
+      <x:c r="F606" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="607">
+      <x:c r="A607" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B607" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C607" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D607" t="str">
+        <x:v>move.b $26(a5,d0.w),d1</x:v>
+      </x:c>
+      <x:c r="E607" t="str">
+        <x:v>Loads the clicked party-position entry before exchanging it with the entry from the initially selected slot.</x:v>
+      </x:c>
+      <x:c r="F607" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="608">
+      <x:c r="A608" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B608" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C608" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D608" t="str">
+        <x:v>move.b $26(a5,d2.w),$26(a5,d0.w)</x:v>
+      </x:c>
+      <x:c r="E608" t="str">
+        <x:v>Moves the initially selected party-position entry into the different clicked slot; the next instruction writes the saved entry back, completing the swap.</x:v>
+      </x:c>
+      <x:c r="F608" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="609">
+      <x:c r="A609" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B609" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C609" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D609" t="str">
+        <x:v>moveq #-$01,d0</x:v>
+      </x:c>
+      <x:c r="E609" t="str">
+        <x:v>Marks the pending selection invalid after a party-position swap; it does not change the current champion.</x:v>
+      </x:c>
+      <x:c r="F609" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="610">
+      <x:c r="A610" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B610" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C610" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D610" t="str">
+        <x:v>move.b $26(a5,d0.w),d0</x:v>
+      </x:c>
+      <x:c r="E610" t="str">
+        <x:v>Loads the champion ID from the committed party slot before making it the current champion.</x:v>
+      </x:c>
+      <x:c r="F610" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="611">
+      <x:c r="A611" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B611" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C611" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D611" t="str">
+        <x:v>move.w d0,$0006(a5)</x:v>
+      </x:c>
+      <x:c r="E611" t="str">
+        <x:v>Stores the selected champion ID as PlayerX_Data current champion, driving the name panel and large avatar.</x:v>
+      </x:c>
+      <x:c r="F611" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="612">
+      <x:c r="A612" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B612" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C612" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D612" t="str">
+        <x:v>move.w #$FFFF,$0016(a5)</x:v>
+      </x:c>
+      <x:c r="E612" t="str">
+        <x:v>Clears the pending party-slot selection after committing the current champion.</x:v>
+      </x:c>
+      <x:c r="F612" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="613">
+      <x:c r="A613" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B613" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C613" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D613" t="str">
+        <x:v>btst d7,$003E(a5)</x:v>
+      </x:c>
+      <x:c r="E613" t="str">
+        <x:v>Continues only for a party slot marked as the active selected member.</x:v>
+      </x:c>
+      <x:c r="F613" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="614">
+      <x:c r="A614" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B614" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C614" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D614" t="str">
+        <x:v>move.b $18(a5,d7.w),d1</x:v>
+      </x:c>
+      <x:c r="E614" t="str">
+        <x:v>Loads the party-slot state byte: low nibble is champion ID; bits $20/$40 suppress the living full-character rendering.</x:v>
+      </x:c>
+      <x:c r="F614" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="615">
+      <x:c r="A615" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B615" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C615" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D615" t="str">
+        <x:v>move.w ActivePartyChampionShieldDrawParameters(pc,d7.w),d4</x:v>
+      </x:c>
+      <x:c r="E615" t="str">
+        <x:v>Loads the selected champion X anchor: $11 for upper slot, then $08, $28 and $48 for the three shield slots.</x:v>
+      </x:c>
+      <x:c r="F615" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="616">
+      <x:c r="A616" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B616" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C616" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D616" t="str">
+        <x:v>move.w adrW_007EAA(pc,d7.w),d5</x:v>
+      </x:c>
+      <x:c r="E616" t="str">
+        <x:v>Loads the selected champion Y anchor: $1C for upper slot or $48 for a lower shield slot.</x:v>
+      </x:c>
+      <x:c r="F616" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="617">
+      <x:c r="A617" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B617" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C617" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D617" t="str">
+        <x:v>move.w adrW_007EAC(pc,d7.w),d1</x:v>
+      </x:c>
+      <x:c r="E617" t="str">
+        <x:v>Loads Draw_Character distance: $00 for the upper full-size champion and $01 for the lower one-step-away champion.</x:v>
+      </x:c>
+      <x:c r="F617" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="618">
+      <x:c r="A618" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B618" t="str">
+        <x:v>Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C618" t="str">
+        <x:v>Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="D618" t="str">
+        <x:v>bra Draw_Character</x:v>
+      </x:c>
+      <x:c r="E618" t="str">
+        <x:v>Tail-calls the multipart character renderer after passing front-facing direction, selected slot anchor, and distance.</x:v>
+      </x:c>
+      <x:c r="F618" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="619">
+      <x:c r="A619" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B619" t="str">
+        <x:v>Draw_PartyShieldSlot</x:v>
+      </x:c>
+      <x:c r="C619" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="D619" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_SelectedPartyShieldFrameOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="E619" t="str">
+        <x:v>Selects the 32 by 41 Pockets.gfx surround at $5070 for a living selected party member before drawing its multipart character.</x:v>
+      </x:c>
+      <x:c r="F619" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="620">
+      <x:c r="A620" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B620" t="str">
+        <x:v>Draw_SelectedPartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="C620" t="str">
+        <x:v>Return_PartyShieldDrawing</x:v>
+      </x:c>
+      <x:c r="D620" t="str">
+        <x:v>bsr Draw_ActivePartyChampionInShield</x:v>
+      </x:c>
+      <x:c r="E620" t="str">
+        <x:v>Draws the active champion as a full multipart character inside the already drawn selected shield surround.</x:v>
+      </x:c>
+      <x:c r="F620" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="621">
+      <x:c r="A621" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B621" t="str">
+        <x:v>Draw_ChampionNamePanelBackground</x:v>
+      </x:c>
+      <x:c r="C621" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="D621" t="str">
+        <x:v>move.l #$005E00E1,d4</x:v>
+      </x:c>
+      <x:c r="E621" t="str">
+        <x:v>Supplies BW_draw_bar with X=$E1 and DBRA width $5E, clearing a 95-pixel-wide right-hand panel from X=$E1 through $13F.</x:v>
+      </x:c>
+      <x:c r="F621" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="622">
+      <x:c r="A622" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B622" t="str">
+        <x:v>Draw_ChampionNamePanelBackground</x:v>
+      </x:c>
+      <x:c r="C622" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="D622" t="str">
+        <x:v>move.l #$00560009,d5</x:v>
+      </x:c>
+      <x:c r="E622" t="str">
+        <x:v>Supplies BW_draw_bar with Y=$09 and DBRA height $56, clearing 87 rows through player-local Y=$5F.</x:v>
+      </x:c>
+      <x:c r="F622" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="623">
+      <x:c r="A623" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B623" t="str">
+        <x:v>Draw_ChampionNamePanelBackground</x:v>
+      </x:c>
+      <x:c r="C623" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="D623" t="str">
+        <x:v>moveq #$00,d3</x:v>
+      </x:c>
+      <x:c r="E623" t="str">
+        <x:v>Uses palette index $00 to clear the champion-name panel background before the decorative frame is drawn.</x:v>
+      </x:c>
+      <x:c r="F623" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="624">
+      <x:c r="A624" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B624" t="str">
+        <x:v>Draw_ChampionNamePanelBackground</x:v>
+      </x:c>
+      <x:c r="C624" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="D624" t="str">
+        <x:v>bra BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E624" t="str">
+        <x:v>Fills the source-sized name/display panel rectangle using the packed dimensions in D4 and D5.</x:v>
+      </x:c>
+      <x:c r="F624" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="625">
+      <x:c r="A625" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B625" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C625" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D625" t="str">
+        <x:v>move.w #$00E2,d4</x:v>
+      </x:c>
+      <x:c r="E625" t="str">
+        <x:v>Sets the bevel-line X coordinate to $E2, one pixel inside the cleared panel's left edge.</x:v>
+      </x:c>
+      <x:c r="F625" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="626">
+      <x:c r="A626" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B626" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C626" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D626" t="str">
+        <x:v>moveq #$0A,d5</x:v>
+      </x:c>
+      <x:c r="E626" t="str">
+        <x:v>Starts the five-scanline upper grey bevel at player-local Y=$0A.</x:v>
+      </x:c>
+      <x:c r="F626" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="627">
+      <x:c r="A627" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B627" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C627" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D627" t="str">
+        <x:v>move.l #$005D0001,d3</x:v>
+      </x:c>
+      <x:c r="E627" t="str">
+        <x:v>Sets DBRA width $5D (94 pixels) and the first upper-bevel colour index $01.</x:v>
+      </x:c>
+      <x:c r="F627" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="628">
+      <x:c r="A628" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B628" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C628" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D628" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E628" t="str">
+        <x:v>Draws the upper bevel's four stepped grey lines at Y=$0A-$0D, then its final colour-$01 line at Y=$0E.</x:v>
+      </x:c>
+      <x:c r="F628" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="629">
+      <x:c r="A629" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B629" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C629" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D629" t="str">
+        <x:v>move.l #$00070010,d5</x:v>
+      </x:c>
+      <x:c r="E629" t="str">
+        <x:v>Supplies BW_draw_bar with the primary-colour name strip's Y=$10 and DBRA height $07, producing eight rows Y=$10-$17.</x:v>
+      </x:c>
+      <x:c r="F629" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="630">
+      <x:c r="A630" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B630" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C630" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D630" t="str">
+        <x:v>move.l #$005D00E2,d4</x:v>
+      </x:c>
+      <x:c r="E630" t="str">
+        <x:v>Supplies the primary-colour name strip's X=$E2 and DBRA width $5D, producing 94 pixels through X=$13F.</x:v>
+      </x:c>
+      <x:c r="F630" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="631">
+      <x:c r="A631" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B631" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C631" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D631" t="str">
+        <x:v>move.w $0010(a5),d3</x:v>
+      </x:c>
+      <x:c r="E631" t="str">
+        <x:v>Loads PlayerData_UIPrimaryColourOffset as the fill colour for the eight-pixel champion-name strip.</x:v>
+      </x:c>
+      <x:c r="F631" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="632">
+      <x:c r="A632" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B632" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C632" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D632" t="str">
+        <x:v>bsr BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E632" t="str">
+        <x:v>Fills the complete primary-colour champion-name strip before the lower grey bevel starts.</x:v>
+      </x:c>
+      <x:c r="F632" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="633">
+      <x:c r="A633" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B633" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C633" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D633" t="str">
+        <x:v>addq.w #$01,d5</x:v>
+      </x:c>
+      <x:c r="E633" t="str">
+        <x:v>Advances from the name bar's final Y=$17 to the lower bevel's first scanline at Y=$19, leaving Y=$18 as background.</x:v>
+      </x:c>
+      <x:c r="F633" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="634">
+      <x:c r="A634" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B634" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C634" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D634" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E634" t="str">
+        <x:v>Draws the four-scanline lower grey bevel at Y=$19-$1C with colour indices $01-$04.</x:v>
+      </x:c>
+      <x:c r="F634" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="635">
+      <x:c r="A635" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B635" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C635" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D635" t="str">
+        <x:v>moveq #$20,d5</x:v>
+      </x:c>
+      <x:c r="E635" t="str">
+        <x:v>Sets the mini status-icon bevel's first horizontal line to player-local Y=$20.</x:v>
+      </x:c>
+      <x:c r="F635" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="636">
+      <x:c r="A636" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B636" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C636" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D636" t="str">
+        <x:v>move.w #$0120,d4</x:v>
+      </x:c>
+      <x:c r="E636" t="str">
+        <x:v>Sets the mini status-icon bevel's X coordinate to $120, immediately right of the 64-pixel status graphic.</x:v>
+      </x:c>
+      <x:c r="F636" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="637">
+      <x:c r="A637" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B637" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C637" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D637" t="str">
+        <x:v>move.l #$001F0001,d3</x:v>
+      </x:c>
+      <x:c r="E637" t="str">
+        <x:v>Sets the mini bevel's DBRA width $1F (32 pixels) and initial grey colour index $01.</x:v>
+      </x:c>
+      <x:c r="F637" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="638">
+      <x:c r="A638" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B638" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C638" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D638" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E638" t="str">
+        <x:v>Draws the mini bevel's top line at Y=$20 and its icon-height divider at Y=$31.</x:v>
+      </x:c>
+      <x:c r="F638" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="639">
+      <x:c r="A639" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B639" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C639" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D639" t="str">
+        <x:v>add.w #$0011,d5</x:v>
+      </x:c>
+      <x:c r="E639" t="str">
+        <x:v>Moves from the top mini-bevel line to Y=$31, immediately below the 16-pixel status-icon row.</x:v>
+      </x:c>
+      <x:c r="F639" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="640">
+      <x:c r="A640" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B640" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C640" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D640" t="str">
+        <x:v>addq.w #$02,d5</x:v>
+      </x:c>
+      <x:c r="E640" t="str">
+        <x:v>Moves from the divider to player-local Y=$33 for the stepped lower part of the mini bevel.</x:v>
+      </x:c>
+      <x:c r="F640" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="641">
+      <x:c r="A641" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B641" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="C641" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="D641" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E641" t="str">
+        <x:v>Draws the mini bevel's lower scale at Y=$33-$37: colour $01, then $02-$04, then $01.</x:v>
+      </x:c>
+      <x:c r="F641" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="642">
+      <x:c r="A642" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B642" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C642" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D642" t="str">
+        <x:v>moveq #$00,d7</x:v>
+      </x:c>
+      <x:c r="E642" t="str">
+        <x:v>Starts the four party-position profession-control loop at slot zero.</x:v>
+      </x:c>
+      <x:c r="F642" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="643">
+      <x:c r="A643" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B643" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C643" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D643" t="str">
+        <x:v>add.w adrW_00838E(pc,d2.w),a0</x:v>
+      </x:c>
+      <x:c r="E643" t="str">
+        <x:v>Applies the compact four-slot screen-offset sequence for profession controls: upper-left, upper-right, lower-right, lower-left.</x:v>
+      </x:c>
+      <x:c r="F643" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="644">
+      <x:c r="A644" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B644" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C644" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D644" t="str">
+        <x:v>move.b $26(a5,d7.w),d0</x:v>
+      </x:c>
+      <x:c r="E644" t="str">
+        <x:v>Loads the champion assigned to this party position; a negative entry selects the empty profession-control icon.</x:v>
+      </x:c>
+      <x:c r="F644" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="645">
+      <x:c r="A645" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B645" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C645" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D645" t="str">
+        <x:v>cmp.w $0016(a5),d7</x:v>
+      </x:c>
+      <x:c r="E645" t="str">
+        <x:v>Tests whether this party position is the pending first click; that path draws its profession icon with the neutral grey mask.</x:v>
+      </x:c>
+      <x:c r="F645" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="646">
+      <x:c r="A646" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B646" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C646" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D646" t="str">
+        <x:v>bsr adrCd008430</x:v>
+      </x:c>
+      <x:c r="E646" t="str">
+        <x:v>Draws an occupied party position's $4B-$4E profession icon using the assigned champion's class colour mask.</x:v>
+      </x:c>
+      <x:c r="F646" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="647">
+      <x:c r="A647" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B647" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C647" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D647" t="str">
+        <x:v>bsr adrCd00842C</x:v>
+      </x:c>
+      <x:c r="E647" t="str">
+        <x:v>Draws the pending selected position's profession icon using the neutral mask at adrEA00846A, making it grey.</x:v>
+      </x:c>
+      <x:c r="F647" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="648">
+      <x:c r="A648" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B648" t="str">
+        <x:v>adrCd008462</x:v>
+      </x:c>
+      <x:c r="C648" t="str">
+        <x:v>adrCd00847E</x:v>
+      </x:c>
+      <x:c r="D648" t="str">
+        <x:v>move.w #$003B,d0</x:v>
+      </x:c>
+      <x:c r="E648" t="str">
+        <x:v>Selects Pockets icon $3B for an empty party position.</x:v>
+      </x:c>
+      <x:c r="F648" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="649">
+      <x:c r="A649" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B649" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C649" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D649" t="str">
+        <x:v>move.w $0010(a5),d3</x:v>
+      </x:c>
+      <x:c r="E649" t="str">
+        <x:v>Loads the active player's primary UI colour for the frame surrounding the current lead champion's profession icon.</x:v>
+      </x:c>
+      <x:c r="F649" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="650">
+      <x:c r="A650" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B650" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C650" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D650" t="str">
+        <x:v>move.l #$000F0121,d4</x:v>
+      </x:c>
+      <x:c r="E650" t="str">
+        <x:v>Supplies the lead-profession frame's DBRA width $0F and base X=$121; the slot lookup shifts right-hand frames to X=$131.</x:v>
+      </x:c>
+      <x:c r="F650" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="651">
+      <x:c r="A651" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B651" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C651" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D651" t="str">
+        <x:v>move.l #$000D0039,d5</x:v>
+      </x:c>
+      <x:c r="E651" t="str">
+        <x:v>Supplies the lead-profession frame's DBRA height $0D and upper-row Y=$39; lower slots are shifted to Y=$48.</x:v>
+      </x:c>
+      <x:c r="F651" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="652">
+      <x:c r="A652" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B652" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C652" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D652" t="str">
+        <x:v>bra BW_draw_frame</x:v>
+      </x:c>
+      <x:c r="E652" t="str">
+        <x:v>Draws the 16 by 14 primary-colour frame identifying the current lead champion's profession control.</x:v>
+      </x:c>
+      <x:c r="F652" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="653">
+      <x:c r="A653" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B653" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C653" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D653" t="str">
+        <x:v>tst.w $0042(a5)</x:v>
+      </x:c>
+      <x:c r="E653" t="str">
+        <x:v>Tests PlayerX_Data party-command state: a non-negative value takes the ordinary compact portrait/shield redraw path, while $FFFF enters the dirty selected-character redraw path.</x:v>
+      </x:c>
+      <x:c r="F653" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="654">
+      <x:c r="A654" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B654" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C654" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D654" t="str">
+        <x:v>bmi Refresh_DirtyPartyShieldSlots</x:v>
+      </x:c>
+      <x:c r="E654" t="str">
+        <x:v>Branches only for the negative team-avatar state, allowing individually selected living slots to use Draw_Character rather than their compact avatar graphics.</x:v>
+      </x:c>
+      <x:c r="F654" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="655">
+      <x:c r="A655" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B655" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C655" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D655" t="str">
+        <x:v>bsr Draw_MainChampionAvatarPanel</x:v>
+      </x:c>
+      <x:c r="E655" t="str">
+        <x:v>Draws the default large 32 by 30 avatar panel before any full-length party-character rendering is requested.</x:v>
+      </x:c>
+      <x:c r="F655" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="656">
+      <x:c r="A656" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B656" t="str">
+        <x:v>Click_ShowTeamAvatars</x:v>
+      </x:c>
+      <x:c r="C656" t="str">
+        <x:v>PartyCommand_DispatchSelection</x:v>
+      </x:c>
+      <x:c r="D656" t="str">
+        <x:v>move.w #$FFFF,$0042(a5)</x:v>
+      </x:c>
+      <x:c r="E656" t="str">
+        <x:v>Enters the negative team-avatar state consumed by Draw_PartyCommandInterface; the dirty slot renderer then uses each selected-slot bit to choose full-length drawing.</x:v>
+      </x:c>
+      <x:c r="F656" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="657">
+      <x:c r="A657" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B657" t="str">
+        <x:v>Click_CommsAndOptions</x:v>
+      </x:c>
+      <x:c r="C657" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D657" t="str">
+        <x:v>cmpi.w #$0037,d1</x:v>
+      </x:c>
+      <x:c r="E657" t="str">
+        <x:v>Separates the upper large-avatar selection from the lower shield-slot selection path before the selected PlayerX_Data+$003E bit is toggled.</x:v>
+      </x:c>
+      <x:c r="F657" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="658">
+      <x:c r="A658" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B658" t="str">
+        <x:v>Click_CommsAndOptions</x:v>
+      </x:c>
+      <x:c r="C658" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D658" t="str">
+        <x:v>lsr.w #$05,d1</x:v>
+      </x:c>
+      <x:c r="E658" t="str">
+        <x:v>Converts the lower shield-click X coordinate to a 32-pixel column index; the following add selects PlayerX_Data+$003E bits one through three.</x:v>
+      </x:c>
+      <x:c r="F658" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="659">
+      <x:c r="A659" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B659" t="str">
+        <x:v>Click_CommsAndOptions</x:v>
+      </x:c>
+      <x:c r="C659" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D659" t="str">
+        <x:v>bchg d1,$003E(a5)</x:v>
+      </x:c>
+      <x:c r="E659" t="str">
+        <x:v>Toggles only the clicked left-side avatar's presentation bit. This is independent of right-side Click_PartyMember actions $06-$09.</x:v>
+      </x:c>
+      <x:c r="F659" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="660">
+      <x:c r="A660" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B660" t="str">
+        <x:v>Click_CommsAndOptions</x:v>
+      </x:c>
+      <x:c r="C660" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D660" t="str">
+        <x:v>bsr Refresh_PartyShieldSlotIfDirty</x:v>
+      </x:c>
+      <x:c r="E660" t="str">
+        <x:v>Refreshes the clicked party shield slot after changing its presentation bit; the selected living path draws the one-step-away full character.</x:v>
+      </x:c>
+      <x:c r="F660" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="661">
+      <x:c r="A661" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B661" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C661" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D661" t="str">
+        <x:v>tst.b $26(a5,d0.w)</x:v>
+      </x:c>
+      <x:c r="E661" t="str">
+        <x:v>Tests for an empty destination only when no party slot is pending. Once a living slot is pending, the later byte-exchange path permits moving it into an empty profession-icon slot.</x:v>
+      </x:c>
+      <x:c r="F661" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="662">
+      <x:c r="A662" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B662" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C662" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D662" t="str">
+        <x:v>bsr adrCd004078</x:v>
+      </x:c>
+      <x:c r="E662" t="str">
+        <x:v>Finds the selected champion's current left avatar slot in PlayerX_Data+$18 before replacing the current leader.</x:v>
+      </x:c>
+      <x:c r="F662" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="663">
+      <x:c r="A663" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B663" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C663" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D663" t="str">
+        <x:v>move.b d2,$18(a5,d1.w)</x:v>
+      </x:c>
+      <x:c r="E663" t="str">
+        <x:v>Writes the former leader into the selected champion's previous left avatar slot, refreshing the lower avatar arrangement after a confirmed lead change.</x:v>
+      </x:c>
+      <x:c r="F663" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="664">
+      <x:c r="A664" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B664" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C664" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D664" t="str">
+        <x:v>move.b d0,$0018(a5)</x:v>
+      </x:c>
+      <x:c r="E664" t="str">
+        <x:v>Writes the confirmed new leader into the large-avatar slot at PlayerX_Data+$18; this is separate from the right-side profession-order bytes at $26.</x:v>
+      </x:c>
+      <x:c r="F664" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="665">
+      <x:c r="A665" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B665" t="str">
+        <x:v>Click_PartyMember</x:v>
+      </x:c>
+      <x:c r="C665" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="D665" t="str">
+        <x:v>bset #$04,$0018(a5)</x:v>
+      </x:c>
+      <x:c r="E665" t="str">
+        <x:v>Marks the new large-avatar slot active after its champion ID has been written.</x:v>
+      </x:c>
+      <x:c r="F665" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="666">
+      <x:c r="A666" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B666" t="str">
+        <x:v>Draw_PartyShieldSlot</x:v>
+      </x:c>
+      <x:c r="C666" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="D666" t="str">
+        <x:v>move.b $18(a5,d0.w),d7</x:v>
+      </x:c>
+      <x:c r="E666" t="str">
+        <x:v>Loads the complete left avatar-state byte for this party slot, retaining its champion ID and status bits while positions are refreshed.</x:v>
+      </x:c>
+      <x:c r="F666" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="667">
+      <x:c r="A667" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B667" t="str">
+        <x:v>Select_PartyShieldClassColours</x:v>
+      </x:c>
+      <x:c r="C667" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="D667" t="str">
+        <x:v>btst #$06,d7</x:v>
+      </x:c>
+      <x:c r="E667" t="str">
+        <x:v>Tests the avatar-state dead flag. A dead member uses the fixed dead shield colours and is not eligible for selected living-character drawing.</x:v>
+      </x:c>
+      <x:c r="F667" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="668">
+      <x:c r="A668" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B668" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C668" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D668" t="str">
+        <x:v>moveq #$38,d5</x:v>
+      </x:c>
+      <x:c r="E668" t="str">
+        <x:v>Supplies Draw_ChampionStats with the scroll's DBRA height $38; Draw_ScrollFrame uses this to fill the 57-row centre between its 15-row caps.</x:v>
+      </x:c>
+      <x:c r="F668" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="669">
+      <x:c r="A669" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B669" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C669" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D669" t="str">
+        <x:v>move.w #$00C7,d1</x:v>
+      </x:c>
+      <x:c r="E669" t="str">
+        <x:v>Sets $C7 as the champion food-byte value that represents a completely filled food bar.</x:v>
+      </x:c>
+      <x:c r="F669" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="670">
+      <x:c r="A670" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B670" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C670" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D670" t="str">
+        <x:v>moveq #$30,d2</x:v>
+      </x:c>
+      <x:c r="E670" t="str">
+        <x:v>Sets the food bar's maximum scaled length to $30, yielding 48 rendered pixels.</x:v>
+      </x:c>
+      <x:c r="F670" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="671">
+      <x:c r="A671" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B671" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C671" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D671" t="str">
+        <x:v>move.l #$002F00F9,d4</x:v>
+      </x:c>
+      <x:c r="E671" t="str">
+        <x:v>Supplies BW_draw_bar with X=$F9 and DBRA width $2F, drawing the food fill across 48 pixels through X=$128.</x:v>
+      </x:c>
+      <x:c r="F671" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="672">
+      <x:c r="A672" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B672" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C672" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D672" t="str">
+        <x:v>move.l #$0004004A,d5</x:v>
+      </x:c>
+      <x:c r="E672" t="str">
+        <x:v>Supplies BW_draw_bar with Y=$4A and DBRA height $04, drawing a five-row food bar through Y=$4E.</x:v>
+      </x:c>
+      <x:c r="F672" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="673">
+      <x:c r="A673" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B673" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C673" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D673" t="str">
+        <x:v>moveq #$09,d3</x:v>
+      </x:c>
+      <x:c r="E673" t="str">
+        <x:v>Selects palette index $09 for the scaled champion food-bar fill.</x:v>
+      </x:c>
+      <x:c r="F673" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="674">
+      <x:c r="A674" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B674" t="str">
+        <x:v>Click_ShowStats</x:v>
+      </x:c>
+      <x:c r="C674" t="str">
+        <x:v>Load_CurrentChampionStatRecord</x:v>
+      </x:c>
+      <x:c r="D674" t="str">
+        <x:v>lea ChampionStatsScroll_FoodTextTemplate.l,a6</x:v>
+      </x:c>
+      <x:c r="E674" t="str">
+        <x:v>Selects the FOOD Print_fflim_text stream: heading row $08 followed by end-cap glyph row $09, each printer row eight pixels apart.</x:v>
+      </x:c>
+      <x:c r="F674" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="675">
+      <x:c r="A675" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B675" t="str">
+        <x:v>Draw_ChampionStats</x:v>
+      </x:c>
+      <x:c r="C675" t="str">
+        <x:v>Draw_ScrollFrame</x:v>
+      </x:c>
+      <x:c r="D675" t="str">
+        <x:v>lea ChampionStatsScroll_TextTemplate.l,a6</x:v>
+      </x:c>
+      <x:c r="E675" t="str">
+        <x:v>Selects the stats Print_fflim_text stream. Its $FC commands place LEVEL and the ST, IN, HP, and VI rows at consecutive eight-pixel text rows $03-$07.</x:v>
+      </x:c>
+      <x:c r="F675" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="676">
+      <x:c r="A676" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B676" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C676" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D676" t="str">
+        <x:v>move.l #$005D00E2,d4</x:v>
+      </x:c>
+      <x:c r="E676" t="str">
+        <x:v>Supplies BW_draw_bar with the inventory title bar X=$E2 and DBRA width $5D, producing 94 pixels through X=$13F.</x:v>
+      </x:c>
+      <x:c r="F676" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="677">
+      <x:c r="A677" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B677" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C677" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D677" t="str">
+        <x:v>move.l #$00070018,d5</x:v>
+      </x:c>
+      <x:c r="E677" t="str">
+        <x:v>Supplies the inventory title bar Y=$18 and DBRA height $07, producing eight rows through Y=$1F.</x:v>
+      </x:c>
+      <x:c r="F677" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="678">
+      <x:c r="A678" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B678" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C678" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D678" t="str">
+        <x:v>move.w #$0040,d5</x:v>
+      </x:c>
+      <x:c r="E678" t="str">
+        <x:v>Selects the armour bar Y=$40 after the title bar has been drawn.</x:v>
+      </x:c>
+      <x:c r="F678" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="679">
+      <x:c r="A679" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B679" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C679" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D679" t="str">
+        <x:v>move.l #$0000029C,a0</x:v>
+      </x:c>
+      <x:c r="E679" t="str">
+        <x:v>Uses screen offset $029C for the upper GFX_Pockets inventory-chain strip; this resolves to player-local X=$E0/Y=$10.</x:v>
+      </x:c>
+      <x:c r="F679" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="680">
+      <x:c r="A680" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B680" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C680" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D680" t="str">
+        <x:v>move.l #$00000B5C,a0</x:v>
+      </x:c>
+      <x:c r="E680" t="str">
+        <x:v>Uses screen offset $0B5C for the lower GFX_Pockets inventory-chain strip; this resolves to player-local X=$E0/Y=$48.</x:v>
+      </x:c>
+      <x:c r="F680" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="681">
+      <x:c r="A681" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B681" t="str">
+        <x:v>adrJA00C938</x:v>
+      </x:c>
+      <x:c r="C681" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="D681" t="str">
+        <x:v>lea adrEA00EA14.l,a6</x:v>
+      </x:c>
+      <x:c r="E681" t="str">
+        <x:v>Selects the inventory title Print_fflim_text template. Its text cell is later overwritten with the inspected champion name by the inventory redraw path.</x:v>
+      </x:c>
+      <x:c r="F681" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="682">
+      <x:c r="A682" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B682" t="str">
+        <x:v>adrCd008358</x:v>
+      </x:c>
+      <x:c r="C682" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="D682" t="str">
+        <x:v>lea adrEA050302.l,a1</x:v>
+      </x:c>
+      <x:c r="E682" t="str">
+        <x:v>Uses the packed inventory interface strip at GFX_Pockets+$3C00 as the source graphic for each inventory chain decoration.</x:v>
+      </x:c>
+      <x:c r="F682" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="683">
+      <x:c r="A683" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B683" t="str">
+        <x:v>adrCd008358</x:v>
+      </x:c>
+      <x:c r="C683" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="D683" t="str">
+        <x:v>move.l #$00050006,d5</x:v>
+      </x:c>
+      <x:c r="E683" t="str">
+        <x:v>Sets the chain-strip DBRA dimensions used for both inventory decoration anchors.</x:v>
+      </x:c>
+      <x:c r="F683" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="684">
+      <x:c r="A684" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B684" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="C684" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="D684" t="str">
+        <x:v>bsr Calculate_CharacterArmourLevel</x:v>
+      </x:c>
+      <x:c r="E684" t="str">
+        <x:v>Calculates the selected champion's effective armour level before the inventory modifier is formatted.</x:v>
+      </x:c>
+      <x:c r="F684" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="685">
+      <x:c r="A685" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B685" t="str">
+        <x:v>adrCd00C984</x:v>
+      </x:c>
+      <x:c r="C685" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="D685" t="str">
+        <x:v>moveq #$0A,d0</x:v>
+      </x:c>
+      <x:c r="E685" t="str">
+        <x:v>Starts the displayed armour modifier from baseline 10; the calculated armour level is subtracted to produce the signed three-character result.</x:v>
+      </x:c>
+      <x:c r="F685" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="686">
+      <x:c r="A686" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B686" t="str">
+        <x:v>adrCd00C9A0</x:v>
+      </x:c>
+      <x:c r="C686" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="D686" t="str">
+        <x:v>lea adrEA00EA25.l,a6</x:v>
+      </x:c>
+      <x:c r="E686" t="str">
+        <x:v>Selects the writable ARMOUR text template whose last three characters receive the sign and decimal digits.</x:v>
+      </x:c>
+      <x:c r="F686" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="687">
+      <x:c r="A687" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B687" t="str">
+        <x:v>adrCd00C9A0</x:v>
+      </x:c>
+      <x:c r="C687" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="D687" t="str">
+        <x:v>bsr Convert_ByteToDecimalText</x:v>
+      </x:c>
+      <x:c r="E687" t="str">
+        <x:v>Converts the absolute armour difference into the two decimal characters stored in the inventory ARMOUR template.</x:v>
+      </x:c>
+      <x:c r="F687" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="688">
+      <x:c r="A688" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B688" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="C688" t="str">
+        <x:v>adrCd00CA66</x:v>
+      </x:c>
+      <x:c r="D688" t="str">
+        <x:v>add.w #$051C,a0</x:v>
+      </x:c>
+      <x:c r="E688" t="str">
+        <x:v>Starts the first six inventory slots at screen offset $051C, player-local X=$E0/Y=$20.</x:v>
+      </x:c>
+      <x:c r="F688" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="689">
+      <x:c r="A689" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B689" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="C689" t="str">
+        <x:v>adrCd00CA66</x:v>
+      </x:c>
+      <x:c r="D689" t="str">
+        <x:v>add.w #$0274,a0</x:v>
+      </x:c>
+      <x:c r="E689" t="str">
+        <x:v>After the sixth 16-pixel pocket, advances to the second six-slot row at player-local Y=$30.</x:v>
+      </x:c>
+      <x:c r="F689" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="690">
+      <x:c r="A690" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B690" t="str">
+        <x:v>Draw_HeldItemPanel</x:v>
+      </x:c>
+      <x:c r="C690" t="str">
+        <x:v>adrCd006C90</x:v>
+      </x:c>
+      <x:c r="D690" t="str">
+        <x:v>add.w #$0B5C,a0</x:v>
+      </x:c>
+      <x:c r="E690" t="str">
+        <x:v>Starts the lower inventory panel at player-local X=$E0/Y=$48, after the page has supplied the shared lower chain strip.</x:v>
+      </x:c>
+      <x:c r="F690" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="691">
+      <x:c r="A691" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B691" t="str">
+        <x:v>Draw_HeldItemPanel</x:v>
+      </x:c>
+      <x:c r="C691" t="str">
+        <x:v>adrCd006C90</x:v>
+      </x:c>
+      <x:c r="D691" t="str">
+        <x:v>moveq #$00,d7</x:v>
+      </x:c>
+      <x:c r="E691" t="str">
+        <x:v>Initialises the four-position inventory profession-icon loop.</x:v>
+      </x:c>
+      <x:c r="F691" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="692">
+      <x:c r="A692" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B692" t="str">
+        <x:v>Draw_HeldItemPanel</x:v>
+      </x:c>
+      <x:c r="C692" t="str">
+        <x:v>adrCd006C90</x:v>
+      </x:c>
+      <x:c r="D692" t="str">
+        <x:v>moveq #$74,d0</x:v>
+      </x:c>
+      <x:c r="E692" t="str">
+        <x:v>Selects the fixed empty held-item pocket graphic placed after the four profession positions.</x:v>
+      </x:c>
+      <x:c r="F692" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="693">
+      <x:c r="A693" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B693" t="str">
+        <x:v>Draw_HeldItemPanel</x:v>
+      </x:c>
+      <x:c r="C693" t="str">
+        <x:v>adrCd006C90</x:v>
+      </x:c>
+      <x:c r="D693" t="str">
+        <x:v>bsr adrCd006D1E</x:v>
+      </x:c>
+      <x:c r="E693" t="str">
+        <x:v>Draws the yellow 16 by 15 selection frame around the party position stored at PlayerX_Data+$000F.</x:v>
+      </x:c>
+      <x:c r="F693" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="694">
+      <x:c r="A694" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B694" t="str">
+        <x:v>adrCd006D1E</x:v>
+      </x:c>
+      <x:c r="C694" t="str">
+        <x:v>adrCd006D3C</x:v>
+      </x:c>
+      <x:c r="D694" t="str">
+        <x:v>move.l #$000E0049,d5</x:v>
+      </x:c>
+      <x:c r="E694" t="str">
+        <x:v>Sets the inventory profession-selection frame's DBRA height $0E and Y=$49, one pixel below the lower strip's Y=$48 anchor.</x:v>
+      </x:c>
+      <x:c r="F694" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="695">
+      <x:c r="A695" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B695" t="str">
+        <x:v>adrCd006D1E</x:v>
+      </x:c>
+      <x:c r="C695" t="str">
+        <x:v>adrCd006D3C</x:v>
+      </x:c>
+      <x:c r="D695" t="str">
+        <x:v>add.w #$00E1,d4</x:v>
+      </x:c>
+      <x:c r="E695" t="str">
+        <x:v>Places the selection frame at X=$E1 plus sixteen pixels per selected party position.</x:v>
+      </x:c>
+      <x:c r="F695" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="696">
+      <x:c r="A696" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B696" t="str">
+        <x:v>Calculate_CharacterArmourLevel</x:v>
+      </x:c>
+      <x:c r="C696" t="str">
+        <x:v>adrCd006382</x:v>
+      </x:c>
+      <x:c r="D696" t="str">
+        <x:v>move.b $0002(a1),d2</x:v>
+      </x:c>
+      <x:c r="E696" t="str">
+        <x:v>Reads the selected champion's body-armour pocket before converting body armour object IDs into armour protection.</x:v>
+      </x:c>
+      <x:c r="F696" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="697">
+      <x:c r="A697" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B697" t="str">
+        <x:v>Calculate_CharacterArmourLevel</x:v>
+      </x:c>
+      <x:c r="C697" t="str">
+        <x:v>adrCd006382</x:v>
+      </x:c>
+      <x:c r="D697" t="str">
+        <x:v>move.b $0012(a4),d2</x:v>
+      </x:c>
+      <x:c r="E697" t="str">
+        <x:v>Reads the worn-hand-armour object and adds its source-defined protection after body and spell protection have been resolved.</x:v>
+      </x:c>
+      <x:c r="F697" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="698">
+      <x:c r="A698" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B698" t="str">
+        <x:v>Calculate_CharacterArmourLevel</x:v>
+      </x:c>
+      <x:c r="C698" t="str">
+        <x:v>adrCd006382</x:v>
+      </x:c>
+      <x:c r="D698" t="str">
+        <x:v>move.b $0003(a1),d2</x:v>
+      </x:c>
+      <x:c r="E698" t="str">
+        <x:v>Reads the shield pocket and adds the matching protection byte only for object IDs $24 through $2A.</x:v>
+      </x:c>
+      <x:c r="F698" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
improved spellbook view UI
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L508"/>
+  <dimension ref="A1:L509"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -26075,6 +26075,66 @@
       <c r="L508" s="8" t="inlineStr">
         <is>
           <t>High word $0001 produces two planar words (32 pixels); low word $001D produces 30 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B509" s="8" t="inlineStr">
+        <is>
+          <t>SpellBook_PageSpreadIncrement</t>
+        </is>
+      </c>
+      <c r="C509" s="8" t="inlineStr">
+        <is>
+          <t>$0002</t>
+        </is>
+      </c>
+      <c r="D509" s="8" t="inlineStr">
+        <is>
+          <t>Click_TurnSpellBookPage</t>
+        </is>
+      </c>
+      <c r="E509" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C322</t>
+        </is>
+      </c>
+      <c r="F509" s="8" t="inlineStr">
+        <is>
+          <t>addq.w #$02,$002A(a5)</t>
+        </is>
+      </c>
+      <c r="G509" s="8" t="inlineStr">
+        <is>
+          <t>546D002A</t>
+        </is>
+      </c>
+      <c r="H509" s="8" t="inlineStr">
+        <is>
+          <t>addq.w #SpellBook_PageSpreadIncrement,$002A(a5)</t>
+        </is>
+      </c>
+      <c r="I509" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J509" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K509" s="8" t="inlineStr">
+        <is>
+          <t>Advances the spell book by one two-page spread.</t>
+        </is>
+      </c>
+      <c r="L509" s="8" t="inlineStr">
+        <is>
+          <t>The page word is masked to $0007 immediately afterwards, selecting one of four two-page spreads.</t>
         </is>
       </c>
     </row>
@@ -26148,7 +26208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F737"/>
+  <dimension ref="A1:F824"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -49425,6 +49485,2616 @@
         </is>
       </c>
       <c r="F737" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B738" s="8" t="inlineStr">
+        <is>
+          <t>Draw_SpellPointValues</t>
+        </is>
+      </c>
+      <c r="C738" s="8" t="inlineStr">
+        <is>
+          <t>adrJA00C852</t>
+        </is>
+      </c>
+      <c r="D738" s="8" t="inlineStr">
+        <is>
+          <t>move.b $0009(a4),d0</t>
+        </is>
+      </c>
+      <c r="E738" s="8" t="inlineStr">
+        <is>
+          <t>Loads the champion's current spell points for the SP.PTS value.</t>
+        </is>
+      </c>
+      <c r="F738" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B739" s="8" t="inlineStr">
+        <is>
+          <t>Draw_SpellPointValues</t>
+        </is>
+      </c>
+      <c r="C739" s="8" t="inlineStr">
+        <is>
+          <t>adrJA00C852</t>
+        </is>
+      </c>
+      <c r="D739" s="8" t="inlineStr">
+        <is>
+          <t>move.b $000A(a4),d0</t>
+        </is>
+      </c>
+      <c r="E739" s="8" t="inlineStr">
+        <is>
+          <t>Loads the champion's maximum spell points for the SP.PTS value.</t>
+        </is>
+      </c>
+      <c r="F739" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B740" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C740" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D740" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$36,d4</t>
+        </is>
+      </c>
+      <c r="E740" s="8" t="inlineStr">
+        <is>
+          <t>Sets the compact STATS frame's upper bevel left edge to player-local X=$36.</t>
+        </is>
+      </c>
+      <c r="F740" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B741" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C741" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D741" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$0A,d5</t>
+        </is>
+      </c>
+      <c r="E741" s="8" t="inlineStr">
+        <is>
+          <t>Sets the compact STATS frame's upper bevel to player-local Y=$0A before the player screen Y offset is added.</t>
+        </is>
+      </c>
+      <c r="F741" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B742" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C742" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D742" s="8" t="inlineStr">
+        <is>
+          <t>add.w $0008(a5),d5</t>
+        </is>
+      </c>
+      <c r="E742" s="8" t="inlineStr">
+        <is>
+          <t>Applies the active player's screen Y offset to the current drawing coordinate.</t>
+        </is>
+      </c>
+      <c r="F742" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B743" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C743" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D743" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_blit_horiz_line</t>
+        </is>
+      </c>
+      <c r="E743" s="8" t="inlineStr">
+        <is>
+          <t>Calls the horizontal-line drawing routine for one bevel edge segment.</t>
+        </is>
+      </c>
+      <c r="F743" s="8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B744" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C744" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D744" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$31,d5</t>
+        </is>
+      </c>
+      <c r="E744" s="8" t="inlineStr">
+        <is>
+          <t>Sets the first lower STATS-frame bevel line to player-local Y=$31.</t>
+        </is>
+      </c>
+      <c r="F744" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B745" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C745" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D745" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$33,d4</t>
+        </is>
+      </c>
+      <c r="E745" s="8" t="inlineStr">
+        <is>
+          <t>Sets the first lower STATS-frame bevel line to player-local X=$33.</t>
+        </is>
+      </c>
+      <c r="F745" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B746" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C746" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D746" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$10,d5</t>
+        </is>
+      </c>
+      <c r="E746" s="8" t="inlineStr">
+        <is>
+          <t>Sets the two vertical STATS-frame side lines to start at player-local Y=$10.</t>
+        </is>
+      </c>
+      <c r="F746" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B747" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C747" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D747" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$34,d4</t>
+        </is>
+      </c>
+      <c r="E747" s="8" t="inlineStr">
+        <is>
+          <t>Sets the left vertical STATS-frame side line to player-local X=$34.</t>
+        </is>
+      </c>
+      <c r="F747" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B748" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C748" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D748" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_blit_vertical_line</t>
+        </is>
+      </c>
+      <c r="E748" s="8" t="inlineStr">
+        <is>
+          <t>Calls the vertical-line drawing routine for a STATS-frame side edge.</t>
+        </is>
+      </c>
+      <c r="F748" s="8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B749" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C749" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D749" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$5C,d4</t>
+        </is>
+      </c>
+      <c r="E749" s="8" t="inlineStr">
+        <is>
+          <t>Sets the right vertical STATS-frame side line to player-local X=$5C.</t>
+        </is>
+      </c>
+      <c r="F749" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B750" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C750" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D750" s="8" t="inlineStr">
+        <is>
+          <t>move.w #$001F,d5</t>
+        </is>
+      </c>
+      <c r="E750" s="8" t="inlineStr">
+        <is>
+          <t>Sets the STATS background rectangle to player-local Y=$1F after packing its height into D5.</t>
+        </is>
+      </c>
+      <c r="F750" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B751" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C751" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D751" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_draw_bar</t>
+        </is>
+      </c>
+      <c r="E751" s="8" t="inlineStr">
+        <is>
+          <t>Calls the filled-rectangle drawing routine for the compact STATS background.</t>
+        </is>
+      </c>
+      <c r="F751" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B752" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C752" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D752" s="8" t="inlineStr">
+        <is>
+          <t>move.l screen_ptr.l,a0</t>
+        </is>
+      </c>
+      <c r="E752" s="8" t="inlineStr">
+        <is>
+          <t>Starts from the player framebuffer before positioning the packed STATS title graphic.</t>
+        </is>
+      </c>
+      <c r="F752" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B753" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C753" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D753" s="8" t="inlineStr">
+        <is>
+          <t>add.w #$0286,a0</t>
+        </is>
+      </c>
+      <c r="E753" s="8" t="inlineStr">
+        <is>
+          <t>Places the packed STATS title graphic at its native compact-panel framebuffer offset.</t>
+        </is>
+      </c>
+      <c r="F753" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B754" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsFrame</t>
+        </is>
+      </c>
+      <c r="C754" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D754" s="8" t="inlineStr">
+        <is>
+          <t>bsr Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="E754" s="8" t="inlineStr">
+        <is>
+          <t>Calls the common four-plane graphic renderer for the pre-drawn STATS title.</t>
+        </is>
+      </c>
+      <c r="F754" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B755" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C755" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D755" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$00240036,d4</t>
+        </is>
+      </c>
+      <c r="E755" s="8" t="inlineStr">
+        <is>
+          <t>Packs compact-bar background X=$36 and horizontal terminal count $24, producing a 37-pixel-wide rectangle.</t>
+        </is>
+      </c>
+      <c r="F755" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B756" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C756" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D756" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$00160017,d5</t>
+        </is>
+      </c>
+      <c r="E756" s="8" t="inlineStr">
+        <is>
+          <t>Packs compact-bar background Y=$17 and vertical terminal count $16, producing 23 rows.</t>
+        </is>
+      </c>
+      <c r="F756" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B757" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C757" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D757" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_draw_bar</t>
+        </is>
+      </c>
+      <c r="E757" s="8" t="inlineStr">
+        <is>
+          <t>Calls the filled-rectangle drawing routine for the compact-stat bar background.</t>
+        </is>
+      </c>
+      <c r="F757" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B758" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C758" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D758" s="8" t="inlineStr">
+        <is>
+          <t>btst #$00,$003E(a5)</t>
+        </is>
+      </c>
+      <c r="E758" s="8" t="inlineStr">
+        <is>
+          <t>Chooses individual compact stats when no champion presentation is expanded; otherwise enters the party-shield status-bar path.</t>
+        </is>
+      </c>
+      <c r="F758" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B759" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C759" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D759" s="8" t="inlineStr">
+        <is>
+          <t>move.w $0006(a5),d7</t>
+        </is>
+      </c>
+      <c r="E759" s="8" t="inlineStr">
+        <is>
+          <t>Loads the current leader champion ID for the ordinary three-bar compact-stat display.</t>
+        </is>
+      </c>
+      <c r="F759" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B760" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C760" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D760" s="8" t="inlineStr">
+        <is>
+          <t>asl.w #$05,d7</t>
+        </is>
+      </c>
+      <c r="E760" s="8" t="inlineStr">
+        <is>
+          <t>Converts the champion ID to its 32-byte Character_Stats_DataTable record offset.</t>
+        </is>
+      </c>
+      <c r="F760" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B761" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C761" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D761" s="8" t="inlineStr">
+        <is>
+          <t>lea $05(a6,d7.w),a6</t>
+        </is>
+      </c>
+      <c r="E761" s="8" t="inlineStr">
+        <is>
+          <t>Points A6 at the first current/maximum statistic pair used by the three compact bars.</t>
+        </is>
+      </c>
+      <c r="F761" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B762" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C762" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D762" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$00040019,d5</t>
+        </is>
+      </c>
+      <c r="E762" s="8" t="inlineStr">
+        <is>
+          <t>Packs the first compact-stat bar Y=$19 and its five-pixel terminal height.</t>
+        </is>
+      </c>
+      <c r="F762" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B763" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C763" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D763" s="8" t="inlineStr">
+        <is>
+          <t>moveq #CompactStatsBar_LastIndex,d6</t>
+        </is>
+      </c>
+      <c r="E763" s="8" t="inlineStr">
+        <is>
+          <t>Uses DBRA terminal index two so exactly three compact statistic bars are drawn.</t>
+        </is>
+      </c>
+      <c r="F763" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B764" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C764" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D764" s="8" t="inlineStr">
+        <is>
+          <t>moveq #Player1_CompactStatsColourIndex,d3</t>
+        </is>
+      </c>
+      <c r="E764" s="8" t="inlineStr">
+        <is>
+          <t>Selects Player 1's hard-coded compact-stat palette index.</t>
+        </is>
+      </c>
+      <c r="F764" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B765" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="C765" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="D765" s="8" t="inlineStr">
+        <is>
+          <t>moveq #Player2_CompactStatsColourIndex,d3</t>
+        </is>
+      </c>
+      <c r="E765" s="8" t="inlineStr">
+        <is>
+          <t>Selects Player 2's hard-coded compact-stat palette index.</t>
+        </is>
+      </c>
+      <c r="F765" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B766" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsBarsLoop</t>
+        </is>
+      </c>
+      <c r="C766" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="D766" s="8" t="inlineStr">
+        <is>
+          <t>move.b (a6)+,d0</t>
+        </is>
+      </c>
+      <c r="E766" s="8" t="inlineStr">
+        <is>
+          <t>Loads the current statistic value and advances A6 to its maximum-value byte.</t>
+        </is>
+      </c>
+      <c r="F766" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B767" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsBarsLoop</t>
+        </is>
+      </c>
+      <c r="C767" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="D767" s="8" t="inlineStr">
+        <is>
+          <t>move.b (a6),d1</t>
+        </is>
+      </c>
+      <c r="E767" s="8" t="inlineStr">
+        <is>
+          <t>Loads the maximum statistic value used to scale the current bar length.</t>
+        </is>
+      </c>
+      <c r="F767" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B768" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsBarsLoop</t>
+        </is>
+      </c>
+      <c r="C768" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="D768" s="8" t="inlineStr">
+        <is>
+          <t>bsr Prepare_CompactStatBarLength</t>
+        </is>
+      </c>
+      <c r="E768" s="8" t="inlineStr">
+        <is>
+          <t>Prepares the compact-bar geometry and scales current D0 against maximum D1.</t>
+        </is>
+      </c>
+      <c r="F768" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B769" s="8" t="inlineStr">
+        <is>
+          <t>Draw_CompactStatsBarsLoop</t>
+        </is>
+      </c>
+      <c r="C769" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="D769" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_draw_bar</t>
+        </is>
+      </c>
+      <c r="E769" s="8" t="inlineStr">
+        <is>
+          <t>Calls the filled-rectangle drawing routine for one of the three compact statistic bars.</t>
+        </is>
+      </c>
+      <c r="F769" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B770" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="C770" s="8" t="inlineStr">
+        <is>
+          <t>Prepare_CompactStatBarLength</t>
+        </is>
+      </c>
+      <c r="D770" s="8" t="inlineStr">
+        <is>
+          <t>addq.w #$07,d5</t>
+        </is>
+      </c>
+      <c r="E770" s="8" t="inlineStr">
+        <is>
+          <t>Moves the next compact-stat bar down seven pixels, leaving its one-pixel inter-bar gap.</t>
+        </is>
+      </c>
+      <c r="F770" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B771" s="8" t="inlineStr">
+        <is>
+          <t>Advance_CompactStatsBarRow</t>
+        </is>
+      </c>
+      <c r="C771" s="8" t="inlineStr">
+        <is>
+          <t>Prepare_CompactStatBarLength</t>
+        </is>
+      </c>
+      <c r="D771" s="8" t="inlineStr">
+        <is>
+          <t>addq.w #$01,a6</t>
+        </is>
+      </c>
+      <c r="E771" s="8" t="inlineStr">
+        <is>
+          <t>Advances from the current/maximum pair just consumed to the next pair.</t>
+        </is>
+      </c>
+      <c r="F771" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B772" s="8" t="inlineStr">
+        <is>
+          <t>Prepare_CompactStatBarLength</t>
+        </is>
+      </c>
+      <c r="C772" s="8" t="inlineStr">
+        <is>
+          <t>Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="D772" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$00220037,d4</t>
+        </is>
+      </c>
+      <c r="E772" s="8" t="inlineStr">
+        <is>
+          <t>Sets compact-stat bar X=$37 and its maximum terminal width $22 before scaling.</t>
+        </is>
+      </c>
+      <c r="F772" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B773" s="8" t="inlineStr">
+        <is>
+          <t>Prepare_CompactStatBarLength</t>
+        </is>
+      </c>
+      <c r="C773" s="8" t="inlineStr">
+        <is>
+          <t>Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="D773" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$23,d2</t>
+        </is>
+      </c>
+      <c r="E773" s="8" t="inlineStr">
+        <is>
+          <t>Sets the compact-stat bar maximum drawable length to $23 pixels.</t>
+        </is>
+      </c>
+      <c r="F773" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B774" s="8" t="inlineStr">
+        <is>
+          <t>Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="C774" s="8" t="inlineStr">
+        <is>
+          <t>Return_ScaledBarLength</t>
+        </is>
+      </c>
+      <c r="D774" s="8" t="inlineStr">
+        <is>
+          <t>cmp.b d1,d0</t>
+        </is>
+      </c>
+      <c r="E774" s="8" t="inlineStr">
+        <is>
+          <t>Avoids division when the current value is already at or above its maximum; the bar remains full width.</t>
+        </is>
+      </c>
+      <c r="F774" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B775" s="8" t="inlineStr">
+        <is>
+          <t>Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="C775" s="8" t="inlineStr">
+        <is>
+          <t>Return_ScaledBarLength</t>
+        </is>
+      </c>
+      <c r="D775" s="8" t="inlineStr">
+        <is>
+          <t>mulu d2,d0</t>
+        </is>
+      </c>
+      <c r="E775" s="8" t="inlineStr">
+        <is>
+          <t>Multiplies the current value by the target pixel length before integer division by the maximum.</t>
+        </is>
+      </c>
+      <c r="F775" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B776" s="8" t="inlineStr">
+        <is>
+          <t>Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="C776" s="8" t="inlineStr">
+        <is>
+          <t>Return_ScaledBarLength</t>
+        </is>
+      </c>
+      <c r="D776" s="8" t="inlineStr">
+        <is>
+          <t>divu d1,d0</t>
+        </is>
+      </c>
+      <c r="E776" s="8" t="inlineStr">
+        <is>
+          <t>Divides the scaled current value by the maximum to obtain the bar length in pixels.</t>
+        </is>
+      </c>
+      <c r="F776" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B777" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="C777" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D777" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$0E,d3</t>
+        </is>
+      </c>
+      <c r="E777" s="8" t="inlineStr">
+        <is>
+          <t>Initialises the party-shield status-bar fallback colour before each living champion's class colour is selected.</t>
+        </is>
+      </c>
+      <c r="F777" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B778" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="C778" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D778" s="8" t="inlineStr">
+        <is>
+          <t>lea Character_Stats_DataTable+$05.l,a6</t>
+        </is>
+      </c>
+      <c r="E778" s="8" t="inlineStr">
+        <is>
+          <t>Uses offset $05 within each character record as the first current/maximum value pair for shield status bars.</t>
+        </is>
+      </c>
+      <c r="F778" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B779" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBars</t>
+        </is>
+      </c>
+      <c r="C779" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D779" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$03,d6</t>
+        </is>
+      </c>
+      <c r="E779" s="8" t="inlineStr">
+        <is>
+          <t>Uses DBRA terminal index three to visit all four party shield slots.</t>
+        </is>
+      </c>
+      <c r="F779" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B780" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBarsLoop</t>
+        </is>
+      </c>
+      <c r="C780" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D780" s="8" t="inlineStr">
+        <is>
+          <t>move.b $18(a5,d6.w),d0</t>
+        </is>
+      </c>
+      <c r="E780" s="8" t="inlineStr">
+        <is>
+          <t>Loads one party-slot state byte so vacant, dead, and occupied slots can be distinguished.</t>
+        </is>
+      </c>
+      <c r="F780" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B781" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBarsLoop</t>
+        </is>
+      </c>
+      <c r="C781" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D781" s="8" t="inlineStr">
+        <is>
+          <t>and.w #$00E0,d1</t>
+        </is>
+      </c>
+      <c r="E781" s="8" t="inlineStr">
+        <is>
+          <t>Tests the party-slot vacant/dead suppression bits before drawing a status bar.</t>
+        </is>
+      </c>
+      <c r="F781" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B782" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBarsLoop</t>
+        </is>
+      </c>
+      <c r="C782" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D782" s="8" t="inlineStr">
+        <is>
+          <t>asl.w #$05,d0</t>
+        </is>
+      </c>
+      <c r="E782" s="8" t="inlineStr">
+        <is>
+          <t>Converts the occupied slot's champion ID to its 32-byte character-stat record offset.</t>
+        </is>
+      </c>
+      <c r="F782" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B783" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBarsLoop</t>
+        </is>
+      </c>
+      <c r="C783" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D783" s="8" t="inlineStr">
+        <is>
+          <t>bsr Scale_ValueToBarLength</t>
+        </is>
+      </c>
+      <c r="E783" s="8" t="inlineStr">
+        <is>
+          <t>Calls the common scaler to convert the selected champion's current value into a shield-bar width.</t>
+        </is>
+      </c>
+      <c r="F783" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B784" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PartyShieldStatusBarsLoop</t>
+        </is>
+      </c>
+      <c r="C784" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="D784" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_draw_bar</t>
+        </is>
+      </c>
+      <c r="E784" s="8" t="inlineStr">
+        <is>
+          <t>Calls the filled-rectangle drawing routine for one occupied party-shield status bar.</t>
+        </is>
+      </c>
+      <c r="F784" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B785" s="8" t="inlineStr">
+        <is>
+          <t>Advance_PartyShieldStatusBarRow</t>
+        </is>
+      </c>
+      <c r="C785" s="8" t="inlineStr">
+        <is>
+          <t>Return_FromMainPlayerInterface</t>
+        </is>
+      </c>
+      <c r="D785" s="8" t="inlineStr">
+        <is>
+          <t>sub.w #$0009,d5</t>
+        </is>
+      </c>
+      <c r="E785" s="8" t="inlineStr">
+        <is>
+          <t>Moves to the next party-shield status-bar Y position, nine pixels above the current bar.</t>
+        </is>
+      </c>
+      <c r="F785" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B786" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C786" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D786" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$002F0000,d4</t>
+        </is>
+      </c>
+      <c r="E786" s="8" t="inlineStr">
+        <is>
+          <t>Sets the large avatar panel outer bevel to X=$00 with horizontal terminal count $2F, producing a 48-pixel width.</t>
+        </is>
+      </c>
+      <c r="F786" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B787" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C787" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D787" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$0A,d5</t>
+        </is>
+      </c>
+      <c r="E787" s="8" t="inlineStr">
+        <is>
+          <t>Sets the large avatar panel outer bevel to player-local Y=$0A.</t>
+        </is>
+      </c>
+      <c r="F787" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B788" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C788" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D788" s="8" t="inlineStr">
+        <is>
+          <t>bsr Draw_BevelledPanelFrame</t>
+        </is>
+      </c>
+      <c r="E788" s="8" t="inlineStr">
+        <is>
+          <t>Calls the shared bevelled-panel renderer for the large avatar background and three inset grey outlines.</t>
+        </is>
+      </c>
+      <c r="F788" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B789" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C789" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D789" s="8" t="inlineStr">
+        <is>
+          <t>move.w $0006(a5),d7</t>
+        </is>
+      </c>
+      <c r="E789" s="8" t="inlineStr">
+        <is>
+          <t>Loads the current leader champion ID for the large-avatar graphic selection.</t>
+        </is>
+      </c>
+      <c r="F789" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B790" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C790" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D790" s="8" t="inlineStr">
+        <is>
+          <t>moveq #-$01,d4</t>
+        </is>
+      </c>
+      <c r="E790" s="8" t="inlineStr">
+        <is>
+          <t>Passes the large-avatar rendering sentinel to the avatar compositor.</t>
+        </is>
+      </c>
+      <c r="F790" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B791" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C791" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D791" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$000002A9,a0</t>
+        </is>
+      </c>
+      <c r="E791" s="8" t="inlineStr">
+        <is>
+          <t>Selects the framebuffer offset for the 32×30 large champion avatar.</t>
+        </is>
+      </c>
+      <c r="F791" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B792" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarPanel</t>
+        </is>
+      </c>
+      <c r="C792" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="D792" s="8" t="inlineStr">
+        <is>
+          <t>bsr Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="E792" s="8" t="inlineStr">
+        <is>
+          <t>Calls the large-avatar compositor, which selects the leader portrait and applies its palette ink.</t>
+        </is>
+      </c>
+      <c r="F792" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B793" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="C793" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D793" s="8" t="inlineStr">
+        <is>
+          <t>btst #$00,$003E(a5)</t>
+        </is>
+      </c>
+      <c r="E793" s="8" t="inlineStr">
+        <is>
+          <t>Suppresses the large-avatar inner frame while the main champion presentation bit is active.</t>
+        </is>
+      </c>
+      <c r="F793" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B794" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="C794" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D794" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$0021000F,d5</t>
+        </is>
+      </c>
+      <c r="E794" s="8" t="inlineStr">
+        <is>
+          <t>Packs the inner avatar-frame height and player-local Y=$0F.</t>
+        </is>
+      </c>
+      <c r="F794" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B795" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="C795" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D795" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$00230006,d4</t>
+        </is>
+      </c>
+      <c r="E795" s="8" t="inlineStr">
+        <is>
+          <t>Packs the inner avatar-frame horizontal terminal count $23 and player-local X=$06.</t>
+        </is>
+      </c>
+      <c r="F795" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B796" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="C796" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D796" s="8" t="inlineStr">
+        <is>
+          <t>bsr Select_ChampionShieldInkColour</t>
+        </is>
+      </c>
+      <c r="E796" s="8" t="inlineStr">
+        <is>
+          <t>Obtains the leader class colour used for the optional large-avatar inner-frame ink.</t>
+        </is>
+      </c>
+      <c r="F796" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B797" s="8" t="inlineStr">
+        <is>
+          <t>Draw_MainChampionAvatarInnerFrame</t>
+        </is>
+      </c>
+      <c r="C797" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD12</t>
+        </is>
+      </c>
+      <c r="D797" s="8" t="inlineStr">
+        <is>
+          <t>bra BW_draw_frame</t>
+        </is>
+      </c>
+      <c r="E797" s="8" t="inlineStr">
+        <is>
+          <t>Tail-calls the procedural frame renderer for the large avatar inner border.</t>
+        </is>
+      </c>
+      <c r="F797" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B798" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="C798" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD4A</t>
+        </is>
+      </c>
+      <c r="D798" s="8" t="inlineStr">
+        <is>
+          <t>add.l screen_ptr.l,a0</t>
+        </is>
+      </c>
+      <c r="E798" s="8" t="inlineStr">
+        <is>
+          <t>Converts the avatar-local framebuffer offset to an address in the active player screen buffer.</t>
+        </is>
+      </c>
+      <c r="F798" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B799" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="C799" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD4A</t>
+        </is>
+      </c>
+      <c r="D799" s="8" t="inlineStr">
+        <is>
+          <t>lea GFX_Avatars.l,a1</t>
+        </is>
+      </c>
+      <c r="E799" s="8" t="inlineStr">
+        <is>
+          <t>Selects the packed champion portrait graphics source.</t>
+        </is>
+      </c>
+      <c r="F799" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B800" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="C800" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD4A</t>
+        </is>
+      </c>
+      <c r="D800" s="8" t="inlineStr">
+        <is>
+          <t>asl.w #$05,d0</t>
+        </is>
+      </c>
+      <c r="E800" s="8" t="inlineStr">
+        <is>
+          <t>Begins converting the champion ID to its portrait-record source offset.</t>
+        </is>
+      </c>
+      <c r="F800" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B801" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="C801" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD4A</t>
+        </is>
+      </c>
+      <c r="D801" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$0001001D,-(sp)</t>
+        </is>
+      </c>
+      <c r="E801" s="8" t="inlineStr">
+        <is>
+          <t>Supplies the large portrait renderer with a two-word-wide, 30-row graphic size.</t>
+        </is>
+      </c>
+      <c r="F801" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B802" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionLargeAvatar</t>
+        </is>
+      </c>
+      <c r="C802" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CD4A</t>
+        </is>
+      </c>
+      <c r="D802" s="8" t="inlineStr">
+        <is>
+          <t>bra Draw_PlanarGraphicCore</t>
+        </is>
+      </c>
+      <c r="E802" s="8" t="inlineStr">
+        <is>
+          <t>Enters the common four-plane renderer with the resolved avatar source and destination.</t>
+        </is>
+      </c>
+      <c r="F802" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B803" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionStats</t>
+        </is>
+      </c>
+      <c r="C803" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="D803" s="8" t="inlineStr">
+        <is>
+          <t>move.w $0006(a5),-(sp)</t>
+        </is>
+      </c>
+      <c r="E803" s="8" t="inlineStr">
+        <is>
+          <t>Saves the current leader champion ID while the generic scroll frame is drawn.</t>
+        </is>
+      </c>
+      <c r="F803" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B804" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionStats</t>
+        </is>
+      </c>
+      <c r="C804" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="D804" s="8" t="inlineStr">
+        <is>
+          <t>bsr Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="E804" s="8" t="inlineStr">
+        <is>
+          <t>Calls the shared scroll-frame drawing routine before printing champion statistics.</t>
+        </is>
+      </c>
+      <c r="F804" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B805" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionStats</t>
+        </is>
+      </c>
+      <c r="C805" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="D805" s="8" t="inlineStr">
+        <is>
+          <t>lea ChampionStatsScroll_TextTemplate.l,a6</t>
+        </is>
+      </c>
+      <c r="E805" s="8" t="inlineStr">
+        <is>
+          <t>Selects the writable packed-text template for the champion statistics scroll.</t>
+        </is>
+      </c>
+      <c r="F805" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B806" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionStats</t>
+        </is>
+      </c>
+      <c r="C806" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="D806" s="8" t="inlineStr">
+        <is>
+          <t>asl.w #$05,d0</t>
+        </is>
+      </c>
+      <c r="E806" s="8" t="inlineStr">
+        <is>
+          <t>Converts the champion ID to its 32-byte Character_Stats_DataTable record offset.</t>
+        </is>
+      </c>
+      <c r="F806" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B807" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="C807" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CB7E</t>
+        </is>
+      </c>
+      <c r="D807" s="8" t="inlineStr">
+        <is>
+          <t>move.b $00(a2,d7.w),d0</t>
+        </is>
+      </c>
+      <c r="E807" s="8" t="inlineStr">
+        <is>
+          <t>Loads one source-field offset from the seven-entry champion-statistics scroll lookup table.</t>
+        </is>
+      </c>
+      <c r="F807" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B808" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="C808" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CB7E</t>
+        </is>
+      </c>
+      <c r="D808" s="8" t="inlineStr">
+        <is>
+          <t>move.b $00(a0,d0.w),d0</t>
+        </is>
+      </c>
+      <c r="E808" s="8" t="inlineStr">
+        <is>
+          <t>Reads the selected champion statistic identified by the lookup entry.</t>
+        </is>
+      </c>
+      <c r="F808" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B809" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="C809" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CB7E</t>
+        </is>
+      </c>
+      <c r="D809" s="8" t="inlineStr">
+        <is>
+          <t>bsr Convert_ByteToDecimalText</t>
+        </is>
+      </c>
+      <c r="E809" s="8" t="inlineStr">
+        <is>
+          <t>Converts the binary champion statistic to its printable decimal digits.</t>
+        </is>
+      </c>
+      <c r="F809" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B810" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="C810" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00CB7E</t>
+        </is>
+      </c>
+      <c r="D810" s="8" t="inlineStr">
+        <is>
+          <t>dbra d7,ChampionStats_InsertFieldsLoop</t>
+        </is>
+      </c>
+      <c r="E810" s="8" t="inlineStr">
+        <is>
+          <t>Repeats for all seven lookup-defined champion-statistic fields.</t>
+        </is>
+      </c>
+      <c r="F810" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B811" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ChampionStats</t>
+        </is>
+      </c>
+      <c r="C811" s="8" t="inlineStr">
+        <is>
+          <t>ChampionStatsScroll_FieldAndTextOffsets</t>
+        </is>
+      </c>
+      <c r="D811" s="8" t="inlineStr">
+        <is>
+          <t>bra Print_fflim_text</t>
+        </is>
+      </c>
+      <c r="E811" s="8" t="inlineStr">
+        <is>
+          <t>Prints the completed champion-statistics scroll text template after all values have been inserted.</t>
+        </is>
+      </c>
+      <c r="F811" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B812" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C812" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D812" s="8" t="inlineStr">
+        <is>
+          <t>move.w #$0018,d5</t>
+        </is>
+      </c>
+      <c r="E812" s="8" t="inlineStr">
+        <is>
+          <t>Sets the scroll-frame background rectangle to player-local Y=$18 while preserving the caller-provided scroll Y in the other word of D5.</t>
+        </is>
+      </c>
+      <c r="F812" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B813" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C813" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D813" s="8" t="inlineStr">
+        <is>
+          <t>move.l #$003F00F0,d4</t>
+        </is>
+      </c>
+      <c r="E813" s="8" t="inlineStr">
+        <is>
+          <t>Packs the scroll-frame background X=$F0 and horizontal terminal count $3F, producing a 64-pixel-wide fill.</t>
+        </is>
+      </c>
+      <c r="F813" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B814" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C814" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D814" s="8" t="inlineStr">
+        <is>
+          <t>bsr BW_draw_bar</t>
+        </is>
+      </c>
+      <c r="E814" s="8" t="inlineStr">
+        <is>
+          <t>Calls the filled-rectangle drawing routine for the scroll-frame background.</t>
+        </is>
+      </c>
+      <c r="F814" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B815" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C815" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D815" s="8" t="inlineStr">
+        <is>
+          <t>lea GFX_Scroll_Edge_Left.l,a1</t>
+        </is>
+      </c>
+      <c r="E815" s="8" t="inlineStr">
+        <is>
+          <t>Selects the pre-drawn left scroll edge graphic.</t>
+        </is>
+      </c>
+      <c r="F815" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B816" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C816" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D816" s="8" t="inlineStr">
+        <is>
+          <t>add.w #$03DC,a0</t>
+        </is>
+      </c>
+      <c r="E816" s="8" t="inlineStr">
+        <is>
+          <t>Positions the left scroll edge at its player-local framebuffer offset.</t>
+        </is>
+      </c>
+      <c r="F816" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B817" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C817" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D817" s="8" t="inlineStr">
+        <is>
+          <t>lea GFX_Scroll_Edge_Right.l,a1</t>
+        </is>
+      </c>
+      <c r="E817" s="8" t="inlineStr">
+        <is>
+          <t>Selects the pre-drawn right scroll edge graphic.</t>
+        </is>
+      </c>
+      <c r="F817" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B818" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C818" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D818" s="8" t="inlineStr">
+        <is>
+          <t>add.w #$03E6,a0</t>
+        </is>
+      </c>
+      <c r="E818" s="8" t="inlineStr">
+        <is>
+          <t>Positions the right scroll edge at its player-local framebuffer offset.</t>
+        </is>
+      </c>
+      <c r="F818" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B819" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C819" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D819" s="8" t="inlineStr">
+        <is>
+          <t>lea GFX_Scroll_Edge_Bottom.l,a1</t>
+        </is>
+      </c>
+      <c r="E819" s="8" t="inlineStr">
+        <is>
+          <t>Selects the pre-drawn bottom scroll cap graphic.</t>
+        </is>
+      </c>
+      <c r="F819" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B820" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C820" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D820" s="8" t="inlineStr">
+        <is>
+          <t>lea GFX_Scroll_Edge_Top.l,a1</t>
+        </is>
+      </c>
+      <c r="E820" s="8" t="inlineStr">
+        <is>
+          <t>Selects the pre-drawn top scroll cap graphic.</t>
+        </is>
+      </c>
+      <c r="F820" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B821" s="8" t="inlineStr">
+        <is>
+          <t>Draw_ScrollFrame</t>
+        </is>
+      </c>
+      <c r="C821" s="8" t="inlineStr">
+        <is>
+          <t>Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="D821" s="8" t="inlineStr">
+        <is>
+          <t>bsr Draw_PlanarGraphic</t>
+        </is>
+      </c>
+      <c r="E821" s="8" t="inlineStr">
+        <is>
+          <t>Calls the common four-plane graphic renderer for one scroll-frame edge or cap.</t>
+        </is>
+      </c>
+      <c r="F821" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B822" s="8" t="inlineStr">
+        <is>
+          <t>Draw_SpellBookRunePage</t>
+        </is>
+      </c>
+      <c r="C822" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C8D6</t>
+        </is>
+      </c>
+      <c r="D822" s="8" t="inlineStr">
+        <is>
+          <t>add.w #$0164,a0</t>
+        </is>
+      </c>
+      <c r="E822" s="8" t="inlineStr">
+        <is>
+          <t>Moves from one left-page rune entry to the next: eight screen rows down and back to the left text column.</t>
+        </is>
+      </c>
+      <c r="F822" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B823" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C8D6</t>
+        </is>
+      </c>
+      <c r="C823" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C906</t>
+        </is>
+      </c>
+      <c r="D823" s="8" t="inlineStr">
+        <is>
+          <t>add.w #$0114,a0</t>
+        </is>
+      </c>
+      <c r="E823" s="8" t="inlineStr">
+        <is>
+          <t>Moves from one right-page rune entry to the next after the separately placed first rune glyph.</t>
+        </is>
+      </c>
+      <c r="F823" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B824" s="8" t="inlineStr">
+        <is>
+          <t>adrCd006698</t>
+        </is>
+      </c>
+      <c r="C824" s="8" t="inlineStr">
+        <is>
+          <t>adrCd0066BE</t>
+        </is>
+      </c>
+      <c r="D824" s="8" t="inlineStr">
+        <is>
+          <t>sub.w #$02DC,a0</t>
+        </is>
+      </c>
+      <c r="E824" s="8" t="inlineStr">
+        <is>
+          <t>Rebases the completed SP.PTS text cursor from $0E38 to $0B5C, the first lower spell-book decoration slot.</t>
+        </is>
+      </c>
+      <c r="F824" s="8" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
various spellbook UI viewer updates
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -26208,7 +26208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F824"/>
+  <dimension ref="A1:F841"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -52095,6 +52095,516 @@
         </is>
       </c>
       <c r="F824" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B825" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C3A6</t>
+        </is>
+      </c>
+      <c r="C825" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C3DE</t>
+        </is>
+      </c>
+      <c r="D825" s="8" t="inlineStr">
+        <is>
+          <t>move.b d6,(a6)+</t>
+        </is>
+      </c>
+      <c r="E825" s="8" t="inlineStr">
+        <is>
+          <t>Builds the four-entry colour mask used when the spell-book overlay is drawn.</t>
+        </is>
+      </c>
+      <c r="F825" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B826" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C3DE</t>
+        </is>
+      </c>
+      <c r="C826" s="8" t="inlineStr">
+        <is>
+          <t>Click_SwitchView</t>
+        </is>
+      </c>
+      <c r="D826" s="8" t="inlineStr">
+        <is>
+          <t>asl.w #$03,d0</t>
+        </is>
+      </c>
+      <c r="E826" s="8" t="inlineStr">
+        <is>
+          <t>After screen-address doubling, converts the frame index to its 16-byte GFX_Pockets+$4130 source offset (32 pixels per frame).</t>
+        </is>
+      </c>
+      <c r="F826" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B827" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C322</t>
+        </is>
+      </c>
+      <c r="C827" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C3A6</t>
+        </is>
+      </c>
+      <c r="D827" s="8" t="inlineStr">
+        <is>
+          <t>cmpi.w #$0003,d1</t>
+        </is>
+      </c>
+      <c r="E827" s="8" t="inlineStr">
+        <is>
+          <t>At the final page-turn phase, redraws the adjacent page before the rightmost rune-column overlay is added.</t>
+        </is>
+      </c>
+      <c r="F827" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B828" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C322</t>
+        </is>
+      </c>
+      <c r="C828" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C3A6</t>
+        </is>
+      </c>
+      <c r="D828" s="8" t="inlineStr">
+        <is>
+          <t>lea SpellBookRunes+$03.l,a6</t>
+        </is>
+      </c>
+      <c r="E828" s="8" t="inlineStr">
+        <is>
+          <t>Selects the offset-three rune stream for four rightmost-column glyph stamps during the final page-turn phase.</t>
+        </is>
+      </c>
+      <c r="F828" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B829" s="8" t="inlineStr">
+        <is>
+          <t>adrCd006900</t>
+        </is>
+      </c>
+      <c r="C829" s="8" t="inlineStr">
+        <is>
+          <t>adrJA006914</t>
+        </is>
+      </c>
+      <c r="D829" s="8" t="inlineStr">
+        <is>
+          <t>not.w d0</t>
+        </is>
+      </c>
+      <c r="E829" s="8" t="inlineStr">
+        <is>
+          <t>Folds spell indices $10-$1F before deriving their mirrored magic-class order.</t>
+        </is>
+      </c>
+      <c r="F829" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B830" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C906</t>
+        </is>
+      </c>
+      <c r="C830" s="8" t="inlineStr">
+        <is>
+          <t>adrJA00C938</t>
+        </is>
+      </c>
+      <c r="D830" s="8" t="inlineStr">
+        <is>
+          <t>move.b adrB_00C934(pc,d0.w),d6</t>
+        </is>
+      </c>
+      <c r="E830" s="8" t="inlineStr">
+        <is>
+          <t>Maps Serpent, Chaos, Dragon and Moon class indices to palette inks $06, $0D, $0C and $07 for available runes.</t>
+        </is>
+      </c>
+      <c r="F830" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B831" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C906</t>
+        </is>
+      </c>
+      <c r="C831" s="8" t="inlineStr">
+        <is>
+          <t>adrJA00C938</t>
+        </is>
+      </c>
+      <c r="D831" s="8" t="inlineStr">
+        <is>
+          <t>btst d7,$000C(a3)</t>
+        </is>
+      </c>
+      <c r="E831" s="8" t="inlineStr">
+        <is>
+          <t>Tests this page entry's ownership bit in the champion's four spell-book bytes at $0C-$0F; clear entries use grey ink.</t>
+        </is>
+      </c>
+      <c r="F831" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B832" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00C2AC</t>
+        </is>
+      </c>
+      <c r="C832" s="8" t="inlineStr">
+        <is>
+          <t>Click_TurnSpellBookPage</t>
+        </is>
+      </c>
+      <c r="D832" s="8" t="inlineStr">
+        <is>
+          <t>btst d0,$0C(a4,d3.w)</t>
+        </is>
+      </c>
+      <c r="E832" s="8" t="inlineStr">
+        <is>
+          <t>Tests the clicked rune entry against its page nibble; a clear bit deselects the currently loaded spell instead of selecting that rune.</t>
+        </is>
+      </c>
+      <c r="F832" s="8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>adrCd0068F8</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>move.b (a4),d0</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr">
+        <is>
+          <t>Loads the champion's selected spell index from byte  before calculating its displayed spell-point cost.</t>
+        </is>
+      </c>
+      <c r="F833" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>adrCd0068F8</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>addq.w #,d0</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr">
+        <is>
+          <t>The displayed base cost is twice the stored SpellCost_DataTable value plus one.</t>
+        </is>
+      </c>
+      <c r="F834" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>adrCd0068F8</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>add.w d0,d0</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr">
+        <is>
+          <t>Doubles the adjusted base spell cost before the cast-power adjustment is added.</t>
+        </is>
+      </c>
+      <c r="F835" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>adrCd0068F8</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>add.w d1,d0</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>Adds the source cast-power curve adjustment to form the COST +nn+ value.</t>
+        </is>
+      </c>
+      <c r="F836" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>adrCd006698</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>adrCd006712</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>bsr adrCd00CFBC</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr">
+        <is>
+          <t>Prints the selected spell name from its fixed eight-character SpellNames record using the spell-book name origin.</t>
+        </is>
+      </c>
+      <c r="F837" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>adrCd006698</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>adrCd006712</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>lea adrEA00EA36.l,a6</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr">
+        <is>
+          <t>Selects the COST text stream: FC positions it at column 30, row 10; FE switches colour around glyphs / and the two cost digits.</t>
+        </is>
+      </c>
+      <c r="F838" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>adrCd00CFBC</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>adrLp00CFDA</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>add.w #/bin/zshBAE,a0</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>Sets the selected-spell-name drawing origin in the right-hand spell-book panel.</t>
+        </is>
+      </c>
+      <c r="F839" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Exec_char_extensions</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Exec_char_extensions</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>asl.w #,d4</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr">
+        <is>
+          <t>FC text extension converts its byte column to native 8-pixel X coordinates before calculating the text origin.</t>
+        </is>
+      </c>
+      <c r="F840" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>adrCd00C650</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>adrCd00C708</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>cmpi.w #,d1</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr">
+        <is>
+          <t>C69C limits the spell-book top controls to Y -/bin/zshF; its X tests preserve 8-pixel gaps between page, close and page-forward targets.</t>
+        </is>
+      </c>
+      <c r="F841" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
multiple fixes to the data viewer and added savegame overlay in all areas.
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L509"/>
+  <dimension ref="A1:L515"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -26135,6 +26135,378 @@
       <c r="L509" s="8" t="inlineStr">
         <is>
           <t>The page word is masked to $0007 immediately afterwards, selecting one of four two-page spreads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B510" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_PracticeFirstThreshold</t>
+        </is>
+      </c>
+      <c r="C510" s="8" t="inlineStr">
+        <is>
+          <t>$05</t>
+        </is>
+      </c>
+      <c r="D510" s="8" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="E510" s="8" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="F510" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$05,d2</t>
+        </is>
+      </c>
+      <c r="G510" s="8" t="inlineStr">
+        <is>
+          <t>7405</t>
+        </is>
+      </c>
+      <c r="H510" s="8" t="inlineStr">
+        <is>
+          <t>moveq #SpellCasting_PracticeFirstThreshold,d2</t>
+        </is>
+      </c>
+      <c r="I510" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J510" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K510" s="8" t="inlineStr">
+        <is>
+          <t>First spell-practice threshold for matching spells.</t>
+        </is>
+      </c>
+      <c r="L510" s="8" t="inlineStr">
+        <is>
+          <t>The non-matching branch doubles D2 to $0A before its first comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B511" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_MatchingWandBonus</t>
+        </is>
+      </c>
+      <c r="C511" s="8" t="inlineStr">
+        <is>
+          <t>$03</t>
+        </is>
+      </c>
+      <c r="D511" s="8" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="E511" s="8" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="F511" s="8" t="inlineStr">
+        <is>
+          <t>addq.b #$03,d7</t>
+        </is>
+      </c>
+      <c r="G511" s="8" t="inlineStr">
+        <is>
+          <t>5607</t>
+        </is>
+      </c>
+      <c r="H511" s="8" t="inlineStr">
+        <is>
+          <t>addq.b #SpellCasting_MatchingWandBonus,d7</t>
+        </is>
+      </c>
+      <c r="I511" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J511" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K511" s="8" t="inlineStr">
+        <is>
+          <t>Cast-quality bonus for a held wand matching a non-matching spell.</t>
+        </is>
+      </c>
+      <c r="L511" s="8" t="inlineStr">
+        <is>
+          <t>Applied only when the champion class does not match the selected spell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B512" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_CooldownBaseIncrement</t>
+        </is>
+      </c>
+      <c r="C512" s="8" t="inlineStr">
+        <is>
+          <t>$05</t>
+        </is>
+      </c>
+      <c r="D512" s="8" t="inlineStr">
+        <is>
+          <t>CastSpell_CalculateQualityAndCooldown</t>
+        </is>
+      </c>
+      <c r="E512" s="8" t="inlineStr">
+        <is>
+          <t>CastSpell_RecordPractice</t>
+        </is>
+      </c>
+      <c r="F512" s="8" t="inlineStr">
+        <is>
+          <t>addq.b #$05,d1</t>
+        </is>
+      </c>
+      <c r="G512" s="8" t="inlineStr">
+        <is>
+          <t>5A01</t>
+        </is>
+      </c>
+      <c r="H512" s="8" t="inlineStr">
+        <is>
+          <t>addq.b #SpellCasting_CooldownBaseIncrement,d1</t>
+        </is>
+      </c>
+      <c r="I512" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J512" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K512" s="8" t="inlineStr">
+        <is>
+          <t>Base spell-cooldown increment added to the selected spell cost value after quality is calculated.</t>
+        </is>
+      </c>
+      <c r="L512" s="8" t="inlineStr">
+        <is>
+          <t>The accumulated byte $15 is clamped to SpellCasting_CooldownMaximum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B513" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_ManaCostMinimum</t>
+        </is>
+      </c>
+      <c r="C513" s="8" t="inlineStr">
+        <is>
+          <t>$01</t>
+        </is>
+      </c>
+      <c r="D513" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="E513" s="8" t="inlineStr">
+        <is>
+          <t>Character_GetClassIndex</t>
+        </is>
+      </c>
+      <c r="F513" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$01,d0</t>
+        </is>
+      </c>
+      <c r="G513" s="8" t="inlineStr">
+        <is>
+          <t>7001</t>
+        </is>
+      </c>
+      <c r="H513" s="8" t="inlineStr">
+        <is>
+          <t>moveq #SpellCasting_ManaCostMinimum,d0</t>
+        </is>
+      </c>
+      <c r="I513" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J513" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K513" s="8" t="inlineStr">
+        <is>
+          <t>Minimum calculated spell-point cost.</t>
+        </is>
+      </c>
+      <c r="L513" s="8" t="inlineStr">
+        <is>
+          <t>C688C restores byte $14 by one when the calculated cost would otherwise be zero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B514" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_ManaCostMaximum</t>
+        </is>
+      </c>
+      <c r="C514" s="8" t="inlineStr">
+        <is>
+          <t>$64</t>
+        </is>
+      </c>
+      <c r="D514" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="E514" s="8" t="inlineStr">
+        <is>
+          <t>Character_GetClassIndex</t>
+        </is>
+      </c>
+      <c r="F514" s="8" t="inlineStr">
+        <is>
+          <t>cmpi.w #$0064,d0</t>
+        </is>
+      </c>
+      <c r="G514" s="8" t="inlineStr">
+        <is>
+          <t>0C400064</t>
+        </is>
+      </c>
+      <c r="H514" s="8" t="inlineStr">
+        <is>
+          <t>cmpi.w #SpellCasting_ManaCostMaximum,d0</t>
+        </is>
+      </c>
+      <c r="I514" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J514" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K514" s="8" t="inlineStr">
+        <is>
+          <t>Exclusive spell-point cost ceiling used while normalising byte $14.</t>
+        </is>
+      </c>
+      <c r="L514" s="8" t="inlineStr">
+        <is>
+          <t>Costs are reduced until they are below 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="8" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B515" s="8" t="inlineStr">
+        <is>
+          <t>SpellCasting_CastBarMaximumWidth</t>
+        </is>
+      </c>
+      <c r="C515" s="8" t="inlineStr">
+        <is>
+          <t>$34</t>
+        </is>
+      </c>
+      <c r="D515" s="8" t="inlineStr">
+        <is>
+          <t>adrCd006720</t>
+        </is>
+      </c>
+      <c r="E515" s="8" t="inlineStr">
+        <is>
+          <t>adrCd00675E</t>
+        </is>
+      </c>
+      <c r="F515" s="8" t="inlineStr">
+        <is>
+          <t>moveq #$34,d2</t>
+        </is>
+      </c>
+      <c r="G515" s="8" t="inlineStr">
+        <is>
+          <t>7434</t>
+        </is>
+      </c>
+      <c r="H515" s="8" t="inlineStr">
+        <is>
+          <t>moveq #SpellCasting_CastBarMaximumWidth,d2</t>
+        </is>
+      </c>
+      <c r="I515" s="8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J515" s="8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="K515" s="8" t="inlineStr">
+        <is>
+          <t>Maximum CAST bar width in pixels.</t>
+        </is>
+      </c>
+      <c r="L515" s="8" t="inlineStr">
+        <is>
+          <t>C8144 scales this 52-pixel width by the percentage selected from the 20-byte cast-bar lookup.</t>
         </is>
       </c>
     </row>
@@ -26208,7 +26580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F841"/>
+  <dimension ref="A1:F858"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -52356,12 +52728,12 @@
       </c>
       <c r="D833" t="inlineStr">
         <is>
-          <t>move.b (a4),d0</t>
+          <t>move.b $0015(a4),d0</t>
         </is>
       </c>
       <c r="E833" t="inlineStr">
         <is>
-          <t>Loads the champion's selected spell index from byte  before calculating its displayed spell-point cost.</t>
+          <t>Loads champion byte $15, the spell cooldown penalty; matching champion and spell classes halve it.</t>
         </is>
       </c>
       <c r="F833" t="n">
@@ -52511,7 +52883,7 @@
       </c>
       <c r="E838" t="inlineStr">
         <is>
-          <t>Selects the COST text stream: FC positions it at column 30, row 10; FE switches colour around glyphs / and the two cost digits.</t>
+          <t>Selects the COST text stream. Its FC ($1E,$0A) position plus the text renderer base $0050 places visible glyphs at X=$F0, Y=$52.</t>
         </is>
       </c>
       <c r="F838" t="n">
@@ -52536,12 +52908,12 @@
       </c>
       <c r="D839" t="inlineStr">
         <is>
-          <t>add.w #/bin/zshBAE,a0</t>
+          <t>add.w #$0BAE,a0</t>
         </is>
       </c>
       <c r="E839" t="inlineStr">
         <is>
-          <t>Sets the selected-spell-name drawing origin in the right-hand spell-book panel.</t>
+          <t>Sets the selected-spell name raster origin to X=$F0, Y=$4A: $0BAE is 74 rows of $28 bytes plus 30 bytes.</t>
         </is>
       </c>
       <c r="F839" t="n">
@@ -52606,6 +52978,538 @@
       </c>
       <c r="F841" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>adrCd0068F8</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>cmpi.w #,d0</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr">
+        <is>
+          <t>Rejects a cast-power setting when the calculated spell-point cost reaches ; displayed costs are therefore limited to /bin/zsh-.</t>
+        </is>
+      </c>
+      <c r="F842" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>adrCd006698</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>adrCd006712</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>moveq #,d6</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>The selected spell name printer emits exactly eight characters from SpellNames at the spell-book name origin.</t>
+        </is>
+      </c>
+      <c r="F843" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>adrCd006720</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>adrCd00675E</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>moveq #SpellCasting_CastBarMaximumWidth,d2</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr">
+        <is>
+          <t>Supplies C8144 with the 52-pixel maximum CAST bar width before percentage scaling.</t>
+        </is>
+      </c>
+      <c r="F844" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>adrCd006778</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>move.b $0015(a4),d0</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr">
+        <is>
+          <t>Loads champion byte $15, the spell cooldown penalty; matching champion and spell classes halve it.</t>
+        </is>
+      </c>
+      <c r="F845" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>adrCd006778</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>sub.b SpellCasting_SpellDifficultyPenalties(pc,d6.w),d7</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>Subtracts the source difficulty-penalty byte for the selected spell before C6720 maps the negated score to the CAST bar.</t>
+        </is>
+      </c>
+      <c r="F846" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>adrCd006720</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>adrCd00675E</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>move.b adrB_006760(pc,d7.w),d0</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr">
+        <is>
+          <t>Converts the clamped negated cast score to one of 20 percentage values used to scale the 52-pixel CAST bar.</t>
+        </is>
+      </c>
+      <c r="F847" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>move.b $00(a1,d6.w),d0</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr">
+        <is>
+          <t>Loads the selected spell's per-champion success-practice count from the runtime 16 by 32 practice area.</t>
+        </is>
+      </c>
+      <c r="F848" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>moveq #SpellCasting_PracticeFirstThreshold,d2</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr">
+        <is>
+          <t>Starts the matching spell-practice curve at five successes; the non-matching path doubles this to ten.</t>
+        </is>
+      </c>
+      <c r="F849" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>addq.b #SpellCasting_MatchingWandBonus,d7</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr">
+        <is>
+          <t>Awards the matching-wand quality bonus when the champion class itself does not match.</t>
+        </is>
+      </c>
+      <c r="F850" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>add.w d2,d2</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr">
+        <is>
+          <t>Doubles the practice threshold after each band and increments the companion right-shift count.</t>
+        </is>
+      </c>
+      <c r="F851" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>CastSpell_CalculateQualityAndCooldown</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>CastSpell_RecordPractice</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>addq.b #SpellCasting_CooldownBaseIncrement,d1</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr">
+        <is>
+          <t>Adds the fixed cooldown increment after loading the selected spell cost value.</t>
+        </is>
+      </c>
+      <c r="F852" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>CastSpell_RecordPractice</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>CastSpell_Complete</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>addq.b #$01,$00(a0,d0.w)</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr">
+        <is>
+          <t>Increments this champion and spell's practice byte after a successful handler dispatch.</t>
+        </is>
+      </c>
+      <c r="F853" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>CastSpell_RecordPractice</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>CastSpell_Complete</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>subq.b #$01,$00(a0,d0.w)</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr">
+        <is>
+          <t>Restores the practice byte after overflow, saturating the counter at $FF.</t>
+        </is>
+      </c>
+      <c r="F854" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Calculate_SpellCastingQuality</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>adrCd006836</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>lsr.b d1,d0</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr">
+        <is>
+          <t>Halves cooldown only when the repeated champion/spell class comparison set D1 to one.</t>
+        </is>
+      </c>
+      <c r="F855" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Character_GetClassIndex</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>bmi.s adrCd0068DC</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr">
+        <is>
+          <t>Uses negative byte $14 values directly as low-cost penalties instead of indexing the non-negative extra-mana curve.</t>
+        </is>
+      </c>
+      <c r="F856" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>adrCd00688C</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Character_GetClassIndex</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>addq.b #$01,$0014(a4)</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>Reverses the final decrement when cost normalisation reaches zero, preserving the one-point minimum.</t>
+        </is>
+      </c>
+      <c r="F857" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>BLOODWYCH439</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>adrCd006720</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>adrCd00675E</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>move.b adrB_006760(pc,d7.w),d0</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr">
+        <is>
+          <t>Selects one of 20 CAST percentages using the clamped negated signed quality score.</t>
+        </is>
+      </c>
+      <c r="F858" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added some asm source recovery which was accidently dc.w
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Re9b5889e8936415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R58aabe07f84a4be6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R99d14713a14c492f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Rf741535eb9cd45f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rb3c795a76b504f24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="Re31782dcd32948f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R65497b0e63264d30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:sz val="12"/>
       <x:color theme="1"/>
@@ -32,8 +33,14 @@
       <x:color theme="1"/>
       <x:name val="Aptos Narrow"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos Narrow"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -53,6 +60,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor theme="4" tint="0.79995"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7E6E6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -76,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="16">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -96,6 +108,20 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -170,6 +196,25 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AsmRecoveryTable" displayName="AsmRecoveryTable" ref="A1:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="profile"/>
+    <x:tableColumn id="2" name="recovery_id"/>
+    <x:tableColumn id="3" name="scope_start"/>
+    <x:tableColumn id="4" name="scope_end"/>
+    <x:tableColumn id="5" name="sequence"/>
+    <x:tableColumn id="6" name="source_match"/>
+    <x:tableColumn id="7" name="source_replace"/>
+    <x:tableColumn id="8" name="expected_opcode"/>
+    <x:tableColumn id="9" name="status"/>
+    <x:tableColumn id="10" name="source_comment"/>
+    <x:tableColumn id="11" name="notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -27078,14 +27123,310 @@
         <x:v>The low two bits of the same live byte are the team mini-space selector; use MonsterTeamMember_SlotMask for that separate interpretation.</x:v>
       </x:c>
     </x:row>
-    <x:row r="532" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="533" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="534" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="535" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="536" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="537" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="538" s="6" customFormat="1" ht="26" customHeight="1"/>
-    <x:row r="539" s="6" customFormat="1" ht="26" customHeight="1"/>
+    <x:row r="532" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A532" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B532" t="str">
+        <x:v>Dungeon_ViewCell_LastIndex</x:v>
+      </x:c>
+      <x:c r="C532" t="str">
+        <x:v>$12</x:v>
+      </x:c>
+      <x:c r="D532" t="str">
+        <x:v>Draw_DungeonViewport</x:v>
+      </x:c>
+      <x:c r="E532" t="str">
+        <x:v>Draw_VisibleDungeonCells_Loop</x:v>
+      </x:c>
+      <x:c r="F532" t="str">
+        <x:v>moveq #$12,d6</x:v>
+      </x:c>
+      <x:c r="G532" t="str">
+        <x:v>7C12</x:v>
+      </x:c>
+      <x:c r="H532" t="str">
+        <x:v>moveq #Dungeon_ViewCell_LastIndex,d6</x:v>
+      </x:c>
+      <x:c r="I532" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J532" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K532" t="str">
+        <x:v>Highest zero-based index of the nineteen dungeon view cells.</x:v>
+      </x:c>
+      <x:c r="L532" t="str">
+        <x:v>Initialises the reverse occlusion-mask loop.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A533" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B533" t="str">
+        <x:v>Dungeon_ViewCell_LastIndex</x:v>
+      </x:c>
+      <x:c r="C533" t="str">
+        <x:v>$12</x:v>
+      </x:c>
+      <x:c r="D533" t="str">
+        <x:v>Build_DungeonVisibilityMasks_Loop</x:v>
+      </x:c>
+      <x:c r="E533" t="str">
+        <x:v>Apply_DungeonOcclusionMasks_Loop</x:v>
+      </x:c>
+      <x:c r="F533" t="str">
+        <x:v>cmpi.w #$0012,d6</x:v>
+      </x:c>
+      <x:c r="G533" t="str">
+        <x:v>0C460012</x:v>
+      </x:c>
+      <x:c r="H533" t="str">
+        <x:v>cmpi.w #Dungeon_ViewCell_LastIndex,d6</x:v>
+      </x:c>
+      <x:c r="I533" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J533" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K533" t="str">
+        <x:v>Highest zero-based index of the nineteen dungeon view cells.</x:v>
+      </x:c>
+      <x:c r="L533" t="str">
+        <x:v>Identifies the central-near view cell while building directional visibility masks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="534" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A534" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B534" t="str">
+        <x:v>Dungeon_MapCell_MainWallType</x:v>
+      </x:c>
+      <x:c r="C534" t="str">
+        <x:v>$01</x:v>
+      </x:c>
+      <x:c r="D534" t="str">
+        <x:v>Build_DungeonVisibilityMasks_Loop</x:v>
+      </x:c>
+      <x:c r="E534" t="str">
+        <x:v>Apply_DungeonOcclusionMasks_Loop</x:v>
+      </x:c>
+      <x:c r="F534" t="str">
+        <x:v>cmpi.b #$01,d0</x:v>
+      </x:c>
+      <x:c r="G534" t="str">
+        <x:v>0C000001</x:v>
+      </x:c>
+      <x:c r="H534" t="str">
+        <x:v>cmpi.b #Dungeon_MapCell_MainWallType,d0</x:v>
+      </x:c>
+      <x:c r="I534" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J534" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K534" t="str">
+        <x:v>Dungeon map-cell type for a main stone wall and its wall-mounted features.</x:v>
+      </x:c>
+      <x:c r="L534" t="str">
+        <x:v>The type is selected after Dungeon_CellTypeMask has removed the map-cell flag bits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A535" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B535" t="str">
+        <x:v>Dungeon_MapCell_MainWallType</x:v>
+      </x:c>
+      <x:c r="C535" t="str">
+        <x:v>$01</x:v>
+      </x:c>
+      <x:c r="D535" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="E535" t="str">
+        <x:v>Draw_ObjectOnFloor_ResolveGraphic</x:v>
+      </x:c>
+      <x:c r="F535" t="str">
+        <x:v>subq.w #$01,d3</x:v>
+      </x:c>
+      <x:c r="G535" t="str">
+        <x:v>5343</x:v>
+      </x:c>
+      <x:c r="H535" t="str">
+        <x:v>subq.w #Dungeon_MapCell_MainWallType,d3</x:v>
+      </x:c>
+      <x:c r="I535" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J535" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K535" t="str">
+        <x:v>Dungeon map-cell type for a main stone wall and its wall-mounted features.</x:v>
+      </x:c>
+      <x:c r="L535" t="str">
+        <x:v>The zero result selects the shelf-specific object X/Y placement path.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="536" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A536" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B536" t="str">
+        <x:v>ObjectFloor_SubpositionCount</x:v>
+      </x:c>
+      <x:c r="C536" t="str">
+        <x:v>$04</x:v>
+      </x:c>
+      <x:c r="D536" t="str">
+        <x:v>Draw_DungeonCellFloorObjects</x:v>
+      </x:c>
+      <x:c r="E536" t="str">
+        <x:v>GFX_ObjectsOnFloor_SubpositionRotation</x:v>
+      </x:c>
+      <x:c r="F536" t="str">
+        <x:v>cmpi.w #$0004,d1</x:v>
+      </x:c>
+      <x:c r="G536" t="str">
+        <x:v>0C410004</x:v>
+      </x:c>
+      <x:c r="H536" t="str">
+        <x:v>cmpi.w #ObjectFloor_SubpositionCount,d1</x:v>
+      </x:c>
+      <x:c r="I536" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J536" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K536" t="str">
+        <x:v>Number of rotated NW/NE/SW/SE object mini-spaces inspected in each dungeon cell.</x:v>
+      </x:c>
+      <x:c r="L536" t="str">
+        <x:v>The object stack position nibble selects one of these four values.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A537" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B537" t="str">
+        <x:v>ObjectFloor_HiddenXPosition</x:v>
+      </x:c>
+      <x:c r="C537" t="str">
+        <x:v>$80</x:v>
+      </x:c>
+      <x:c r="D537" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="E537" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="F537" t="str">
+        <x:v>cmpi.b #$80,d4</x:v>
+      </x:c>
+      <x:c r="G537" t="str">
+        <x:v>0C040080</x:v>
+      </x:c>
+      <x:c r="H537" t="str">
+        <x:v>cmpi.b #ObjectFloor_HiddenXPosition,d4</x:v>
+      </x:c>
+      <x:c r="I537" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J537" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K537" t="str">
+        <x:v>Signed X-position sentinel that suppresses an unavailable projected floor-object mini-space.</x:v>
+      </x:c>
+      <x:c r="L537" t="str">
+        <x:v>The same sentinel is stored in the X-position tables; it is tested before a sprite is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="538" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A538" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B538" t="str">
+        <x:v>ObjectFloor_WideShapeFirst</x:v>
+      </x:c>
+      <x:c r="C538" t="str">
+        <x:v>$12</x:v>
+      </x:c>
+      <x:c r="D538" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="E538" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="F538" t="str">
+        <x:v>cmpi.b #$12,d3</x:v>
+      </x:c>
+      <x:c r="G538" t="str">
+        <x:v>0C030012</x:v>
+      </x:c>
+      <x:c r="H538" t="str">
+        <x:v>cmpi.b #ObjectFloor_WideShapeFirst,d3</x:v>
+      </x:c>
+      <x:c r="I538" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="J538" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K538" t="str">
+        <x:v>First object floor-shape that uses the wide graphics bank and explicit projection-width selector.</x:v>
+      </x:c>
+      <x:c r="L538" t="str">
+        <x:v>Both comparisons use the same shape-family threshold.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539" s="6" customFormat="1" ht="26" customHeight="1">
+      <x:c r="A539" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B539" t="str">
+        <x:v>ObjectFloor_WideGraphicsOffset</x:v>
+      </x:c>
+      <x:c r="C539" t="str">
+        <x:v>$0CB8</x:v>
+      </x:c>
+      <x:c r="D539" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="E539" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="F539" t="str">
+        <x:v>add.w #$0CB8,a1</x:v>
+      </x:c>
+      <x:c r="G539" t="str">
+        <x:v>D2FC0CB8</x:v>
+      </x:c>
+      <x:c r="H539" t="str">
+        <x:v>add.w #ObjectFloor_WideGraphicsOffset,a1</x:v>
+      </x:c>
+      <x:c r="I539" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J539" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K539" t="str">
+        <x:v>Byte offset from the ordinary ObjectsOnFloor graphics to the wide-shape graphics bank.</x:v>
+      </x:c>
+      <x:c r="L539" t="str">
+        <x:v>Applied only after ObjectFloor_WideShapeFirst has selected a wide object shape.</x:v>
+      </x:c>
+    </x:row>
     <x:row r="540" s="6" customFormat="1" ht="26" customHeight="1"/>
     <x:row r="541" s="6" customFormat="1" ht="26" customHeight="1"/>
     <x:row r="542" s="6" customFormat="1" ht="26" customHeight="1"/>
@@ -54536,6 +54877,166 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="884">
+      <x:c r="A884" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B884" t="str">
+        <x:v>Draw_DungeonCellFloorObjects</x:v>
+      </x:c>
+      <x:c r="C884" t="str">
+        <x:v>GFX_ObjectsOnFloor_SubpositionRotation</x:v>
+      </x:c>
+      <x:c r="D884" t="str">
+        <x:v>bsr.s Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="E884" t="str">
+        <x:v>Draws every record attached to the selected rotated object mini-space before advancing to the next mini-space.</x:v>
+      </x:c>
+      <x:c r="F884" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="885">
+      <x:c r="A885" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B885" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="C885" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="D885" t="str">
+        <x:v>move.b GFX_ObjectsOnFloor_SubpositionRotation(pc,d0.w),d6</x:v>
+      </x:c>
+      <x:c r="E885" t="str">
+        <x:v>Rotates the stored NW/NE/SW/SE object mini-space into the viewer-relative mini-space.</x:v>
+      </x:c>
+      <x:c r="F885" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="886">
+      <x:c r="A886" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B886" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="C886" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="D886" t="str">
+        <x:v>subq.w #Dungeon_MapCell_MainWallType,d3</x:v>
+      </x:c>
+      <x:c r="E886" t="str">
+        <x:v>A zero result selects the shelf-specific X-position and Y-adjustment path; other map-cell types use floor placement.</x:v>
+      </x:c>
+      <x:c r="F886" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="887">
+      <x:c r="A887" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B887" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="C887" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="D887" t="str">
+        <x:v>cmpi.b #ObjectFloor_HiddenXPosition,d4</x:v>
+      </x:c>
+      <x:c r="E887" t="str">
+        <x:v>Skips this object mini-space when its source X-position entry is the hidden sentinel.</x:v>
+      </x:c>
+      <x:c r="F887" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="888">
+      <x:c r="A888" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B888" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="C888" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="D888" t="str">
+        <x:v>cmpi.b #ObjectFloor_WideShapeFirst,d3</x:v>
+      </x:c>
+      <x:c r="E888" t="str">
+        <x:v>Selects the wide graphics bank and explicit width selector for the wide floor-object shapes.</x:v>
+      </x:c>
+      <x:c r="F888" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="889">
+      <x:c r="A889" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B889" t="str">
+        <x:v>Draw_ObjectOnFloor</x:v>
+      </x:c>
+      <x:c r="C889" t="str">
+        <x:v>GFX_ObjectsOnFloor_Widths</x:v>
+      </x:c>
+      <x:c r="D889" t="str">
+        <x:v>add.w #ObjectFloor_WideGraphicsOffset,a1</x:v>
+      </x:c>
+      <x:c r="E889" t="str">
+        <x:v>Moves the sprite pointer from ordinary ObjectsOnFloor pictures to the wide-shape graphics bank.</x:v>
+      </x:c>
+      <x:c r="F889" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="890">
+      <x:c r="A890" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B890" t="str">
+        <x:v>Draw_Main_Shelf_Overlay</x:v>
+      </x:c>
+      <x:c r="C890" t="str">
+        <x:v>Draw_Main_Shelf_Visible</x:v>
+      </x:c>
+      <x:c r="D890" t="str">
+        <x:v>btst #$03,-$0011(a3)</x:v>
+      </x:c>
+      <x:c r="E890" t="str">
+        <x:v>In the normal player-view context, suppresses a shelf whose selected wall face is hidden by the current visibility mask.</x:v>
+      </x:c>
+      <x:c r="F890" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="891">
+      <x:c r="A891" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B891" t="str">
+        <x:v>Draw_DungeonCellOccupants</x:v>
+      </x:c>
+      <x:c r="C891" t="str">
+        <x:v>Draw_MonsterTeamOccupants</x:v>
+      </x:c>
+      <x:c r="D891" t="str">
+        <x:v>bsr Find_DungeonCellOccupant</x:v>
+      </x:c>
+      <x:c r="E891" t="str">
+        <x:v>Finds the player, champion, or unpacked monster occupying the current visible map coordinates before selecting its renderer.</x:v>
+      </x:c>
+      <x:c r="F891" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -54651,4 +55152,391 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="52" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>profile</x:v>
+      </x:c>
+      <x:c r="B1" s="13" t="str">
+        <x:v>recovery_id</x:v>
+      </x:c>
+      <x:c r="C1" s="13" t="str">
+        <x:v>scope_start</x:v>
+      </x:c>
+      <x:c r="D1" s="13" t="str">
+        <x:v>scope_end</x:v>
+      </x:c>
+      <x:c r="E1" s="13" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="F1" s="13" t="str">
+        <x:v>source_match</x:v>
+      </x:c>
+      <x:c r="G1" s="13" t="str">
+        <x:v>source_replace</x:v>
+      </x:c>
+      <x:c r="H1" s="13" t="str">
+        <x:v>expected_opcode</x:v>
+      </x:c>
+      <x:c r="I1" s="13" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="J1" s="13" t="str">
+        <x:v>source_comment</x:v>
+      </x:c>
+      <x:c r="K1" s="13" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A2" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B2" s="14" t="str">
+        <x:v>write_message_default</x:v>
+      </x:c>
+      <x:c r="C2" s="14" t="str">
+        <x:v>Ask_CC96</x:v>
+      </x:c>
+      <x:c r="D2" s="14" t="str">
+        <x:v>adrCd00D042</x:v>
+      </x:c>
+      <x:c r="E2" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="14" t="str">
+        <x:v>dc.w $7400</x:v>
+      </x:c>
+      <x:c r="G2" s="14" t="str">
+        <x:v>moveq #$00,d2</x:v>
+      </x:c>
+      <x:c r="H2" s="14" t="str">
+        <x:v>7400</x:v>
+      </x:c>
+      <x:c r="I2" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J2" s="15" t="str">
+        <x:v>Restores the zero-action alternate entry into the shared communication-message handler.</x:v>
+      </x:c>
+      <x:c r="K2" s="15" t="str">
+        <x:v>The missing entry label remains unresolved; the ;fiX Label expected marker is retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="28.799999237060547" hidden="0" customHeight="1">
+      <x:c r="A3" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>npc_message_default</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>adrCd00D81C</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="str">
+        <x:v>adrCd00D824</x:v>
+      </x:c>
+      <x:c r="E3" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="14" t="str">
+        <x:v>dc.w $7400</x:v>
+      </x:c>
+      <x:c r="G3" s="14" t="str">
+        <x:v>moveq #$00,d2</x:v>
+      </x:c>
+      <x:c r="H3" s="14" t="str">
+        <x:v>7400</x:v>
+      </x:c>
+      <x:c r="I3" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J3" s="15" t="str">
+        <x:v>Restores the zero-action alternate entry into the shared NPC/message handler.</x:v>
+      </x:c>
+      <x:c r="K3" s="15" t="str">
+        <x:v>The missing entry label remains unresolved; the ;fiX Label expected marker is retained.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="43.20000076293945" hidden="0" customHeight="1">
+      <x:c r="A4" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B4" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C4" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D4" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E4" s="14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F4" s="14" t="str">
+        <x:v>dc.w $4843</x:v>
+      </x:c>
+      <x:c r="G4" s="14" t="str">
+        <x:v>swap d3</x:v>
+      </x:c>
+      <x:c r="H4" s="14" t="str">
+        <x:v>4843</x:v>
+      </x:c>
+      <x:c r="I4" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J4" s="15" t="str">
+        <x:v>Restores the square filled-bar setup which copies one common size into the packed width and height before falling through to BW_draw_bar.</x:v>
+      </x:c>
+      <x:c r="K4" s="15" t="str">
+        <x:v>The instruction sequence is statically verified; the eventual entry label remains a separate FIX_LABELS investigation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>dc.w $4844</x:v>
+      </x:c>
+      <x:c r="G5" s="14" t="str">
+        <x:v>swap d4</x:v>
+      </x:c>
+      <x:c r="H5" s="14" t="str">
+        <x:v>4844</x:v>
+      </x:c>
+      <x:c r="I5" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J5" s="15" t="str"/>
+      <x:c r="K5" s="15" t="str"/>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>dc.w $4845</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str">
+        <x:v>swap d5</x:v>
+      </x:c>
+      <x:c r="H6" s="14" t="str">
+        <x:v>4845</x:v>
+      </x:c>
+      <x:c r="I6" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J6" s="15" t="str"/>
+      <x:c r="K6" s="15" t="str"/>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>dc.w $3803</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="str">
+        <x:v>move.w d3,d4</x:v>
+      </x:c>
+      <x:c r="H7" s="14" t="str">
+        <x:v>3803</x:v>
+      </x:c>
+      <x:c r="I7" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J7" s="15" t="str"/>
+      <x:c r="K7" s="15" t="str"/>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C8" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D8" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E8" s="14" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F8" s="14" t="str">
+        <x:v>dc.w $3A03</x:v>
+      </x:c>
+      <x:c r="G8" s="14" t="str">
+        <x:v>move.w d3,d5</x:v>
+      </x:c>
+      <x:c r="H8" s="14" t="str">
+        <x:v>3A03</x:v>
+      </x:c>
+      <x:c r="I8" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J8" s="15" t="str"/>
+      <x:c r="K8" s="15" t="str"/>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C9" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D9" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E9" s="14" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="F9" s="14" t="str">
+        <x:v>dc.w $4843</x:v>
+      </x:c>
+      <x:c r="G9" s="14" t="str">
+        <x:v>swap d3</x:v>
+      </x:c>
+      <x:c r="H9" s="14" t="str">
+        <x:v>4843</x:v>
+      </x:c>
+      <x:c r="I9" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J9" s="15" t="str"/>
+      <x:c r="K9" s="15" t="str"/>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B10" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C10" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D10" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E10" s="14" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F10" s="14" t="str">
+        <x:v>dc.w $4844</x:v>
+      </x:c>
+      <x:c r="G10" s="14" t="str">
+        <x:v>swap d4</x:v>
+      </x:c>
+      <x:c r="H10" s="14" t="str">
+        <x:v>4844</x:v>
+      </x:c>
+      <x:c r="I10" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J10" s="15" t="str"/>
+      <x:c r="K10" s="15" t="str"/>
+    </x:row>
+    <x:row r="11" ht="15" hidden="0" customHeight="1">
+      <x:c r="A11" s="14" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B11" s="14" t="str">
+        <x:v>draw_square</x:v>
+      </x:c>
+      <x:c r="C11" s="14" t="str">
+        <x:v>BW_blitchar_data</x:v>
+      </x:c>
+      <x:c r="D11" s="14" t="str">
+        <x:v>BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E11" s="14" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F11" s="14" t="str">
+        <x:v>dc.w $4845</x:v>
+      </x:c>
+      <x:c r="G11" s="14" t="str">
+        <x:v>swap d5</x:v>
+      </x:c>
+      <x:c r="H11" s="14" t="str">
+        <x:v>4845</x:v>
+      </x:c>
+      <x:c r="I11" s="14" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="J11" s="15" t="str"/>
+      <x:c r="K11" s="15" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="I2:I200">
+      <x:formula1>"verified,proposed,disabled"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d6085451e1543af"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Improved map and object editor
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Rf741535eb9cd45f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rb3c795a76b504f24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="Re31782dcd32948f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R65497b0e63264d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Rd41e12ce743a4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R1e2ae629d9d44348"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R2b3083025c004bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="Rd11583fb66dc4f1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -88,7 +88,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="16">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -122,6 +122,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -55037,6 +55040,66 @@
         <x:v>1</x:v>
       </x:c>
     </x:row>
+    <x:row r="892" ht="45" customHeight="1">
+      <x:c r="A892" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B892" t="str">
+        <x:v>adrCd008702</x:v>
+      </x:c>
+      <x:c r="C892" t="str">
+        <x:v>adrCd008726</x:v>
+      </x:c>
+      <x:c r="D892" t="str">
+        <x:v>clr.b adrB_0088A2.l</x:v>
+      </x:c>
+      <x:c r="E892" s="16" t="str">
+        <x:v>Clears the cached floppy-side state before pulsing DF0 select with the CIAB side-select bit set.</x:v>
+      </x:c>
+      <x:c r="F892" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="893" ht="45" customHeight="1">
+      <x:c r="A893" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B893" t="str">
+        <x:v>adrCd008726</x:v>
+      </x:c>
+      <x:c r="C893" t="str">
+        <x:v>adrCd008760</x:v>
+      </x:c>
+      <x:c r="D893" t="str">
+        <x:v>tst.b adrB_0088A2.l</x:v>
+      </x:c>
+      <x:c r="E893" s="16" t="str">
+        <x:v>Chooses the CIAB head-step control pattern from the cached floppy-side state.</x:v>
+      </x:c>
+      <x:c r="F893" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="894" ht="45" customHeight="1">
+      <x:c r="A894" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B894" t="str">
+        <x:v>adrCd0087A6</x:v>
+      </x:c>
+      <x:c r="C894" t="str">
+        <x:v>adrCd0087AC</x:v>
+      </x:c>
+      <x:c r="D894" t="str">
+        <x:v>moveq #$03,d6</x:v>
+      </x:c>
+      <x:c r="E894" s="16" t="str">
+        <x:v>Initialises the disk-read retry counter to three attempts; the internal entry at $879A decrements it before restarting DMA setup.</x:v>
+      </x:c>
+      <x:c r="F894" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -55206,7 +55269,7 @@
         <x:v>notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="28.799999237060547" hidden="0" customHeight="1">
+    <x:row r="2" ht="84" hidden="0" customHeight="1">
       <x:c r="A2" s="14" t="str">
         <x:v>BLOODWYCH439</x:v>
       </x:c>
@@ -55238,10 +55301,10 @@
         <x:v>Restores the zero-action alternate entry into the shared communication-message handler.</x:v>
       </x:c>
       <x:c r="K2" s="15" t="str">
-        <x:v>The missing entry label remains unresolved; the ;fiX Label expected marker is retained.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="28.799999237060547" hidden="0" customHeight="1">
+        <x:v>The missing entry label remains unresolved. Static analysis found no direct control-flow reference, absolute code pointer, or word-offset jump-table entry to $D040; a live breakpoint should record the caller/return PC if this alternate entry executes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="84" hidden="0" customHeight="1">
       <x:c r="A3" s="14" t="str">
         <x:v>BLOODWYCH439</x:v>
       </x:c>
@@ -55273,10 +55336,10 @@
         <x:v>Restores the zero-action alternate entry into the shared NPC/message handler.</x:v>
       </x:c>
       <x:c r="K3" s="15" t="str">
-        <x:v>The missing entry label remains unresolved; the ;fiX Label expected marker is retained.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="43.20000076293945" hidden="0" customHeight="1">
+        <x:v>The missing entry label remains unresolved. Static analysis found no direct control-flow reference, absolute code pointer, or word-offset jump-table entry to $D822; a live breakpoint should record the caller/return PC if this alternate entry executes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="84" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="str">
         <x:v>BLOODWYCH439</x:v>
       </x:c>
@@ -55308,7 +55371,7 @@
         <x:v>Restores the square filled-bar setup which copies one common size into the packed width and height before falling through to BW_draw_bar.</x:v>
       </x:c>
       <x:c r="K4" s="15" t="str">
-        <x:v>The instruction sequence is statically verified; the eventual entry label remains a separate FIX_LABELS investigation.</x:v>
+        <x:v>The instructions and square filled-bar behaviour are statically verified. No direct control-flow reference, absolute code pointer, or word-offset jump-table entry to $DA58 was found; a live breakpoint should record the caller PC and D3/D4/D5 if this entry executes.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
@@ -55536,7 +55599,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d6085451e1543af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38489c5f1f5249c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
allow book of skulls pre-patch data to be used, minor bug fix for monster viewer and added layout editor for maps
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="Rd41e12ce743a4d31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R1e2ae629d9d44348"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R2b3083025c004bb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="Rd11583fb66dc4f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R5caa659f67b14c42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R7c4461eaec3c4280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="Rb8068ab6101142a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="Re45e182a939940d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_NOTES" sheetId="5" r:id="R59c96514632f498b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,6 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="0"/>
+  </x:numFmts>
   <x:fonts count="4">
     <x:font>
       <x:sz val="12"/>
@@ -40,7 +44,7 @@
       <x:name val="Aptos Narrow"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,8 +71,13 @@
         <x:fgColor rgb="FFE7E6E6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="4">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -84,11 +93,24 @@
         <x:color auto="1"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -125,6 +147,22 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -55599,7 +55637,182 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38489c5f1f5249c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12d8447098a94fad"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="64" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="20" t="str">
+        <x:v>profile</x:v>
+      </x:c>
+      <x:c r="B1" s="20" t="str">
+        <x:v>scope_start</x:v>
+      </x:c>
+      <x:c r="C1" s="20" t="str">
+        <x:v>scope_end</x:v>
+      </x:c>
+      <x:c r="D1" s="20" t="str">
+        <x:v>source_match</x:v>
+      </x:c>
+      <x:c r="E1" s="20" t="str">
+        <x:v>source_comment</x:v>
+      </x:c>
+      <x:c r="F1" s="20" t="str">
+        <x:v>expected_matches</x:v>
+      </x:c>
+      <x:c r="G1" s="20" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="H1" s="20" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="21" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B2" s="21" t="str">
+        <x:v>CopyProtection</x:v>
+      </x:c>
+      <x:c r="C2" s="21" t="str">
+        <x:v>adrEA00D186</x:v>
+      </x:c>
+      <x:c r="D2" s="21" t="str">
+        <x:v>;fiX Label expected</x:v>
+      </x:c>
+      <x:c r="E2" s="21" t="str">
+        <x:v>COPY_PROTECTION_INTERNAL ($D140): Reserved workspace leading into the saved-register area.</x:v>
+      </x:c>
+      <x:c r="F2" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="21" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="H2" s="21" t="str">
+        <x:v>Protection internal; preserve the original raw declarations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="21" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B3" s="21" t="str">
+        <x:v>adrCd00D1FC</x:v>
+      </x:c>
+      <x:c r="C3" s="21" t="str">
+        <x:v>adrEA00D2D2</x:v>
+      </x:c>
+      <x:c r="D3" s="21" t="str">
+        <x:v>;fiX Label expected</x:v>
+      </x:c>
+      <x:c r="E3" s="21" t="str">
+        <x:v>COPY_PROTECTION_INTERNAL ($D21C): Opaque instruction/data stream entered through the deliberate exception path.</x:v>
+      </x:c>
+      <x:c r="F3" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G3" s="21" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="H3" s="21" t="str">
+        <x:v>Protection internal; preserve the original raw declarations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="21" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="str">
+        <x:v>adrCd00D332</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="str">
+        <x:v>adrCd00D51E</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="str">
+        <x:v>;fiX Label expected</x:v>
+      </x:c>
+      <x:c r="E4" s="21" t="str">
+        <x:v>COPY_PROTECTION_INTERNAL ($D338): Opaque word stream following the exception-handler return.</x:v>
+      </x:c>
+      <x:c r="F4" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G4" s="21" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="H4" s="21" t="str">
+        <x:v>Protection internal; preserve the original raw declarations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="21" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B5" s="21" t="str">
+        <x:v>adrCd00D56A</x:v>
+      </x:c>
+      <x:c r="C5" s="21" t="str">
+        <x:v>adrCd00D59A</x:v>
+      </x:c>
+      <x:c r="D5" s="21" t="str">
+        <x:v>;fiX Label expected</x:v>
+      </x:c>
+      <x:c r="E5" s="21" t="str">
+        <x:v>COPY_PROTECTION_INTERNAL ($D584): Encoded word block deliberately skipped by the visible execution paths.</x:v>
+      </x:c>
+      <x:c r="F5" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G5" s="21" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="H5" s="21" t="str">
+        <x:v>Protection internal; preserve the original raw declarations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="21" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B6" s="21" t="str">
+        <x:v>adrCd00D59A</x:v>
+      </x:c>
+      <x:c r="C6" s="21" t="str">
+        <x:v>adrEA00D740</x:v>
+      </x:c>
+      <x:c r="D6" s="21" t="str">
+        <x:v>;fiX Label expected</x:v>
+      </x:c>
+      <x:c r="E6" s="21" t="str">
+        <x:v>COPY_PROTECTION_INTERNAL ($D59E): Opaque stream following the deliberate illegal instruction; retained as raw words.</x:v>
+      </x:c>
+      <x:c r="F6" s="22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="21" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="H6" s="21" t="str">
+        <x:v>Protection internal; preserve the original raw declarations.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
New investigation data and updated source files. PLus minor fixes for joypad controls.
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R957b6ad5bfdd4433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="R4f4943cddd844106"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R552f86f35bb9417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R880cb76e18ad4ba0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_NOTES" sheetId="5" r:id="R5a5b5e820e5c4b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R54bdfbcae3ef4eb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rdb797eab24324ff0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R5954448ee2f44e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R98b9dd3391754991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_NOTES" sheetId="5" r:id="Rcd31dcd29c3e494b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -40225,30 +40225,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B294" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">UnpackTowerMonsters</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C294" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">.ClearMonsterTeamIndexLoop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D294" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr		Map_Traps_InitProcessing_AI_TBC</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E294" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Initialises the trap-processing state before monster placement changes the current tower map.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F294" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
+      <x:c r="B294" t="str">
+        <x:v>UnpackTowerMonsters</x:v>
+      </x:c>
+      <x:c r="C294" t="str">
+        <x:v>.ClearMonsterTeamIndexLoop</x:v>
+      </x:c>
+      <x:c r="D294" t="str">
+        <x:v>bsr Mark_CurrentTowerTrapCells</x:v>
+      </x:c>
+      <x:c r="E294" t="str">
+        <x:v>Initialises the trap-processing state before monster placement changes the current tower map.</x:v>
+      </x:c>
+      <x:c r="F294" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="295">
@@ -49507,30 +49497,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B594" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd007BC0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C594" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd007BE8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D594" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">move.w $0012(a5),d3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E594" s="9" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Loads PlayerData_UISecondaryColourOffset: the replacement ink palette index for the player-coloured Pockets command and toggle icons.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F594" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
+      <x:c r="B594" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C594" t="str">
+        <x:v>Draw_PartyCommandIconStrip</x:v>
+      </x:c>
+      <x:c r="D594" t="str">
+        <x:v>move.w $0012(a5),d3</x:v>
+      </x:c>
+      <x:c r="E594" s="9" t="str">
+        <x:v>Loads PlayerData_UISecondaryColourOffset: the replacement ink palette index for the player-coloured Pockets command and toggle icons.</x:v>
+      </x:c>
+      <x:c r="F594" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="595" ht="28.799999237060547" customHeight="1">
@@ -50543,28 +50523,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B628" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionNamePanelFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C628" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionNamePanelLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D628" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr BW_blit_horiz_line</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E628" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draws the upper bevel's four stepped grey lines at Y=$0A-$0D, then its final colour-$01 line at Y=$0E.</x:t>
-        </x:is>
+      <x:c r="B628" t="str">
+        <x:v>Draw_ChampionNamePanelFrame</x:v>
+      </x:c>
+      <x:c r="C628" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="D628" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E628" t="str">
+        <x:v>Draws an upper champion-name bevel scanline; the loop produces colours $01-$04 and the final call closes it with colour $01.</x:v>
       </x:c>
       <x:c r="F628" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="629">
@@ -50723,28 +50695,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B634" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionNamePanelLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C634" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_DungeonDisplayLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D634" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr BW_blit_horiz_line</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E634" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draws the four-scanline lower grey bevel at Y=$19-$1C with colour indices $01-$04.</x:t>
-        </x:is>
+      <x:c r="B634" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C634" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="D634" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E634" t="str">
+        <x:v>Draws one scanline of the lower champion-name bevel; the loop repeats it for palette colours $01-$04.</x:v>
       </x:c>
       <x:c r="F634" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="635">
@@ -50843,25 +50807,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B638" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionNamePanelLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C638" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_DungeonDisplayLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D638" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr BW_blit_horiz_line</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E638" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draws the mini bevel's top line at Y=$20 and its icon-height divider at Y=$31.</x:t>
-        </x:is>
+      <x:c r="B638" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="C638" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="D638" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E638" t="str">
+        <x:v>Draws the mini bevel's top line at Y=$20 and its icon-height divider at Y=$31.</x:v>
       </x:c>
       <x:c r="F638" t="n">
         <x:v>2</x:v>
@@ -50933,28 +50889,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B641" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_DungeonDisplayLowerEdge</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C641" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd008396</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D641" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr BW_blit_horiz_line</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E641" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draws the mini bevel's lower scale at Y=$33-$37: colour $01, then $02-$04, then $01.</x:t>
-        </x:is>
+      <x:c r="B641" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="C641" t="str">
+        <x:v>adrCd008358</x:v>
+      </x:c>
+      <x:c r="D641" t="str">
+        <x:v>bsr BW_blit_horiz_line</x:v>
+      </x:c>
+      <x:c r="E641" t="str">
+        <x:v>Draws a lower mini-bevel scanline; the loop produces colours $01-$04 and the final call closes it with colour $01.</x:v>
       </x:c>
       <x:c r="F641" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="642">
@@ -50993,28 +50941,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B643" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd008396</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C643" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd008416</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D643" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">add.w adrW_00838E(pc,d2.w),a0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E643" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Applies the compact four-slot screen-offset sequence for profession controls: upper-left, upper-right, lower-right, lower-left.</x:t>
-        </x:is>
+      <x:c r="B643" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="C643" t="str">
+        <x:v>adrCd008416</x:v>
+      </x:c>
+      <x:c r="D643" t="str">
+        <x:v>add.w adrW_00838E(pc,d2.w),a0</x:v>
+      </x:c>
+      <x:c r="E643" t="str">
+        <x:v>Applies the compact four-slot screen-offset sequence for profession controls: upper-left, upper-right, lower-right, lower-left.</x:v>
       </x:c>
       <x:c r="F643" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="644">
@@ -51413,25 +51353,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B657" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_CommsAndOptions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C657" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_PauseGame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D657" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cmpi.w #$0037,d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E657" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Separates the upper large-avatar selection from the lower shield-slot selection path before the selected PlayerX_Data+$003E bit is toggled.</x:t>
-        </x:is>
+      <x:c r="B657" t="str">
+        <x:v>Click_ChampionPresentationOrPartyCommand</x:v>
+      </x:c>
+      <x:c r="C657" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D657" t="str">
+        <x:v>cmpi.w #PartyPresentation_LowerFirstY,d1</x:v>
+      </x:c>
+      <x:c r="E657" t="str">
+        <x:v>Separates lower shield clicks from the main-avatar and party-command region above.</x:v>
       </x:c>
       <x:c r="F657" t="n">
         <x:v>1</x:v>
@@ -51443,25 +51375,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B658" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_CommsAndOptions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C658" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_PauseGame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D658" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lsr.w #$05,d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E658" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Converts the lower shield-click X coordinate to a 32-pixel column index; the following add selects PlayerX_Data+$003E bits one through three.</x:t>
-        </x:is>
+      <x:c r="B658" t="str">
+        <x:v>Click_ChampionPresentationOrPartyCommand</x:v>
+      </x:c>
+      <x:c r="C658" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D658" t="str">
+        <x:v>lsr.w #$05,d1</x:v>
+      </x:c>
+      <x:c r="E658" t="str">
+        <x:v>Converts the lower shield-click X coordinate to a 32-pixel column index; the following add selects PlayerData_AvatarPresentationState bits one through three.</x:v>
       </x:c>
       <x:c r="F658" t="n">
         <x:v>1</x:v>
@@ -51473,25 +51397,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B659" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_CommsAndOptions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C659" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_PauseGame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D659" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bchg d1,$003E(a5)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E659" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Toggles only the clicked left-side avatar's presentation bit. This is independent of right-side Click_PartyMember actions $06-$09.</x:t>
-        </x:is>
+      <x:c r="B659" t="str">
+        <x:v>Click_ChampionPresentationOrPartyCommand</x:v>
+      </x:c>
+      <x:c r="C659" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D659" t="str">
+        <x:v>bchg d1,PlayerData_AvatarPresentationState(a5)</x:v>
+      </x:c>
+      <x:c r="E659" t="str">
+        <x:v>Toggles only the clicked left-side avatar's presentation bit. This is independent of right-side Click_PartyMember actions $06-$09.</x:v>
       </x:c>
       <x:c r="F659" t="n">
         <x:v>1</x:v>
@@ -51503,25 +51419,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B660" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_CommsAndOptions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C660" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_PauseGame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D660" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Refresh_PartyShieldSlotIfDirty</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E660" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Refreshes the clicked party shield slot after changing its presentation bit; the selected living path draws the one-step-away full character.</x:t>
-        </x:is>
+      <x:c r="B660" t="str">
+        <x:v>Click_ChampionPresentationOrPartyCommand</x:v>
+      </x:c>
+      <x:c r="C660" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D660" t="str">
+        <x:v>bsr Refresh_PartyShieldSlotIfDirty</x:v>
+      </x:c>
+      <x:c r="E660" t="str">
+        <x:v>Refreshes the clicked party shield slot after changing its presentation bit; the selected living path draws the one-step-away full character.</x:v>
       </x:c>
       <x:c r="F660" t="n">
         <x:v>1</x:v>
@@ -52163,25 +52071,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B682" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd008358</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C682" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd008396</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D682" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lea adrEA050302.l,a1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E682" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Uses the packed inventory interface strip at GFX_Pockets+$3C00 as the source graphic for each inventory chain decoration.</x:t>
-        </x:is>
+      <x:c r="B682" t="str">
+        <x:v>adrCd008358</x:v>
+      </x:c>
+      <x:c r="C682" t="str">
+        <x:v>adrCd008396</x:v>
+      </x:c>
+      <x:c r="D682" t="str">
+        <x:v>lea GFX_Pockets+$3C00.l,a1</x:v>
+      </x:c>
+      <x:c r="E682" t="str">
+        <x:v>Uses the packed inventory interface strip at GFX_Pockets+$3C00 as the source graphic for each inventory chain decoration.</x:v>
       </x:c>
       <x:c r="F682" t="n">
         <x:v>1</x:v>
@@ -52733,25 +52633,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B701" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Click_ChampionPresentationOrPartyCommand</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C701" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd0042B8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D701" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cmpi.w #$0037,d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E701" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Separates the three lower party-shield rows (Y &gt;= $37) from the main-avatar/party-command region above.</x:t>
-        </x:is>
+      <x:c r="B701" s="8" t="str">
+        <x:v>Click_ChampionPresentationOrPartyCommand</x:v>
+      </x:c>
+      <x:c r="C701" s="8" t="str">
+        <x:v>Return_PartyCommandEntry</x:v>
+      </x:c>
+      <x:c r="D701" s="8" t="str">
+        <x:v>cmpi.w #PartyPresentation_LowerFirstY,d1</x:v>
+      </x:c>
+      <x:c r="E701" s="8" t="str">
+        <x:v>Separates the three lower party-shield rows from the main-avatar and party-command region above.</x:v>
       </x:c>
       <x:c r="F701" s="8" t="n">
         <x:v>1</x:v>
@@ -52823,25 +52715,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B704" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Toggle_ChampionPresentation</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C704" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrJA00425E</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D704" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bchg d1,$003E(a5)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E704" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Toggles the presentation bit for the selected main or lower champion slot; the renderer uses this state to choose portrait or standing artwork.</x:t>
-        </x:is>
+      <x:c r="B704" s="8" t="str">
+        <x:v>Toggle_ChampionPresentation</x:v>
+      </x:c>
+      <x:c r="C704" s="8" t="str">
+        <x:v>Click_PauseGame</x:v>
+      </x:c>
+      <x:c r="D704" s="8" t="str">
+        <x:v>bchg d1,PlayerData_AvatarPresentationState(a5)</x:v>
+      </x:c>
+      <x:c r="E704" s="8" t="str">
+        <x:v>Toggles the presentation bit for the selected main or lower champion slot; the renderer uses this state to choose portrait or standing artwork.</x:v>
       </x:c>
       <x:c r="F704" s="8" t="n">
         <x:v>1</x:v>
@@ -53303,25 +53187,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B720" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyCommandIconStrip</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C720" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd007BE8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D720" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">moveq #$71,d7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E720" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Starts the command-panel pocket-graphic sequence at GFX_Pockets picture $71.</x:t>
-        </x:is>
+      <x:c r="B720" s="8" t="str">
+        <x:v>Draw_PartyCommandInterface</x:v>
+      </x:c>
+      <x:c r="C720" s="8" t="str">
+        <x:v>Draw_PartyCommandIconStrip</x:v>
+      </x:c>
+      <x:c r="D720" s="8" t="str">
+        <x:v>moveq #$71,d7</x:v>
+      </x:c>
+      <x:c r="E720" s="8" t="str">
+        <x:v>Starts the command-panel pocket-graphic sequence at GFX_Pockets picture $71.</x:v>
       </x:c>
       <x:c r="F720" s="8" t="n">
         <x:v>1</x:v>
@@ -53333,25 +53209,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B721" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyCommandIconStrip</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C721" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd007BE8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D721" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">addi.w #$027C,a0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E721" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advances the destination to the next command-icon row after each pair of pocket graphics.</x:t>
-        </x:is>
+      <x:c r="B721" s="8" t="str">
+        <x:v>Draw_PartyCommandIconStrip</x:v>
+      </x:c>
+      <x:c r="C721" s="8" t="str">
+        <x:v>adrCd007BE8</x:v>
+      </x:c>
+      <x:c r="D721" s="8" t="str">
+        <x:v>add.w #$027C,a0</x:v>
+      </x:c>
+      <x:c r="E721" s="8" t="str">
+        <x:v>Advances the destination to the next command-icon row after each pair of pocket graphics.</x:v>
       </x:c>
       <x:c r="F721" s="8" t="n">
         <x:v>1</x:v>
@@ -53693,25 +53561,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B733" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_InventoryPocketSlots</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C733" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">ObjectGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D733" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">addi.w #$0274,a0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E733" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Moves the pocket-graphic destination from the first six-slot row to the second.</x:t>
-        </x:is>
+      <x:c r="B733" s="8" t="str">
+        <x:v>Draw_InventoryPocketSlots</x:v>
+      </x:c>
+      <x:c r="C733" s="8" t="str">
+        <x:v>ObjectGraphic</x:v>
+      </x:c>
+      <x:c r="D733" s="8" t="str">
+        <x:v>add.w #$0274,a0</x:v>
+      </x:c>
+      <x:c r="E733" s="8" t="str">
+        <x:v>Moves the pocket-graphic destination from the first six-slot row to the second.</x:v>
       </x:c>
       <x:c r="F733" s="8" t="n">
         <x:v>1</x:v>
@@ -53753,25 +53613,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B735" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PocketGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C735" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrJA00CB0A</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D735" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cmpi.b #$14,d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E735" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Splits the Pockets.gfx picture index into 20-icon banks before converting the in-bank index to a source offset.</x:t>
-        </x:is>
+      <x:c r="B735" s="8" t="str">
+        <x:v>Draw_PocketGraphic</x:v>
+      </x:c>
+      <x:c r="C735" s="8" t="str">
+        <x:v>adrCd00CB0A</x:v>
+      </x:c>
+      <x:c r="D735" s="8" t="str">
+        <x:v>cmpi.b #$14,d0</x:v>
+      </x:c>
+      <x:c r="E735" s="8" t="str">
+        <x:v>Splits the Pockets.gfx picture index into 20-icon banks before converting the in-bank index to a source offset.</x:v>
       </x:c>
       <x:c r="F735" s="8" t="n">
         <x:v>1</x:v>
@@ -53783,25 +53635,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B736" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PocketGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C736" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrJA00CB0A</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D736" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">addi.w #$0A00,a1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E736" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advances one 20-icon Pockets.gfx bank (20 × $80 bytes) for picture indices at or above $14.</x:t>
-        </x:is>
+      <x:c r="B736" s="8" t="str">
+        <x:v>Draw_PocketGraphic</x:v>
+      </x:c>
+      <x:c r="C736" s="8" t="str">
+        <x:v>adrCd00CB0A</x:v>
+      </x:c>
+      <x:c r="D736" s="8" t="str">
+        <x:v>add.w #$0A00,a1</x:v>
+      </x:c>
+      <x:c r="E736" s="8" t="str">
+        <x:v>Advances one 20-icon Pockets.gfx bank (20 x $80 bytes) for picture indices at or above $14.</x:v>
       </x:c>
       <x:c r="F736" s="8" t="n">
         <x:v>1</x:v>
@@ -53813,25 +53657,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B737" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PocketGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C737" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrJA00CB0A</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D737" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">asl.w #$03,d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E737" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Converts the in-bank picture index to its 16×16 four-plane source offset.</x:t>
-        </x:is>
+      <x:c r="B737" s="8" t="str">
+        <x:v>adrCd00CB0A</x:v>
+      </x:c>
+      <x:c r="C737" s="8" t="str">
+        <x:v>adrCd00CB1C</x:v>
+      </x:c>
+      <x:c r="D737" s="8" t="str">
+        <x:v>asl.w #$03,d0</x:v>
+      </x:c>
+      <x:c r="E737" s="8" t="str">
+        <x:v>Converts the in-bank picture index to its 16x16 four-plane source offset.</x:v>
       </x:c>
       <x:c r="F737" s="8" t="n">
         <x:v>1</x:v>
@@ -53963,28 +53799,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B742" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_CompactStatsFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C742" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainPlayerInterface</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D742" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">add.w $0008(a5),d5</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E742" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Applies the active player's screen Y offset to the current drawing coordinate.</x:t>
-        </x:is>
+      <x:c r="B742" s="8" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="C742" s="8" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="D742" s="8" t="str">
+        <x:v>add.w $0008(a5),d5</x:v>
+      </x:c>
+      <x:c r="E742" s="8" t="str">
+        <x:v>Applies the active player's screen Y offset to the current drawing coordinate.</x:v>
       </x:c>
       <x:c r="F742" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="743">
@@ -54413,25 +54241,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B757" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainPlayerInterface</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C757" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyShieldStatusBars</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D757" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr BW_draw_bar</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E757" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Calls the filled-rectangle drawing routine for the compact-stat bar background.</x:t>
-        </x:is>
+      <x:c r="B757" s="8" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="C757" s="8" t="str">
+        <x:v>Draw_CompactStatsBarsLoop</x:v>
+      </x:c>
+      <x:c r="D757" s="8" t="str">
+        <x:v>bsr BW_draw_bar</x:v>
+      </x:c>
+      <x:c r="E757" s="8" t="str">
+        <x:v>Calls the filled-rectangle drawing routine for the compact-stat bar background.</x:v>
       </x:c>
       <x:c r="F757" s="8" t="n">
         <x:v>1</x:v>
@@ -54743,25 +54563,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B768" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_CompactStatsBarsLoop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C768" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_CompactStatsBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D768" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Prepare_CompactStatBarLength</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E768" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Prepares the compact-bar geometry and scales current D0 against maximum D1.</x:t>
-        </x:is>
+      <x:c r="B768" s="8" t="str">
+        <x:v>Draw_CompactStatsBarsLoop</x:v>
+      </x:c>
+      <x:c r="C768" s="8" t="str">
+        <x:v>Advance_CompactStatsBarRow</x:v>
+      </x:c>
+      <x:c r="D768" s="8" t="str">
+        <x:v>bsr.s Prepare_CompactStatBarLength</x:v>
+      </x:c>
+      <x:c r="E768" s="8" t="str">
+        <x:v>Prepares the compact-bar geometry and scales current D0 against maximum D1.</x:v>
       </x:c>
       <x:c r="F768" s="8" t="n">
         <x:v>1</x:v>
@@ -55073,25 +54885,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B779" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyShieldStatusBars</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C779" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_PartyShieldStatusBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D779" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">moveq #$03,d6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E779" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Uses DBRA terminal index three to visit all four party shield slots.</x:t>
-        </x:is>
+      <x:c r="B779" s="8" t="str">
+        <x:v>Draw_PartyShieldStatusBars</x:v>
+      </x:c>
+      <x:c r="C779" s="8" t="str">
+        <x:v>Draw_PartyShieldStatusBarsLoop</x:v>
+      </x:c>
+      <x:c r="D779" s="8" t="str">
+        <x:v>moveq #PartyShieldStatusBar_LastSlot,d6</x:v>
+      </x:c>
+      <x:c r="E779" s="8" t="str">
+        <x:v>Uses the last-slot index to visit all four party shield slots with DBRA.</x:v>
       </x:c>
       <x:c r="F779" s="8" t="n">
         <x:v>1</x:v>
@@ -55103,28 +54907,20 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B780" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyShieldStatusBarsLoop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C780" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_PartyShieldStatusBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D780" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">move.b $18(a5,d6.w),d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E780" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Loads one party-slot state byte so vacant, dead, and occupied slots can be distinguished.</x:t>
-        </x:is>
+      <x:c r="B780" s="8" t="str">
+        <x:v>Draw_PartyShieldStatusBarsLoop</x:v>
+      </x:c>
+      <x:c r="C780" s="8" t="str">
+        <x:v>Advance_PartyShieldStatusBarRow</x:v>
+      </x:c>
+      <x:c r="D780" s="8" t="str">
+        <x:v>move.b $18(a5,d6.w),d0</x:v>
+      </x:c>
+      <x:c r="E780" s="8" t="str">
+        <x:v>Loads or reloads the current party-slot state byte for suppression checks and champion selection.</x:v>
       </x:c>
       <x:c r="F780" s="8" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="781">
@@ -55133,25 +54929,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B781" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyShieldStatusBarsLoop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C781" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_PartyShieldStatusBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D781" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">and.w #$00E0,d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E781" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Tests the party-slot vacant/dead suppression bits before drawing a status bar.</x:t>
-        </x:is>
+      <x:c r="B781" s="8" t="str">
+        <x:v>Draw_PartyShieldStatusBarsLoop</x:v>
+      </x:c>
+      <x:c r="C781" s="8" t="str">
+        <x:v>Advance_PartyShieldStatusBarRow</x:v>
+      </x:c>
+      <x:c r="D781" s="8" t="str">
+        <x:v>and.w #PartyShieldStatusBar_SuppressionMask,d1</x:v>
+      </x:c>
+      <x:c r="E781" s="8" t="str">
+        <x:v>Tests the party-slot vacant and dead suppression bits before drawing a status bar.</x:v>
       </x:c>
       <x:c r="F781" s="8" t="n">
         <x:v>1</x:v>
@@ -55193,25 +54981,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B783" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PartyShieldStatusBarsLoop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C783" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_PartyShieldStatusBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D783" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Scale_ValueToBarLength</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E783" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Calls the common scaler to convert the selected champion's current value into a shield-bar width.</x:t>
-        </x:is>
+      <x:c r="B783" s="8" t="str">
+        <x:v>Draw_PartyShieldStatusBarsLoop</x:v>
+      </x:c>
+      <x:c r="C783" s="8" t="str">
+        <x:v>Advance_PartyShieldStatusBarRow</x:v>
+      </x:c>
+      <x:c r="D783" s="8" t="str">
+        <x:v>bsr.s Scale_ValueToBarLength</x:v>
+      </x:c>
+      <x:c r="E783" s="8" t="str">
+        <x:v>Calls the common scaler to convert the selected champion's current value into a shield-bar width.</x:v>
       </x:c>
       <x:c r="F783" s="8" t="n">
         <x:v>1</x:v>
@@ -55253,20 +55033,14 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B785" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Advance_PartyShieldStatusBarRow</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C785" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Return_FromMainPlayerInterface</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D785" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sub.w #$0009,d5</x:t>
-        </x:is>
+      <x:c r="B785" s="8" t="str">
+        <x:v>Advance_PartyShieldStatusBarRow</x:v>
+      </x:c>
+      <x:c r="C785" s="8" t="str">
+        <x:v>Return_PartyShieldStatusBars</x:v>
+      </x:c>
+      <x:c r="D785" s="8" t="str">
+        <x:v>sub.w #$0009,d5</x:v>
       </x:c>
       <x:c r="E785" s="8" t="str">
         <x:v>Moves to the next party-shield status-bar X position, nine pixels left of the current bar.</x:v>
@@ -55431,25 +55205,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B791" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainChampionAvatarPanel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C791" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainChampionAvatarInnerFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D791" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">move.l #$000002A9,a0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E791" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Selects the framebuffer offset for the 32×30 large champion avatar.</x:t>
-        </x:is>
+      <x:c r="B791" s="8" t="str">
+        <x:v>Draw_MainChampionAvatarPanel</x:v>
+      </x:c>
+      <x:c r="C791" s="8" t="str">
+        <x:v>Draw_MainChampionAvatarInnerFrame</x:v>
+      </x:c>
+      <x:c r="D791" s="8" t="str">
+        <x:v>move.l #MainChampionAvatar_ScreenByteOffset,a0</x:v>
+      </x:c>
+      <x:c r="E791" s="8" t="str">
+        <x:v>Selects the framebuffer offset for the 32x30 large champion avatar.</x:v>
       </x:c>
       <x:c r="F791" s="8" t="n">
         <x:v>1</x:v>
@@ -55461,25 +55227,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B792" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainChampionAvatarPanel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C792" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainChampionAvatarInnerFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D792" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Draw_ChampionLargeAvatar</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E792" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Calls the large-avatar compositor, which selects the leader portrait and applies its palette ink.</x:t>
-        </x:is>
+      <x:c r="B792" s="8" t="str">
+        <x:v>Draw_MainChampionAvatarPanel</x:v>
+      </x:c>
+      <x:c r="C792" s="8" t="str">
+        <x:v>Draw_MainChampionAvatarInnerFrame</x:v>
+      </x:c>
+      <x:c r="D792" s="8" t="str">
+        <x:v>bsr.s Draw_ChampionLargeAvatar</x:v>
+      </x:c>
+      <x:c r="E792" s="8" t="str">
+        <x:v>Calls the large-avatar compositor, which selects the leader portrait and applies its palette ink.</x:v>
       </x:c>
       <x:c r="F792" s="8" t="n">
         <x:v>1</x:v>
@@ -55581,25 +55339,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B796" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainChampionAvatarInnerFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C796" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00CD12</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D796" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Select_ChampionShieldInkColour</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E796" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Obtains the leader class colour used for the optional large-avatar inner-frame ink.</x:t>
-        </x:is>
+      <x:c r="B796" s="8" t="str">
+        <x:v>Draw_MainChampionAvatarInnerFrame</x:v>
+      </x:c>
+      <x:c r="C796" s="8" t="str">
+        <x:v>adrCd00CD12</x:v>
+      </x:c>
+      <x:c r="D796" s="8" t="str">
+        <x:v>bsr.s Select_ChampionShieldInkColour</x:v>
+      </x:c>
+      <x:c r="E796" s="8" t="str">
+        <x:v>Obtains the leader class colour used for the optional large-avatar inner-frame ink.</x:v>
       </x:c>
       <x:c r="F796" s="8" t="n">
         <x:v>1</x:v>
@@ -55671,25 +55421,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B799" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionLargeAvatar</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C799" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00CD4A</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D799" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lea GFX_Avatars.l,a1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E799" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Selects the packed champion portrait graphics source.</x:t>
-        </x:is>
+      <x:c r="B799" s="8" t="str">
+        <x:v>Draw_ChampionLargeAvatar</x:v>
+      </x:c>
+      <x:c r="C799" s="8" t="str">
+        <x:v>Get_ChampionShieldScreenPosition</x:v>
+      </x:c>
+      <x:c r="D799" s="8" t="str">
+        <x:v>lea GFX_Avatars_Large.l,a1</x:v>
+      </x:c>
+      <x:c r="E799" s="8" t="str">
+        <x:v>Selects the packed large champion portrait graphics source.</x:v>
       </x:c>
       <x:c r="F799" s="8" t="n">
         <x:v>1</x:v>
@@ -55731,25 +55473,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B801" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ChampionLargeAvatar</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C801" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00CD4A</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D801" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">move.l #$0001001D,-(sp)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E801" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Supplies the large portrait renderer with a two-word-wide, 30-row graphic size.</x:t>
-        </x:is>
+      <x:c r="B801" s="8" t="str">
+        <x:v>Draw_ChampionLargeAvatar</x:v>
+      </x:c>
+      <x:c r="C801" s="8" t="str">
+        <x:v>Get_ChampionShieldScreenPosition</x:v>
+      </x:c>
+      <x:c r="D801" s="8" t="str">
+        <x:v>move.l #ChampionLargeAvatar_DrawDimensions,-(sp)</x:v>
+      </x:c>
+      <x:c r="E801" s="8" t="str">
+        <x:v>Supplies the large portrait renderer with a two-word-wide, 30-row graphic size.</x:v>
       </x:c>
       <x:c r="F801" s="8" t="n">
         <x:v>1</x:v>
@@ -56331,25 +56065,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B821" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_ScrollFrame</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C821" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_PlanarGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D821" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">bsr Draw_PlanarGraphic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E821" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Calls the common four-plane graphic renderer for one scroll-frame edge or cap.</x:t>
-        </x:is>
+      <x:c r="B821" s="8" t="str">
+        <x:v>Draw_ScrollFrame</x:v>
+      </x:c>
+      <x:c r="C821" s="8" t="str">
+        <x:v>Draw_PlanarGraphic</x:v>
+      </x:c>
+      <x:c r="D821" s="8" t="str">
+        <x:v>bsr.s Draw_PlanarGraphic</x:v>
+      </x:c>
+      <x:c r="E821" s="8" t="str">
+        <x:v>Calls the common four-plane graphic renderer for one scroll-frame edge or cap.</x:v>
       </x:c>
       <x:c r="F821" s="8" t="n">
         <x:v>3</x:v>
@@ -56691,25 +56417,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B833" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00688C</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C833" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd0068F8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D833" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">move.b $0015(a4),d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E833" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Loads champion byte $15, the spell cooldown penalty; matching champion and spell classes halve it.</x:t>
-        </x:is>
+      <x:c r="B833" t="str">
+        <x:v>adrCd0068DC</x:v>
+      </x:c>
+      <x:c r="C833" t="str">
+        <x:v>adrCd0068F8</x:v>
+      </x:c>
+      <x:c r="D833" t="str">
+        <x:v>move.b $0013(a4),d0</x:v>
+      </x:c>
+      <x:c r="E833" t="str">
+        <x:v>Loads the selected spell index from champion byte $13 before choosing its base SpellCost_DataTable entry.</x:v>
       </x:c>
       <x:c r="F833" t="n">
         <x:v>1</x:v>
@@ -56721,25 +56439,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B834" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00688C</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C834" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd0068F8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D834" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">addq.w #,d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E834" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The displayed base cost is twice the stored SpellCost_DataTable value plus one.</x:t>
-        </x:is>
+      <x:c r="B834" t="str">
+        <x:v>Calculate_SpellPointCost</x:v>
+      </x:c>
+      <x:c r="C834" t="str">
+        <x:v>adrCd0068F8</x:v>
+      </x:c>
+      <x:c r="D834" t="str">
+        <x:v>addq.w #$01,d0</x:v>
+      </x:c>
+      <x:c r="E834" t="str">
+        <x:v>Increments the stored base spell cost before doubling it, so the base contribution is twice (the table value plus one).</x:v>
       </x:c>
       <x:c r="F834" t="n">
         <x:v>1</x:v>
@@ -56901,25 +56611,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B840" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Exec_char_extensions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C840" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Exec_char_extensions</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D840" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">asl.w #,d4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E840" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FC text extension converts its byte column to native 8-pixel X coordinates before calculating the text origin.</x:t>
-        </x:is>
+      <x:c r="B840" t="str">
+        <x:v>.SetXYPosition</x:v>
+      </x:c>
+      <x:c r="C840" t="str">
+        <x:v>.Exit</x:v>
+      </x:c>
+      <x:c r="D840" t="str">
+        <x:v>asl.w #$03,d4</x:v>
+      </x:c>
+      <x:c r="E840" t="str">
+        <x:v>The FC text extension converts its byte column to native 8-pixel X coordinates before calculating the text origin.</x:v>
       </x:c>
       <x:c r="F840" t="n">
         <x:v>1</x:v>
@@ -56931,25 +56633,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B841" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00C650</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C841" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00C708</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D841" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cmpi.w #,d1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E841" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">C69C limits the spell-book top controls to Y -/bin/zshF; its X tests preserve 8-pixel gaps between page, close and page-forward targets.</x:t>
-        </x:is>
+      <x:c r="B841" t="str">
+        <x:v>adrCd00C69C</x:v>
+      </x:c>
+      <x:c r="C841" t="str">
+        <x:v>adrCd00C708</x:v>
+      </x:c>
+      <x:c r="D841" t="str">
+        <x:v>cmpi.w #$0007,d1</x:v>
+      </x:c>
+      <x:c r="E841" t="str">
+        <x:v>Rejects top-control Y values below $07; the following comparison limits the band to $07-$0F before the X hit tests.</x:v>
       </x:c>
       <x:c r="F841" t="n">
         <x:v>1</x:v>
@@ -56961,25 +56655,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B842" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd00688C</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C842" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd0068F8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D842" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">cmpi.w #,d0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E842" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Rejects a cast-power setting when the calculated spell-point cost reaches ; displayed costs are therefore limited to /bin/zsh-.</x:t>
-        </x:is>
+      <x:c r="B842" t="str">
+        <x:v>adrCd0068F8</x:v>
+      </x:c>
+      <x:c r="C842" t="str">
+        <x:v>Character_GetClassIndex</x:v>
+      </x:c>
+      <x:c r="D842" t="str">
+        <x:v>cmpi.w #SpellCasting_ManaCostMaximum,d0</x:v>
+      </x:c>
+      <x:c r="E842" t="str">
+        <x:v>Rejects a cast-power setting when the calculated spell-point cost reaches $64; displayed costs are therefore limited to $01-$63.</x:v>
       </x:c>
       <x:c r="F842" t="n">
         <x:v>1</x:v>
@@ -56991,25 +56677,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B843" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd006698</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C843" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd006712</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D843" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">moveq #,d6</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E843" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">The selected spell name printer emits exactly eight characters from SpellNames at the spell-book name origin.</x:t>
-        </x:is>
+      <x:c r="B843" t="str">
+        <x:v>adrCd00CFBC</x:v>
+      </x:c>
+      <x:c r="C843" t="str">
+        <x:v>adrLp00CFDA</x:v>
+      </x:c>
+      <x:c r="D843" t="str">
+        <x:v>moveq #$07,d6</x:v>
+      </x:c>
+      <x:c r="E843" t="str">
+        <x:v>Uses DBRA terminal index seven so the selected spell-name printer emits exactly eight characters from its fixed SpellNames record.</x:v>
       </x:c>
       <x:c r="F843" t="n">
         <x:v>1</x:v>
@@ -57081,25 +56759,17 @@
           <x:t xml:space="preserve">BLOODWYCH439</x:t>
         </x:is>
       </x:c>
-      <x:c r="B846" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd006778</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C846" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd006836</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D846" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sub.b SpellCasting_SpellDifficultyPenalties(pc,d6.w),d7</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E846" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Subtracts the source difficulty-penalty byte for the selected spell before C6720 maps the negated score to the CAST bar.</x:t>
-        </x:is>
+      <x:c r="B846" t="str">
+        <x:v>adrCd006836</x:v>
+      </x:c>
+      <x:c r="C846" t="str">
+        <x:v>SpellCasting_SpellDifficultyPenalties</x:v>
+      </x:c>
+      <x:c r="D846" t="str">
+        <x:v>sub.b SpellCasting_SpellDifficultyPenalties(pc,d6.w),d7</x:v>
+      </x:c>
+      <x:c r="E846" t="str">
+        <x:v>Subtracts the source difficulty-penalty byte for the selected spell before Draw_SpellCastingBar maps the negated score to the CAST bar.</x:v>
       </x:c>
       <x:c r="F846" t="n">
         <x:v>1</x:v>
@@ -57612,18 +57282,18 @@
         <x:v>BLOODWYCH439</x:v>
       </x:c>
       <x:c r="B865" t="str">
-        <x:v>Store_PlayerXY_AI_TBC</x:v>
+        <x:v>Store_PlayerMovePosition</x:v>
       </x:c>
       <x:c r="C865" t="str">
-        <x:v>Check_TeamPad_AI_TBC</x:v>
+        <x:v>Check_PlayerMoveTeamPad</x:v>
       </x:c>
       <x:c r="D865" t="str">
         <x:v>clr.b $003E(a5)</x:v>
       </x:c>
       <x:c r="E865" t="str">
-        <x:v>After a successful movement stores the new position, clears all four avatar presentation bits, and redraws the party-command interface.</x:v>
-      </x:c>
-      <x:c r="F865" t="str">
+        <x:v>After a successful movement, clears all four avatar presentation bits and redraws the party-command interface when presentation state was active.</x:v>
+      </x:c>
+      <x:c r="F865" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -66408,16 +66078,16 @@
         <x:v>BLOODWYCH439</x:v>
       </x:c>
       <x:c r="B1306" t="str">
-        <x:v>adrCd00787E</x:v>
+        <x:v>Place_VivifiedChampionAtCell</x:v>
       </x:c>
       <x:c r="C1306" t="str">
-        <x:v>adrCd0078A0</x:v>
+        <x:v>VivifyExternal_RestorePartyMember</x:v>
       </x:c>
       <x:c r="D1306" t="str">
-        <x:v>move.b	adrB_00EE2F.l,$001F(a4)</x:v>
+        <x:v>move.b CurrentTower+$01.l,$001F(a4)</x:v>
       </x:c>
       <x:c r="E1306" t="str">
-        <x:v>Store the current tower in the champion record.</x:v>
+        <x:v>Stores the current tower in the revived champion record.</x:v>
       </x:c>
       <x:c r="F1306" t="n">
         <x:v>1</x:v>
@@ -68042,7 +67712,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf489d456beb46f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0ba1c0869d41ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
allowed Formatting tool to bundle all EQU into a seperate file
</commit_message>
<xml_diff>
--- a/cleanup.xlsx
+++ b/cleanup.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R54bdfbcae3ef4eb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rdb797eab24324ff0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R5954448ee2f44e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R98b9dd3391754991"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_NOTES" sheetId="5" r:id="Rcd31dcd29c3e494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EQUATES" sheetId="1" r:id="R701a8fe6634d45eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMMENTS" sheetId="2" r:id="Rd38d2d5e38614fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIX_LABELS" sheetId="3" r:id="R03d8781dbeb44529"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASM_RECOVERY" sheetId="4" r:id="R3d4ffd98a2cb48e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_NOTES" sheetId="5" r:id="R8802c95024e14cf8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25028,67 +25028,55 @@
       </x:c>
     </x:row>
     <x:row r="484">
-      <x:c r="A484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GFX_Pockets_InventoryInterfaceOffset</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">$3C00</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">verified</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Packed Pockets.gfx offset containing the inventory chain/interface strip.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L484" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EQU-only definition; offset is within GFX_Pockets.</x:t>
-        </x:is>
+      <x:c r="A484" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B484" t="str">
+        <x:v>GFX_Pockets_ChainStripContinuousOffset</x:v>
+      </x:c>
+      <x:c r="C484" t="str">
+        <x:v>$3C00</x:v>
+      </x:c>
+      <x:c r="D484"/>
+      <x:c r="E484"/>
+      <x:c r="F484"/>
+      <x:c r="G484"/>
+      <x:c r="H484"/>
+      <x:c r="I484"/>
+      <x:c r="J484" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K484" t="str">
+        <x:v>Packed Pockets.gfx offset of the continuous 96 by 7 chain strip used at the dungeon-display lower edge and in the inventory presentation.</x:v>
+      </x:c>
+      <x:c r="L484" t="str">
+        <x:v>Renamed from GFX_Pockets_InventoryInterfaceOffset because the same artwork is not inventory-specific.</x:v>
       </x:c>
     </x:row>
     <x:row r="485">
-      <x:c r="A485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GFX_Pockets_SpellBookOffset</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">$4100</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">verified</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Packed Pockets.gfx offset used for the spell-book surface.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L485" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EQU-only definition; offset is within GFX_Pockets.</x:t>
-        </x:is>
+      <x:c r="A485" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B485" t="str">
+        <x:v>GFX_Pockets_SpellBookOffset</x:v>
+      </x:c>
+      <x:c r="C485" t="str">
+        <x:v>$4100</x:v>
+      </x:c>
+      <x:c r="D485"/>
+      <x:c r="E485"/>
+      <x:c r="F485"/>
+      <x:c r="G485"/>
+      <x:c r="H485"/>
+      <x:c r="I485"/>
+      <x:c r="J485" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K485" t="str">
+        <x:v>Packed Pockets.gfx offset of the 96 by 62 spell-book surface, including its page-turn arrows.</x:v>
+      </x:c>
+      <x:c r="L485" t="str">
+        <x:v>EQU-only definition; dimensions and use are confirmed by Prepare_AndDrawSpellBookSurface.</x:v>
       </x:c>
     </x:row>
     <x:row r="486">
@@ -25124,67 +25112,55 @@
       </x:c>
     </x:row>
     <x:row r="487">
-      <x:c r="A487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GFX_Pockets_StatusPanelOffset</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">$67C0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">verified</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Packed Pockets.gfx offset used by the status-panel interface pieces.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L487" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EQU-only definition; offset is within GFX_Pockets.</x:t>
-        </x:is>
+      <x:c r="A487" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B487" t="str">
+        <x:v>GFX_Pockets_StatusPanelOffset</x:v>
+      </x:c>
+      <x:c r="C487" t="str">
+        <x:v>$67C0</x:v>
+      </x:c>
+      <x:c r="D487"/>
+      <x:c r="E487"/>
+      <x:c r="F487"/>
+      <x:c r="G487"/>
+      <x:c r="H487"/>
+      <x:c r="I487"/>
+      <x:c r="J487" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K487" t="str">
+        <x:v>Packed Pockets.gfx offset of the 64 by 22 status-panel graphic containing the book and ledger icons.</x:v>
+      </x:c>
+      <x:c r="L487" t="str">
+        <x:v>EQU-only definition; drawn by Draw_ChampionNamePanelLowerEdge.</x:v>
       </x:c>
     </x:row>
     <x:row r="488">
-      <x:c r="A488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">GFX_Pockets_CommandPanelOffset</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">$7580</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">verified</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Packed Pockets.gfx offset used by the lower status/command interface pieces.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L488" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">EQU-only definition; offset is within GFX_Pockets.</x:t>
-        </x:is>
+      <x:c r="A488" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B488" t="str">
+        <x:v>GFX_Pockets_StatsTitleOffset</x:v>
+      </x:c>
+      <x:c r="C488" t="str">
+        <x:v>$7580</x:v>
+      </x:c>
+      <x:c r="D488"/>
+      <x:c r="E488"/>
+      <x:c r="F488"/>
+      <x:c r="G488"/>
+      <x:c r="H488"/>
+      <x:c r="I488"/>
+      <x:c r="J488" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K488" t="str">
+        <x:v>Packed Pockets.gfx offset of the 48 by 6 STATS title graphic drawn in the compact statistics frame.</x:v>
+      </x:c>
+      <x:c r="L488" t="str">
+        <x:v>Renamed from GFX_Pockets_CommandPanelOffset; the only source use draws the STATS title at player-local screen offset $0286.</x:v>
       </x:c>
     </x:row>
     <x:row r="489">
@@ -30837,6 +30813,414 @@
       </x:c>
       <x:c r="L630" t="str">
         <x:v>Switch/trigger audit: original adrCd007664; instruction bytes verified against binaries/BLOODWYCH439.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="631">
+      <x:c r="A631" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B631" t="str">
+        <x:v>GFX_Pockets_ChainStripContinuousOffset</x:v>
+      </x:c>
+      <x:c r="C631" t="str">
+        <x:v>$3C00</x:v>
+      </x:c>
+      <x:c r="D631" t="str">
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
+      </x:c>
+      <x:c r="E631" t="str">
+        <x:v>adrCd00838C</x:v>
+      </x:c>
+      <x:c r="F631" t="str">
+        <x:v>lea GFX_Pockets+$3C00.l,a1</x:v>
+      </x:c>
+      <x:c r="G631" t="str">
+        <x:v>43F900050302</x:v>
+      </x:c>
+      <x:c r="H631" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripContinuousOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="I631" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J631" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K631" t="str">
+        <x:v>Selects the continuous chain strip for the dungeon-display lower edge and inventory presentation.</x:v>
+      </x:c>
+      <x:c r="L631" t="str">
+        <x:v>Exact instruction and opcode verified in the current relabelled source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="632">
+      <x:c r="A632" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B632" t="str">
+        <x:v>GFX_Pockets_ChainStripShieldGapsOffset</x:v>
+      </x:c>
+      <x:c r="C632" t="str">
+        <x:v>$3C30</x:v>
+      </x:c>
+      <x:c r="D632"/>
+      <x:c r="E632"/>
+      <x:c r="F632"/>
+      <x:c r="G632"/>
+      <x:c r="H632"/>
+      <x:c r="I632"/>
+      <x:c r="J632" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K632" t="str">
+        <x:v>Packed Pockets.gfx offset of the 96 by 7 chain strip whose gaps accommodate the four party shields.</x:v>
+      </x:c>
+      <x:c r="L632" t="str">
+        <x:v>EQU-only definition; the artwork is distinct from the continuous strips at $3C00 and $3C60.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="633">
+      <x:c r="A633" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B633" t="str">
+        <x:v>GFX_Pockets_ChainStripShieldGapsOffset</x:v>
+      </x:c>
+      <x:c r="C633" t="str">
+        <x:v>$3C30</x:v>
+      </x:c>
+      <x:c r="D633" t="str">
+        <x:v>Draw_PartyShieldChainStrip</x:v>
+      </x:c>
+      <x:c r="E633" t="str">
+        <x:v>Refresh_PartyShieldSlotIfDirty</x:v>
+      </x:c>
+      <x:c r="F633" t="str">
+        <x:v>lea GFX_Pockets+$3C30.l,a1</x:v>
+      </x:c>
+      <x:c r="G633" t="str">
+        <x:v>43F900050332</x:v>
+      </x:c>
+      <x:c r="H633" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripShieldGapsOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="I633" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J633" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K633" t="str">
+        <x:v>Selects the chain strip with gaps for the party-shield presentation.</x:v>
+      </x:c>
+      <x:c r="L633" t="str">
+        <x:v>Exact instruction and opcode verified in the current relabelled source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="634">
+      <x:c r="A634" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B634" t="str">
+        <x:v>GFX_Pockets_ChainStripCommandPanelOffset</x:v>
+      </x:c>
+      <x:c r="C634" t="str">
+        <x:v>$3C60</x:v>
+      </x:c>
+      <x:c r="D634"/>
+      <x:c r="E634"/>
+      <x:c r="F634"/>
+      <x:c r="G634"/>
+      <x:c r="H634"/>
+      <x:c r="I634"/>
+      <x:c r="J634" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K634" t="str">
+        <x:v>Packed Pockets.gfx offset of the continuous 96 by 7 chain strip used beneath the party-command menu.</x:v>
+      </x:c>
+      <x:c r="L634" t="str">
+        <x:v>EQU-only definition; this crop is visually continuous like the $3C00 strip but has its own source location.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="635">
+      <x:c r="A635" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B635" t="str">
+        <x:v>GFX_Pockets_ChainStripCommandPanelOffset</x:v>
+      </x:c>
+      <x:c r="C635" t="str">
+        <x:v>$3C60</x:v>
+      </x:c>
+      <x:c r="D635" t="str">
+        <x:v>Draw_PartyCommandIconStrip</x:v>
+      </x:c>
+      <x:c r="E635" t="str">
+        <x:v>PartyCommandDescriptorStream_Mode0</x:v>
+      </x:c>
+      <x:c r="F635" t="str">
+        <x:v>lea GFX_Pockets+$3C60.l,a1</x:v>
+      </x:c>
+      <x:c r="G635" t="str">
+        <x:v>43F900050362</x:v>
+      </x:c>
+      <x:c r="H635" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripCommandPanelOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="I635" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J635" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K635" t="str">
+        <x:v>Selects the continuous chain strip drawn beneath the party-command menu.</x:v>
+      </x:c>
+      <x:c r="L635" t="str">
+        <x:v>Exact instruction and opcode verified in the current relabelled source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="636">
+      <x:c r="A636" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B636" t="str">
+        <x:v>GFX_Pockets_StatsTitleOffset</x:v>
+      </x:c>
+      <x:c r="C636" t="str">
+        <x:v>$7580</x:v>
+      </x:c>
+      <x:c r="D636" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="E636" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="F636" t="str">
+        <x:v>lea GFX_Pockets+$7580.l,a1</x:v>
+      </x:c>
+      <x:c r="G636" t="str">
+        <x:v>43F900053C82</x:v>
+      </x:c>
+      <x:c r="H636" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_StatsTitleOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="I636" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J636" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K636" t="str">
+        <x:v>Selects the pre-drawn STATS title graphic for the compact statistics frame.</x:v>
+      </x:c>
+      <x:c r="L636" t="str">
+        <x:v>Exact instruction and opcode verified in the current relabelled source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="637">
+      <x:c r="A637" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B637" t="str">
+        <x:v>GFX_Pockets_StatusPanelOffset</x:v>
+      </x:c>
+      <x:c r="C637" t="str">
+        <x:v>$67C0</x:v>
+      </x:c>
+      <x:c r="D637" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="E637" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="F637" t="str">
+        <x:v>lea GFX_Pockets+$67C0.l,a1</x:v>
+      </x:c>
+      <x:c r="G637" t="str">
+        <x:v>43F900052EC2</x:v>
+      </x:c>
+      <x:c r="H637" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_StatusPanelOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="I637" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J637" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K637" t="str">
+        <x:v>Selects the status-panel graphic containing the book and ledger icons.</x:v>
+      </x:c>
+      <x:c r="L637" t="str">
+        <x:v>Exact instruction and opcode verified in the current relabelled source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="638">
+      <x:c r="A638" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B638" t="str">
+        <x:v>GFX_Pockets_CommandPadPlayer2Offset</x:v>
+      </x:c>
+      <x:c r="C638" t="str">
+        <x:v>$67E0</x:v>
+      </x:c>
+      <x:c r="D638"/>
+      <x:c r="E638"/>
+      <x:c r="F638"/>
+      <x:c r="G638"/>
+      <x:c r="H638"/>
+      <x:c r="I638"/>
+      <x:c r="J638" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K638" t="str">
+        <x:v>Packed Pockets.gfx offset of the Player 2 command-pad variant.</x:v>
+      </x:c>
+      <x:c r="L638" t="str">
+        <x:v>Player2_Data begins with identity byte $01, so the bit test keeps the base $67E0 source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="639">
+      <x:c r="A639" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B639" t="str">
+        <x:v>GFX_Pockets_CommandPadPlayer2Offset</x:v>
+      </x:c>
+      <x:c r="C639" t="str">
+        <x:v>$67E0</x:v>
+      </x:c>
+      <x:c r="D639" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="E639" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="F639" t="str">
+        <x:v>lea GFX_Pockets+$67E0.l,a1</x:v>
+      </x:c>
+      <x:c r="G639" t="str">
+        <x:v>43F900052EE2</x:v>
+      </x:c>
+      <x:c r="H639" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_CommandPadPlayer2Offset.l,a1</x:v>
+      </x:c>
+      <x:c r="I639" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J639" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K639" t="str">
+        <x:v>Selects the Player 2 command-pad source before the player-identity adjustment.</x:v>
+      </x:c>
+      <x:c r="L639" t="str">
+        <x:v>Corrects the external annotation, which attached this name to unrelated code at runtime address $67E0.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="640">
+      <x:c r="A640" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B640" t="str">
+        <x:v>GFX_Pockets_CommandPadPlayer1Offset</x:v>
+      </x:c>
+      <x:c r="C640" t="str">
+        <x:v>$6800</x:v>
+      </x:c>
+      <x:c r="D640"/>
+      <x:c r="E640"/>
+      <x:c r="F640"/>
+      <x:c r="G640"/>
+      <x:c r="H640"/>
+      <x:c r="I640"/>
+      <x:c r="J640" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K640" t="str">
+        <x:v>Packed Pockets.gfx offset of the Player 1 command-pad variant.</x:v>
+      </x:c>
+      <x:c r="L640" t="str">
+        <x:v>Player1_Data begins with identity byte $00, so the draw path adds $20 to the Player 2 base source.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="641">
+      <x:c r="A641" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B641" t="str">
+        <x:v>GFX_Pockets_CommandPadPlayer1Offset</x:v>
+      </x:c>
+      <x:c r="C641" t="str">
+        <x:v>$6800</x:v>
+      </x:c>
+      <x:c r="D641" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="E641" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="F641" t="str">
+        <x:v>add.w #$0020,a1</x:v>
+      </x:c>
+      <x:c r="G641" t="str">
+        <x:v>D2FC0020</x:v>
+      </x:c>
+      <x:c r="H641" t="str">
+        <x:v>add.w #GFX_Pockets_CommandPadPlayer1Offset-GFX_Pockets_CommandPadPlayer2Offset,a1</x:v>
+      </x:c>
+      <x:c r="I641" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J641" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K641" t="str">
+        <x:v>Moves from the Player 2 command-pad source to the Player 1 variant when the identity bit is clear.</x:v>
+      </x:c>
+      <x:c r="L641" t="str">
+        <x:v>The symbolic difference remains $20 and preserves the immediate-word encoding.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="642">
+      <x:c r="A642" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B642" t="str">
+        <x:v>PlayerData_PlayerIdentityBit</x:v>
+      </x:c>
+      <x:c r="C642" t="str">
+        <x:v>$00</x:v>
+      </x:c>
+      <x:c r="D642" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="E642" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="F642" t="str">
+        <x:v>btst #$00,(a5)</x:v>
+      </x:c>
+      <x:c r="G642" t="str">
+        <x:v>08150000</x:v>
+      </x:c>
+      <x:c r="H642" t="str">
+        <x:v>btst #PlayerData_PlayerIdentityBit,(a5)</x:v>
+      </x:c>
+      <x:c r="I642" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J642" t="str">
+        <x:v>verified</x:v>
+      </x:c>
+      <x:c r="K642" t="str">
+        <x:v>Tests the active player identity before choosing the command-pad variant.</x:v>
+      </x:c>
+      <x:c r="L642" t="str">
+        <x:v>Player 1 stores $00 at Player1_Data; Player 2 stores $01 at Player2_Data.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -48264,35 +48648,23 @@
       </x:c>
     </x:row>
     <x:row r="555">
-      <x:c r="A555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">adrCd007FF8</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Draw_MainPlayerInterface</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">lea GFX_Pockets+$7580.l,a1</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Selects the pre-drawn `&lt;STATS&gt;` title graphic from GFX_Pockets.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F555" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">1</x:t>
-        </x:is>
+      <x:c r="A555" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B555" t="str">
+        <x:v>Draw_CompactStatsFrame</x:v>
+      </x:c>
+      <x:c r="C555" t="str">
+        <x:v>Draw_MainPlayerInterface</x:v>
+      </x:c>
+      <x:c r="D555" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_StatsTitleOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="E555" t="str">
+        <x:v>Selects the pre-drawn 48 by 6 STATS title graphic from GFX_Pockets.</x:v>
+      </x:c>
+      <x:c r="F555" t="n">
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="556">
@@ -52066,22 +52438,20 @@
       </x:c>
     </x:row>
     <x:row r="682">
-      <x:c r="A682" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BLOODWYCH439</x:t>
-        </x:is>
+      <x:c r="A682" t="str">
+        <x:v>BLOODWYCH439</x:v>
       </x:c>
       <x:c r="B682" t="str">
-        <x:v>adrCd008358</x:v>
+        <x:v>Draw_DungeonDisplayLowerEdge</x:v>
       </x:c>
       <x:c r="C682" t="str">
-        <x:v>adrCd008396</x:v>
+        <x:v>adrCd00838C</x:v>
       </x:c>
       <x:c r="D682" t="str">
-        <x:v>lea GFX_Pockets+$3C00.l,a1</x:v>
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripContinuousOffset.l,a1</x:v>
       </x:c>
       <x:c r="E682" t="str">
-        <x:v>Uses the packed inventory interface strip at GFX_Pockets+$3C00 as the source graphic for each inventory chain decoration.</x:v>
+        <x:v>Selects the continuous 96 by 7 chain strip used at the dungeon-display lower edge and in the inventory presentation.</x:v>
       </x:c>
       <x:c r="F682" t="n">
         <x:v>1</x:v>
@@ -67210,6 +67580,126 @@
         <x:v>Refresh the party's champion display and return.</x:v>
       </x:c>
       <x:c r="F1362" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1363">
+      <x:c r="A1363" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1363" t="str">
+        <x:v>Draw_PartyShieldChainStrip</x:v>
+      </x:c>
+      <x:c r="C1363" t="str">
+        <x:v>Refresh_PartyShieldSlotIfDirty</x:v>
+      </x:c>
+      <x:c r="D1363" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripShieldGapsOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="E1363" t="str">
+        <x:v>Selects the 96 by 7 chain strip whose gaps accommodate the four party shields.</x:v>
+      </x:c>
+      <x:c r="F1363" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1364">
+      <x:c r="A1364" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1364" t="str">
+        <x:v>Draw_PartyCommandIconStrip</x:v>
+      </x:c>
+      <x:c r="C1364" t="str">
+        <x:v>PartyCommandDescriptorStream_Mode0</x:v>
+      </x:c>
+      <x:c r="D1364" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_ChainStripCommandPanelOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="E1364" t="str">
+        <x:v>Selects the continuous 96 by 7 chain strip drawn beneath the party-command menu.</x:v>
+      </x:c>
+      <x:c r="F1364" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1365">
+      <x:c r="A1365" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1365" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C1365" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="D1365" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_StatusPanelOffset.l,a1</x:v>
+      </x:c>
+      <x:c r="E1365" t="str">
+        <x:v>Selects the 64 by 22 status-panel graphic containing the book and ledger icons.</x:v>
+      </x:c>
+      <x:c r="F1365" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1366">
+      <x:c r="A1366" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1366" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C1366" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="D1366" t="str">
+        <x:v>lea GFX_Pockets+GFX_Pockets_CommandPadPlayer2Offset.l,a1</x:v>
+      </x:c>
+      <x:c r="E1366" t="str">
+        <x:v>Starts from the Player 2 command-pad source; Player 1 applies the following $20 adjustment.</x:v>
+      </x:c>
+      <x:c r="F1366" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1367">
+      <x:c r="A1367" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1367" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C1367" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="D1367" t="str">
+        <x:v>btst #PlayerData_PlayerIdentityBit,(a5)</x:v>
+      </x:c>
+      <x:c r="E1367" t="str">
+        <x:v>Player 2's set identity bit retains the $67E0 command pad; Player 1 falls through to the $20 source adjustment.</x:v>
+      </x:c>
+      <x:c r="F1367" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="1368">
+      <x:c r="A1368" t="str">
+        <x:v>BLOODWYCH439</x:v>
+      </x:c>
+      <x:c r="B1368" t="str">
+        <x:v>Draw_ChampionNamePanelLowerEdge</x:v>
+      </x:c>
+      <x:c r="C1368" t="str">
+        <x:v>adrCd008308</x:v>
+      </x:c>
+      <x:c r="D1368" t="str">
+        <x:v>add.w #GFX_Pockets_CommandPadPlayer1Offset-GFX_Pockets_CommandPadPlayer2Offset,a1</x:v>
+      </x:c>
+      <x:c r="E1368" t="str">
+        <x:v>Selects the Player 1 command-pad source by advancing from $67E0 to $6800.</x:v>
+      </x:c>
+      <x:c r="F1368" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -67712,7 +68202,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb0ba1c0869d41ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21b9ed0a813d4046"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>